<commit_message>
feat(cwp): add Batch 002 Germany white profiles
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -3274,6 +3274,2726 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SAT_WINE_012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mosel Riesling</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Light-bodied high-acid Riesling from steep slate slopes</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Mosel Riesling</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Mosel</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Middle Mosel / Saar / Ruwer</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Mosel</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>cool continental; river reflection and air movement help ripening and frost protection</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>steep river slopes; exact altitude is less diagnostic than slope and aspect</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>slate soils on very steep slopes next to the river</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>["best vineyards on very steep stony south-facing slopes","hand work is required on extreme slopes","head pruning with individual stakes is used to maximize grape exposure"]</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>["dry to sweet Riesling styles","sweet premium styles made by stopping fermentation early","MLF and new oak avoided to preserve fruit and acidity"]</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>inert vessels or large old oak without new oak aroma; new oak is not a diagnostic marker</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>dry to sweet, with many classic examples off-dry to medium sweet</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>high to very high</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>low to medium; sweet styles often 8-9% abv</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>["floral notes","green apple","citrus","slate-like mineral impression"]</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>["green fruit","citrus","floral fruit","mineral freshness"]</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>medium to long, acid-driven</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>good to outstanding; top villages include Piesport, Bernkastel and Wehlen</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>medium to long ageing for high-quality examples due to acidity and balance</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>["pale lemon","clear","light intensity","medium to pronounced intensity","floral","green apple","lemon","slate mineral note possible","dry to sweet","high acidity","light body","low to medium alcohol","green fruit and citrus"]</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>["Mosel Rieslings are lighter, lower alcohol, and higher acid than Rheingau, Rheinhessen, and Pfalz","floral and green fruit flavours predominate","Riesling is the only permitted variety for GG wines in Mosel"]</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>["low alcohol means simple wine","sweetness means low quality","all German Riesling tastes the same"]</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>["Look for low alcohol plus high acidity.","Use body to separate Mosel from Rheingau."]</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>["pale lemon","clear","light intensity","medium to pronounced intensity","floral","green apple","lemon","slate mineral note possible","dry to sweet","high acidity","light body","low to medium alcohol","green fruit and citrus","lighter body than Rheingau, Rheinhessen, and Pfalz","lower alcohol","higher acidity","floral and green fruit profile","steep slate river slopes"]</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>["do not describe Mosel as full-bodied","do not claim new oak as typical"]</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>Regional profile anchored in WSET Mosel text; SAT calibration adds typical appearance and mineral descriptors as standard wine knowledge.</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 012</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon","clear","light intensity"],"nose":["medium to pronounced intensity","floral","green apple","lemon","slate mineral note possible"],"palate":["dry to sweet","high acidity","light body","low to medium alcohol","green fruit and citrus"],"quality":["very good to outstanding when balance, concentration, and length align"],"ageing":["high-quality Mosel Riesling can age and retain freshness"],"diagnostic_features":["lighter body than Rheingau, Rheinhessen, and Pfalz","lower alcohol","higher acidity","floral and green fruit profile","steep slate river slopes"]}</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["cool continental Riesling","slate slope viticulture","sweet-acid balance"],"learning_objectives":["distinguish Mosel from fuller German regions","connect slope and river to ripening","calibrate low alcohol with residual sugar"],"typical_misconceptions":["low alcohol means simple wine","sweetness means low quality","all German Riesling tastes the same"],"mentor_focus":["ask for body, alcohol, and acidity before region conclusion"],"exam_traps":["calling every German Riesling Mosel","forgetting dry Mosel exists","missing Saar/Ruwer higher acid possibility"],"memory_hooks":["Mosel is the featherweight Riesling with electric acidity"],"comparison_styles":["Rheingau Riesling","Riesling Kabinett","Alsace Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_016"],"frequently_confused_with":["SAT_WINE_013","SAT_WINE_017"],"distinguishing_features":["lighter and lower alcohol than Rheingau","more floral-green than Pfalz","more regional than Pradikat-specific"]}</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Mosel Rieslings are lighter, lower alcohol, and higher acid than Rheingau, Rheinhessen, and Pfalz","floral and green fruit flavours predominate","Riesling is the only permitted variety for GG wines in Mosel"],"mentor_hints":["Look for low alcohol plus high acidity.","Use body to separate Mosel from Rheingau."],"student_traps":["assuming all Mosel is sweet","missing the slate and slope logic"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10421-10520","10774-10804"],"line_reference":["10421-10520","10774-10804"],"evidence":["Mosel Rieslings are described as lighter in body, lower in alcohol, and higher in acidity than Rheingau, Rheinhessen, and Pfalz.","Floral and green fruit flavours predominate."]}</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>Mosel</t>
+        </is>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>108-110</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>["10421-10520","10774-10804"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SAT_WINE_013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Rheingau Riesling</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Medium to full-bodied dry ripe peach Riesling</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Rheingau Riesling</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Rheingau</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Johannisberg / Rudesheim / Hochheim</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Rheingau</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>cool continental moderated by south-facing Rhine and Main slopes; protected by Taunus hills</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>slopes on north bank of Rhine and Main; exact altitude is less diagnostic than southerly aspect</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>varied slope soils; site exposure is emphasized by WSET</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>["vineyards on south-facing slopes","Taunus hills provide protection","humid Rhine conditions enable some BA and TBA production"]</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>["majority of Rieslings made dry","GG wines can be Riesling","sweet BA and TBA also produced in humid conditions"]</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>inert vessels or old neutral vessels; new oak is not typical for Riesling</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>mostly dry, with sweet BA and TBA possible</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>medium to high in dry styles</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>["ripe peach","citrus","floral note","honey with age"]</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>["ripe peach","citrus","mineral freshness","honeyed development with age"]</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>long in top dry wines</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>good to outstanding; small prestigious region</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>medium to long ageing in top dry and sweet examples</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","ripe peach","citrus","floral nuance","honey with age","usually dry","high acidity","medium to full body","medium to high alcohol","ripe peach fruit"]</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>["Rheingau is small and prestigious","Riesling dominates and most wines are dry","Rieslings have medium to full body and ripe peach character"]</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>["German Riesling is always sweet","Rheingau equals Mosel style","peach fruit means warm climate outside Germany"]</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>["Ask whether the wine feels broader than Mosel.","Peach plus dry high acid points toward Rheingau/Pfalz/Rheinhessen rather than Mosel."]</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","ripe peach","citrus","floral nuance","honey with age","usually dry","high acidity","medium to full body","medium to high alcohol","ripe peach fruit","riper peach character","more body than Mosel","prestigious south-facing Rhine slopes","dry style dominance"]</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>["do not force residual sweetness into every Rheingau profile","do not describe as lower alcohol than Mosel"]</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>Rheingau profile uses WSET regional text and standard SAT dry Riesling calibration.</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 013</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","ripe peach","citrus","floral nuance","honey with age"],"palate":["usually dry","high acidity","medium to full body","medium to high alcohol","ripe peach fruit"],"quality":["very good to outstanding for top sites and GG wines"],"ageing":["top Rieslings can mature for years or decades"],"diagnostic_features":["riper peach character","more body than Mosel","prestigious south-facing Rhine slopes","dry style dominance"]}</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["dry German Riesling","river slope ripening","regional body calibration"],"learning_objectives":["separate Rheingau from Mosel by body and peach ripeness","recognize dry German premium Riesling","link humid Rhine to BA/TBA potential"],"typical_misconceptions":["German Riesling is always sweet","Rheingau equals Mosel style","peach fruit means warm climate outside Germany"],"mentor_focus":["anchor dry style and medium-full body"],"exam_traps":["ignoring BA/TBA role","missing Taunus protection and aspect"],"memory_hooks":["Rheingau is the peachier, broader classic dry Riesling"],"comparison_styles":["Mosel Riesling","Pfalz Riesling","Riesling Spatlese"]}</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_014","SAT_WINE_015"],"frequently_confused_with":["SAT_WINE_012","SAT_WINE_017"],"distinguishing_features":["fuller than Mosel","more prestigious compact identity than Rheinhessen","less dry-warm extension than Pfalz"]}</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Rheingau is small and prestigious","Riesling dominates and most wines are dry","Rieslings have medium to full body and ripe peach character"],"mentor_hints":["Ask whether the wine feels broader than Mosel.","Peach plus dry high acid points toward Rheingau/Pfalz/Rheinhessen rather than Mosel."],"student_traps":["assuming low alcohol for all German Riesling","forgetting dry GG context"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10827-10842"],"line_reference":["10827-10842"],"evidence":["Rheingau Rieslings are described as medium to full bodied with ripe peach character.","The majority of wines are made dry."]}</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>Rheingau</t>
+        </is>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>["10827-10842"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SAT_WINE_014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Pfalz Riesling</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ripe fuller-bodied dry Riesling from the Mittelhaardt</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pfalz Riesling</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Pfalz</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Mittelhaardt / Forst / Deidesheim</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Pfalz</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>cool to moderate continental; driest German region due to Haardt Mountains rain shadow</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>steep west-side village slopes; exact altitude is less diagnostic than slope and dryness</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>varied slope soils; WSET emphasizes dry region and established quality vineyards</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>["vineyards run in narrow strip east of the Haardt Mountains","quality vineyards surround Forst and Deidesheim","water stress can occur in very warm years"]</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>["majority of wines now made in drier styles","GG wines can be Riesling","aroma-preserving Riesling winemaking"]</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>inert vessels or old neutral vessels; new oak is not typical for Riesling</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>mostly dry, with broader German Riesling range possible</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>["ripe citrus","peach","stone fruit","floral hint"]</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>["ripe citrus","peach","stone fruit","dry mineral finish"]</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>good to outstanding; long reputation for high-quality Riesling</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>medium to long ageing for top dry examples</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","ripe citrus","peach","stone fruit","floral hint","usually dry","high acidity","medium to full body","medium to high alcohol","ripe fruit concentration"]</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>["Pfalz is the second largest German wine region and the driest","Riesling is the most planted variety and has the longest quality reputation","Mittelhaardt vineyards produce ripe fuller-bodied Riesling"]</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>["Germany only makes delicate sweet Riesling","dry Riesling cannot be high quality","Pfalz equals Alsace"]</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>["Ask whether the style is dry and fuller-bodied.","Use Pfalz dryness as a causal clue."]</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","ripe citrus","peach","stone fruit","floral hint","usually dry","high acidity","medium to full body","medium to high alcohol","ripe fruit concentration","ripe fuller-bodied Riesling","drier style majority","Pfalz dryness and Haardt protection","Forst and Deidesheim quality core"]</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>["do not describe Pfalz as Germanys coolest or most delicate Riesling style"]</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>Pfalz profile follows WSET regional description and standard dry Riesling SAT markers.</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 014</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","ripe citrus","peach","stone fruit","floral hint"],"palate":["usually dry","high acidity","medium to full body","medium to high alcohol","ripe fruit concentration"],"quality":["very good to outstanding for established Mittelhaardt sites"],"ageing":["top dry wines can mature in bottle"],"diagnostic_features":["ripe fuller-bodied Riesling","drier style majority","Pfalz dryness and Haardt protection","Forst and Deidesheim quality core"]}</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["dry German Riesling","rain shadow and ripeness","Mittelhaardt quality"],"learning_objectives":["differentiate Pfalz from Rheingau and Mosel","connect dry climate to fuller ripeness","recognize German dry style trend"],"typical_misconceptions":["Germany only makes delicate sweet Riesling","dry Riesling cannot be high quality","Pfalz equals Alsace"],"mentor_focus":["build climate-to-body reasoning"],"exam_traps":["missing water stress in warm years","forgetting Riesling is most planted in Pfalz"],"memory_hooks":["Pfalz is Germanys dry, ripe Riesling corridor beside Alsace"],"comparison_styles":["Rheingau Riesling","Rheinhessen Riesling","Alsace Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_013","SAT_WINE_015"],"frequently_confused_with":["SAT_WINE_013","SAT_WINE_005"],"distinguishing_features":["driest German region","ripe fuller-bodied style from Mittelhaardt","less low-alcohol delicacy than Mosel"]}</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Pfalz is the second largest German wine region and the driest","Riesling is the most planted variety and has the longest quality reputation","Mittelhaardt vineyards produce ripe fuller-bodied Riesling"],"mentor_hints":["Ask whether the style is dry and fuller-bodied.","Use Pfalz dryness as a causal clue."],"student_traps":["over-associating all German Riesling with Mosel delicacy","ignoring dry style majority"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10879-10922"],"line_reference":["10879-10922"],"evidence":["Pfalz is described as Germanys driest region.","Mittelhaardt vineyards produce a ripe, fuller-bodied style of Riesling and most wines are now drier."]}</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>Pfalz</t>
+        </is>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>["10879-10922"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SAT_WINE_015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Rheinhessen Riesling</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Full-bodied Riesling from Rheinterrasse and innovative producers</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Rheinhessen Riesling</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Rheinhessen</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Rheinterrasse / Nierstein / Worms area</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Rheinhessen</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>cool continental with warmer riper sites along the Rhine</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>steep west bank Rhine slopes; exact altitude is less diagnostic than slope and river exposure</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>varied; WSET emphasizes steeply sloping vineyards around Nierstein</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>["largest vine-growing region","Rheinterrasse slopes around Nierstein have historic reputation","new growers outside historic areas produce top-quality wines"]</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>["dry and Pradikat Riesling possible","GG wines can be Riesling","modern quality-focused dry styles are important"]</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>inert vessels or old neutral vessels; new oak is not typical for Riesling</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>dry to sweet depending on category, with many quality dry styles</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>medium to full; among Germanys fullest-bodied Rieslings from Rheinterrasse</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>medium to high in dry styles</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>["ripe citrus","peach","stone fruit","floral note","honey with age"]</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>["ripe citrus","peach","stone fruit","mineral note","honeyed development"]</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>good to outstanding; reputation for innovation and excellence</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>medium to long ageing for top Rieslings</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","ripe citrus","peach","stone fruit","floral note","dry to sweet","high acidity","medium to full body","medium to high alcohol in dry styles","ripe fruit concentration"]</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>["Rheinhessen is Germanys largest vine-growing region","Rheinterrasse around Nierstein produces some of Germanys fullest-bodied Rieslings","the region has gained reputation for innovation and excellence"]</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>["Rheinhessen is only inexpensive wine","largest region means lowest quality","all Riesling regions are stylistically identical"]</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>["Ask whether the answer needs a broad regional profile rather than a single Pradikat.","Use body and Nierstein clue."]</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","ripe citrus","peach","stone fruit","floral note","dry to sweet","high acidity","medium to full body","medium to high alcohol in dry styles","ripe fruit concentration","fuller-bodied German Riesling","Rheinterrasse/Nierstein identity","innovation and quality revival","Riesling plus broad regional diversity"]</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>["do not treat Rheinhessen as only inexpensive wine","do not conflate Rheinhessen with Rheingau"]</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>Rheinhessen profile focuses on Riesling style, Nierstein, and innovation from WSET regional text.</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 015</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","ripe citrus","peach","stone fruit","floral note"],"palate":["dry to sweet","high acidity","medium to full body","medium to high alcohol in dry styles","ripe fruit concentration"],"quality":["good to outstanding from top Rheinterrasse and innovative producers"],"ageing":["best examples can develop honey and toast while retaining acidity"],"diagnostic_features":["fuller-bodied German Riesling","Rheinterrasse/Nierstein identity","innovation and quality revival","Riesling plus broad regional diversity"]}</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["regional diversity","full-bodied Riesling","quality revival"],"learning_objectives":["separate Rheinhessen from generic inexpensive stereotypes","recognize Rheinterrasse quality","compare fuller German Riesling regions"],"typical_misconceptions":["Rheinhessen is only inexpensive wine","largest region means lowest quality","all Riesling regions are stylistically identical"],"mentor_focus":["connect subregion reputation to style and quality"],"exam_traps":["forgetting Rheinhessen can produce top-quality wines","missing Nierstein/Rheinterrasse"],"memory_hooks":["Rheinhessen is large, innovative, and can make some of Germanys fullest Rieslings"],"comparison_styles":["Pfalz Riesling","Rheingau Riesling","Mosel Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_013","SAT_WINE_014"],"frequently_confused_with":["SAT_WINE_014","SAT_WINE_013"],"distinguishing_features":["largest region with broad variety range","Rheinterrasse produces some of Germanys fullest-bodied Rieslings","more innovation narrative than Rheingau"]}</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Rheinhessen is Germanys largest vine-growing region","Rheinterrasse around Nierstein produces some of Germanys fullest-bodied Rieslings","the region has gained reputation for innovation and excellence"],"mentor_hints":["Ask whether the answer needs a broad regional profile rather than a single Pradikat.","Use body and Nierstein clue."],"student_traps":["writing off Rheinhessen as low quality","confusing it with Rheingau by name"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10844-10875"],"line_reference":["10844-10875"],"evidence":["Rheinhessen is described as the largest vine-growing region.","Rheinterrasse around Nierstein produces some of the fullest-bodied Rieslings in Germany."]}</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>Rheinhessen</t>
+        </is>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>["10844-10875"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SAT_WINE_016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Riesling Kabinett</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Delicate light-bodied Pradikat Riesling</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Riesling Kabinett</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Pradikat category</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Kabinett</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>cool continental German Riesling sites; long cool ripening preserves acidity</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>varies by region; steep south-facing slopes are favored in marginal climates</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>varies by region; slate is important in Mosel examples</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>["picked at Kabinett must weight","multiple passes may be used to select grapes by ripeness","best sites maximize heat and sunlight"]</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>["best sweet styles made by stopping fermentation early","Sussreserve can sweeten but is not used for high-quality wines","MLF and new oak avoided"]</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>no new oak; aromatic purity is the goal</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>dry to medium sweet, commonly off-dry or medium sweet in classic examples</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>8-9% abv in sweet styles; drier styles can reach 12% abv</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>["green apple","citrus","floral notes"]</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>["green apple","citrus","residual sweetness balanced by acidity"]</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>medium to long, delicate and acid-led</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>good to outstanding depending on site and balance</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>medium to long ageing in high-quality examples despite delicacy</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>["pale lemon","light intensity","medium intensity","green apple","citrus","floral note","dry to medium sweet","high acidity","light body","low alcohol in sweet styles","green apple and citrus"]</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>["Kabinett is the most delicate Pradikat","light body, high acidity, and green apple or citrus are key","sweet styles have 8-9% abv while drier styles can reach 12%"]</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>["Kabinett means low quality","sweetness is added in premium examples","low alcohol means weak wine"]</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>["Check whether the wine is delicate rather than concentrated.","Alcohol level is a useful clue."]</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>["pale lemon","light intensity","medium intensity","green apple","citrus","floral note","dry to medium sweet","high acidity","light body","low alcohol in sweet styles","green apple and citrus","most delicate Pradikat","green apple or citrus","8-9% abv sweet style"]</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>["do not describe Kabinett as rich or botrytised by default"]</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>Kabinett profile follows WSET Pradikat description with standard SAT appearance and balance markers.</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 016</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon","light intensity"],"nose":["medium intensity","green apple","citrus","floral note"],"palate":["dry to medium sweet","high acidity","light body","low alcohol in sweet styles","green apple and citrus"],"quality":["good to outstanding where sweetness and acidity are finely balanced"],"ageing":["can age well when concentration and acidity are high"],"diagnostic_features":["most delicate Pradikat","light body","high acidity","green apple or citrus","8-9% abv sweet style"]}</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Pradikat as style indicator","sweet-acid balance","low alcohol from stopped fermentation"],"learning_objectives":["identify Kabinett versus Spatlese","separate sweetness from body","use alcohol as a clue"],"typical_misconceptions":["Kabinett means low quality","sweetness is added in premium examples","low alcohol means weak wine"],"mentor_focus":["ask for balance and delicacy"],"exam_traps":["calling Kabinett Spatlese from sweetness alone","missing high acidity"],"memory_hooks":["Kabinett is the delicate Riesling on a tightrope of sugar and acid"],"comparison_styles":["Mosel Riesling","Riesling Spatlese","Alsace Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_012"],"frequently_confused_with":["SAT_WINE_017"],"distinguishing_features":["lighter and less ripe than Spatlese","less concentrated than Auslese","lower alcohol in sweet styles"]}</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Kabinett is the most delicate Pradikat","light body, high acidity, and green apple or citrus are key","sweet styles have 8-9% abv while drier styles can reach 12%"],"mentor_hints":["Check whether the wine is delicate rather than concentrated.","Alcohol level is a useful clue."],"student_traps":["equating Pradikat with quality ladder only","missing dry Kabinett possibility"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","pradikat_riesling_scale"]</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10494-10527"],"line_reference":["10494-10527"],"evidence":["Kabinett wines are described as the most delicate Pradikatsweine.","They are light-bodied, high acid, green apple/citrus and sweet styles have 8-9% alcohol."]}</t>
+        </is>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>Riesling - Kabinett</t>
+        </is>
+      </c>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>108-109</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>["10494-10527"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SAT_WINE_017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Riesling Spatlese</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Riper more concentrated Pradikat Riesling</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Riesling Spatlese</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Pradikat category</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Spatlese</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>cool continental German Riesling sites with longer hang time for greater ripeness</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>varies by region; best sites maximize sunlight and warmth</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>varies by region</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>["grapes harvested riper than Kabinett","multiple passes can select ideal grapes","long cool ripening retains acidity"]</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>["made similarly to Kabinett","fermentation may be stopped to retain sweetness","dry styles are possible up to Auslese"]</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>no new oak; aromatic purity is the goal</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>dry to medium sweet, often with residual sugar in Pradikat examples</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>light to medium, more body than Kabinett</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>low to medium depending on sweetness; more alcohol than equivalent Kabinett when drier</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>["citrus","peach","apricot","floral notes"]</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","peach","apricot","sweet-acid balance"]</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>good to outstanding depending on site and balance</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>medium to long ageing for quality examples</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","peach","apricot","floral note","dry to medium sweet","high acidity","light to medium body","more concentration than Kabinett","citrus and stone fruit"]</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>["Spatlese wines are more concentrated, riper and have more body, alcohol, and sweetness than Kabinett from the same region","citrus and stone fruit aromas are common"]</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>["Spatlese must be sweet","more sweetness means lower acidity","Spatlese equals botrytis"]</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>["Ask what changed from Kabinett: ripeness, body, alcohol, and sweetness.","Do not rely on sweetness alone."]</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","peach","apricot","floral note","dry to medium sweet","high acidity","light to medium body","more concentration than Kabinett","citrus and stone fruit","riper than Kabinett","more body and concentration","sweetness where relevant"]</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>["do not make noble rot essential for Spatlese","do not collapse Spatlese into a single sweetness level"]</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>Spatlese profile follows WSET category progression and standard SAT descriptors.</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 017</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","citrus","peach","apricot","floral note"],"palate":["dry to medium sweet","high acidity","light to medium body","more concentration than Kabinett","citrus and stone fruit"],"quality":["very good to outstanding when ripeness and acidity are balanced"],"ageing":["can age well, developing honey and toast"],"diagnostic_features":["riper than Kabinett","more body and concentration","citrus and stone fruit","sweetness where relevant"]}</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Pradikat ripeness progression","stone fruit development","sweet-acid balance"],"learning_objectives":["differentiate Spatlese from Kabinett and Auslese","recognize ripeness without assuming low acidity","use body and fruit profile"],"typical_misconceptions":["Spatlese must be sweet","more sweetness means lower acidity","Spatlese equals botrytis"],"mentor_focus":["calibrate concentration relative to Kabinett"],"exam_traps":["overcalling Auslese","ignoring dry Spatlese possibility"],"memory_hooks":["Spatlese is Kabinett with more ripeness and stone fruit"],"comparison_styles":["Riesling Kabinett","Riesling Auslese","Mosel Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_016","SAT_WINE_018"],"frequently_confused_with":["SAT_WINE_016","SAT_WINE_018"],"distinguishing_features":["riper and fuller than Kabinett","less rich and botrytis-influenced than Auslese","stone fruit more common"]}</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Spatlese wines are more concentrated, riper and have more body, alcohol, and sweetness than Kabinett from the same region","citrus and stone fruit aromas are common"],"mentor_hints":["Ask what changed from Kabinett: ripeness, body, alcohol, and sweetness.","Do not rely on sweetness alone."],"student_traps":["forgetting dry style possibility","calling all stone-fruited Riesling Auslese"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","pradikat_riesling_scale"]</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10528-10537"],"line_reference":["10528-10537"],"evidence":["Spatlese is described as more concentrated, riper and with more body, alcohol and sweetness than Kabinett.","Citrus and stone fruit aromas are common."]}</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>Riesling - Spatlese</t>
+        </is>
+      </c>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>["10528-10537"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SAT_WINE_018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Riesling Auslese</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Rich selected extra-ripe bunch Riesling</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Riesling Auslese</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Pradikat category</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Auslese</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>cool continental German Riesling sites with selected extra-ripe bunches</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>varies by region; best sites maximize sunlight and warmth</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>varies by region</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>["made from individually selected extra-ripe bunches","noble rot can play an important role","multiple pickings support selection"]</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>["dry to sweet styles possible","fermentation may stop naturally or be stopped depending on sweetness","MLF and new oak avoided"]</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>no new oak; aromatic purity and noble-rot complexity where present</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>dry to sweet, often sweet in classic SAT examples</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>medium to full compared with Spatlese</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>low to medium in sweet styles; medium to high in dry styles</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>medium lemon to gold</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>["ripe peach","apricot","honey","citrus peel","botrytis spice possible"]</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>["ripe stone fruit","honey","citrus peel","sweet-acid balance","botrytis complexity possible"]</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>very good to outstanding; richer and riper than Spatlese</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>long ageing potential in high-quality sweet examples</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>["medium lemon","gold possible","pronounced intensity","ripe peach","apricot","honey","citrus peel","noble rot note possible","dry to sweet","high acidity","medium to full body","rich ripe fruit","long finish"]</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>["Auslese is made from individually selected extra-ripe bunches","wines are richer and riper than Spatlese","noble rot can play an important part regardless of dry or sweet style"]</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>["Auslese is always botrytised","Auslese must be sweet","richness means low acidity"]</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>["Look for extra ripeness and possible botrytis, but keep category boundaries clear.","Ask whether the wine is BA-level sweet and low alcohol or merely Auslese-rich."]</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>["medium lemon","gold possible","pronounced intensity","ripe peach","apricot","honey","citrus peel","noble rot note possible","dry to sweet","high acidity","medium to full body","rich ripe fruit","long finish","selected extra-ripe bunches","richer and riper than Spatlese","noble rot can influence flavour","long sweet-acid finish"]</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>["do not state Auslese is always sweet","do not make noble rot essential"]</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>Auslese profile follows WSET Pradikat category and standard SAT sweet Riesling calibration.</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 018</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium lemon","gold possible"],"nose":["pronounced intensity","ripe peach","apricot","honey","citrus peel","noble rot note possible"],"palate":["dry to sweet","high acidity","medium to full body","rich ripe fruit","long finish"],"quality":["very good to outstanding when richness and acidity balance"],"ageing":["excellent ageing potential, especially sweet examples"],"diagnostic_features":["selected extra-ripe bunches","richer and riper than Spatlese","noble rot can influence flavour","long sweet-acid finish"]}</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["selected bunch ripeness","noble rot influence","Pradikat escalation"],"learning_objectives":["distinguish Auslese from Spatlese and BA","recognize botrytis as possible but not mandatory","assess richness without losing acidity"],"typical_misconceptions":["Auslese is always botrytised","Auslese must be sweet","richness means low acidity"],"mentor_focus":["make students justify category by ripeness and concentration"],"exam_traps":["confusing Auslese with BA/TBA","forgetting dry Auslese can exist"],"memory_hooks":["Auslese is selected bunch richness before the berry-by-berry sweet wine tier"],"comparison_styles":["Riesling Spatlese","Beerenauslese","Trockenbeerenauslese"]}</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_017","SAT_WINE_019"],"frequently_confused_with":["SAT_WINE_017","SAT_WINE_019"],"distinguishing_features":["richer than Spatlese","less extreme and not necessarily berry-selected like BA","noble rot can play a role but is not the whole identity"]}</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Auslese is made from individually selected extra-ripe bunches","wines are richer and riper than Spatlese","noble rot can play an important part regardless of dry or sweet style"],"mentor_hints":["Look for extra ripeness and possible botrytis, but keep category boundaries clear.","Ask whether the wine is BA-level sweet and low alcohol or merely Auslese-rich."],"student_traps":["making noble rot mandatory","overcalling TBA from honey alone"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","pradikat_riesling_scale","botrytised_sweet_wine"]</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10538-10548"],"line_reference":["10538-10548"],"evidence":["Auslese is described as individually selected extra-ripe bunches.","Richer and riper than Spatlese, with noble rot able to play an important role."]}</t>
+        </is>
+      </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr">
+        <is>
+          <t>Riesling - Auslese</t>
+        </is>
+      </c>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>["10538-10548"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SAT_WINE_019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Beerenauslese</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Sweet botrytised berry-selected Riesling</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Beerenauslese</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Pradikat category</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Beerenauslese</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>cool continental regions where noble rot can develop in suitable humid autumn conditions</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>varies by site; humidity and autumn conditions are more diagnostic than altitude</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>varies by region</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>["BA not necessarily made every year","noble rot is typical though not essential for minimum must weight","selection of very ripe affected berries requires intensive hand work"]</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>["fermentation of highly concentrated must often stops with low alcohol","MLF and new oak avoided","made as sweet wine only"]</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>no new oak; botrytis and Riesling purity dominate</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>sweet only</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>full and viscous despite low alcohol</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>gold to deep gold</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>["honey","dried stone fruit","candied peel","flowers","apricot","botrytis spice"]</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>["honey","dried apricot","candied citrus peel","flowers","intense sweetness balanced by acidity"]</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>very long</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>outstanding; among the best sweet wines in the world</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>very long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>["gold","deep gold possible","viscous tears","pronounced intensity","honey","dried stone fruit","candied peel","flowers","botrytis","sweet","high acidity","low alcohol","full viscous body","very concentrated dried fruit and honey"]</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>["BA wines are sweet and low in alcohol with honey, dried stone fruit, candied peel, and flowers","noble rot is typical for BA but not essential for the legal must weight","BA and TBA are not necessarily made every year"]</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>["BA is just sweeter Auslese","low alcohol means low quality","botrytis is a fault here"]</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>["Ask whether the profile is botrytis or frozen-grape purity.","Use low alcohol plus high sweetness as a clue."]</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>["gold","deep gold possible","viscous tears","pronounced intensity","honey","dried stone fruit","candied peel","flowers","botrytis","sweet","high acidity","low alcohol","full viscous body","very concentrated dried fruit and honey","sweet only","noble rot typical","honey dried stone fruit candied peel flowers","not made every year"]</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>["do not make BA annually produced","do not describe BA as dry"]</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>BA profile uses WSET Pradikat and sweet winemaking passages; SAT additions clarify appearance and texture.</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 019</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>{"appearance":["gold","deep gold possible","viscous tears"],"nose":["pronounced intensity","honey","dried stone fruit","candied peel","flowers","botrytis"],"palate":["sweet","high acidity","low alcohol","full viscous body","very concentrated dried fruit and honey"],"quality":["outstanding when sweetness, acidity, concentration, and length align"],"ageing":["very long ageing potential"],"diagnostic_features":["sweet only","low alcohol","noble rot typical","honey dried stone fruit candied peel flowers","not made every year"]}</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["botrytised sweet wine","low alcohol from concentrated must","sweet-acid balance"],"learning_objectives":["distinguish BA from Auslese and TBA","recognize botrytis descriptors","understand annual rarity"],"typical_misconceptions":["BA is just sweeter Auslese","low alcohol means low quality","botrytis is a fault here"],"mentor_focus":["anchor quality in balance and concentration"],"exam_traps":["forgetting noble rot is typical but not essential for BA","confusing BA with Eiswein"],"memory_hooks":["BA is honeyed botrytis richness with Riesling acidity"],"comparison_styles":["Riesling Auslese","Trockenbeerenauslese","Eiswein"]}</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_020"],"frequently_confused_with":["SAT_WINE_018","SAT_WINE_021"],"distinguishing_features":["sweeter and more botrytised than Auslese","less extreme than TBA","botrytis-driven unlike Eiswein purity"]}</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["BA wines are sweet and low in alcohol with honey, dried stone fruit, candied peel, and flowers","noble rot is typical for BA but not essential for the legal must weight","BA and TBA are not necessarily made every year"],"mentor_hints":["Ask whether the profile is botrytis or frozen-grape purity.","Use low alcohol plus high sweetness as a clue."],"student_traps":["calling BA Eiswein from high acidity","forgetting low alcohol"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","botrytised_sweet_wine"]</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10549-10568","5849-5875"],"line_reference":["10549-10568","5849-5875"],"evidence":["BA/TBA wines are described as sweet and low alcohol with honey, dried stone fruit, candied peel, and flowers.","Noble rot is typical for BA but essential for TBA."]}</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>Beerenauslese and Trockenbeerenauslese</t>
+        </is>
+      </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>109-110</t>
+        </is>
+      </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>["10549-10568","5849-5875"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SAT_WINE_020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Trockenbeerenauslese</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Extremely sweet noble-rot Riesling from shrivelled berries</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Trockenbeerenauslese</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Pradikat category</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Trockenbeerenauslese</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>cool continental regions with rare noble rot conditions: humid mornings and dry afternoons</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>varies by site; noble rot conditions are more diagnostic than altitude</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>varies by region</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>["noble rot is essential","TBA is not necessarily made every year","berry selection is extremely labor intensive"]</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>["fermentation of extremely concentrated must stops naturally at low alcohol","made as sweet wine only","MLF and new oak avoided"]</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>no new oak; noble rot concentration dominates</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>sweet only, extremely sweet</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>full, viscous and concentrated</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>low, sometimes around 7% abv due to sugar concentration</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>deep gold to amber</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>["honey","marmalade","dried apricot","candied peel","dried fruit","botrytis spice"]</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>["honey","dried stone fruit","candied citrus","marmalade","intense botrytis concentration"]</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>exceptionally long</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>outstanding; among the worlds greatest sweet wines</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>very long ageing potential, often decades</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>["deep gold","amber possible","very viscous","pronounced intensity","honey","dried apricot","candied peel","dried fruit","botrytis complexity","lusciously sweet","high acidity","low alcohol","full viscous body","exceptionally concentrated flavours"]</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>["Noble rot is essential for TBA","TBA wines are sweet only and low in alcohol","German TBAs are classic examples of fermentation stopping naturally at low alcohol in very sugary must"]</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>["Trocken means dry in this word","TBA is the same as Eiswein","high sugar means low acidity"]</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>["Ask what concentrated the sugars: botrytis, not freezing.","Flag the word Trocken as a naming trap."]</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>["deep gold","amber possible","very viscous","pronounced intensity","honey","dried apricot","candied peel","dried fruit","botrytis complexity","lusciously sweet","high acidity","low alcohol","full viscous body","exceptionally concentrated flavours","noble rot essential","sweet only","very low alcohol possible","extreme concentration","longest botrytised finish"]</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>["do not translate Trockenbeerenauslese as dry wine","do not describe TBA without noble rot"]</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>TBA profile combines WSET German Pradikat and sweet winemaking passages with standard SAT appearance.</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 020</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep gold","amber possible","very viscous"],"nose":["pronounced intensity","honey","dried apricot","candied peel","dried fruit","botrytis complexity"],"palate":["lusciously sweet","high acidity","low alcohol","full viscous body","exceptionally concentrated flavours"],"quality":["outstanding when acidity balances extreme sugar and concentration"],"ageing":["decades of ageing potential"],"diagnostic_features":["noble rot essential","sweet only","very low alcohol possible","extreme concentration","longest botrytised finish"]}</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["noble rot concentration","extreme Pradikat must weight","natural fermentation stop"],"learning_objectives":["distinguish TBA from BA and Eiswein","understand why alcohol can be very low","identify botrytis flavour set"],"typical_misconceptions":["Trocken means dry in this word","TBA is the same as Eiswein","high sugar means low acidity"],"mentor_focus":["correct the Trockenbeerenauslese naming trap directly"],"exam_traps":["thinking TBA is dry because of Trocken","missing noble rot essentiality"],"memory_hooks":["TBA is not dry: it is the shrivelled noble-rot summit"],"comparison_styles":["Beerenauslese","Eiswein","Sauternes"]}</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_019"],"frequently_confused_with":["SAT_WINE_019","SAT_WINE_021"],"distinguishing_features":["more extreme and concentrated than BA","noble rot essential unlike Eiswein","sweet only despite Trocken in the name"]}</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Noble rot is essential for TBA","TBA wines are sweet only and low in alcohol","German TBAs are classic examples of fermentation stopping naturally at low alcohol in very sugary must"],"mentor_hints":["Ask what concentrated the sugars: botrytis, not freezing.","Flag the word Trocken as a naming trap."],"student_traps":["assuming dry from Trocken","confusing with Eiswein purity"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","botrytised_sweet_wine"]</t>
+        </is>
+      </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10549-10568","5849-5875"],"line_reference":["10549-10568","5849-5875"],"evidence":["Noble rot is essential to achieve the must weights for TBA.","TBA is sweet only and low in alcohol with honey, dried stone fruit, candied peel, and flowers."]}</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>Trockenbeerenauslese</t>
+        </is>
+      </c>
+      <c r="BA21" t="inlineStr">
+        <is>
+          <t>109-110</t>
+        </is>
+      </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>["10549-10568","5849-5875"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SAT_WINE_021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Blancos Alemania</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Eiswein</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Sweet high-acid Riesling from frozen healthy grapes</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Eiswein</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Pradikat category</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Eiswein</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>cool continental regions cold enough for grapes to freeze on the vine</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>varies by site; freezing conditions and healthy grapes are more diagnostic than altitude</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>varies by region</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>["healthy grapes left hanging into winter","grapes are picked and pressed while frozen","made infrequently and is a genuine rarity"]</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>["noble rot is not a key component","careful juice handling preserves varietal purity","MLF and new oak avoided"]</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>no new oak; varietal purity is the focus</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>sweet only</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>medium to full depending on concentration</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>very high</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>low to medium, usually lower because sugar remains unfermented</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>pale gold to gold</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>["pure citrus","green apple","peach","floral notes","honey with age"]</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>["pure Riesling fruit","citrus","apple","peach","intense sweetness balanced by very high acidity"]</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>very long, pure and acid-bright</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>very good to outstanding; best examples show fine balance between acidity and sweetness</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>long ageing potential due to acidity and sugar</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>["pale gold","gold","pronounced intensity","pure citrus","green apple","peach","floral notes","no botrytis emphasis","sweet","very high acidity","low to medium alcohol","medium to full body","pure varietal fruit","long finish"]</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>["Eiswein is made infrequently and is a genuine rarity","noble rot is not key; focus is varietal purity","best examples balance acidity and sweetness finely"]</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>["Eiswein is botrytised","all sweet German wines are BA/TBA","Eiswein is just frozen TBA"]</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>["Ask whether descriptors are pure fruit or botrytis honey/dried fruit.","Freezing is the concentration mechanism."]</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>["pale gold","gold","pronounced intensity","pure citrus","green apple","peach","floral notes","no botrytis emphasis","sweet","very high acidity","low to medium alcohol","medium to full body","pure varietal fruit","long finish","frozen healthy grapes","noble rot not key","pure varietal character","very high acidity and sweetness balance","rarity"]</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>["do not describe noble rot as key for Eiswein","do not make Eiswein dry"]</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>Eiswein profile is anchored in WSET German Pradikat text and sweet winemaking freezing description.</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Alemania - Practica 021</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Germany is the homeland of Riesling and produces dry to lusciously sweet Riesling.","German wine regions have cool continental climates, steep south-facing slopes, and Pradikat categories based on must weight."],"standard_wine_knowledge":["Typical SAT appearance, aroma intensity, finish, and alcohol ranges are calibrated from accepted German Riesling style norms."],"derived_from_style":["Difficulty, comparison, and diagnostic features are derived from regional or Pradikat style."],"inferred_high_confidence":["Mentor traps and memory hooks are pedagogical inferences from WSET style contrasts."]}</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale gold","gold"],"nose":["pronounced intensity","pure citrus","green apple","peach","floral notes","no botrytis emphasis"],"palate":["sweet","very high acidity","low to medium alcohol","medium to full body","pure varietal fruit","long finish"],"quality":["outstanding where sweetness and acidity are finely balanced"],"ageing":["long ageing potential"],"diagnostic_features":["frozen healthy grapes","noble rot not key","pure varietal character","very high acidity and sweetness balance","rarity"]}</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["freezing grapes on the vine","varietal purity","sweet-acid balance without botrytis"],"learning_objectives":["distinguish Eiswein from BA/TBA","connect freezing to concentration","recognize purity rather than honeyed botrytis"],"typical_misconceptions":["Eiswein is botrytised","all sweet German wines are BA/TBA","Eiswein is just frozen TBA"],"mentor_focus":["ask what concentrated the sugars and whether botrytis is present"],"exam_traps":["calling Eiswein TBA because both are sweet","forgetting rarity and healthy grapes"],"memory_hooks":["Eiswein is Riesling purity frozen in place"],"comparison_styles":["Beerenauslese","Trockenbeerenauslese","Canadian Icewine"]}</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_019","SAT_WINE_020"],"frequently_confused_with":["SAT_WINE_019","SAT_WINE_020"],"distinguishing_features":["pure fruit rather than botrytis honey-candied peel profile","noble rot not key","freezing rather than fungal dehydration"]}</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Eiswein is made infrequently and is a genuine rarity","noble rot is not key; focus is varietal purity","best examples balance acidity and sweetness finely"],"mentor_hints":["Ask whether descriptors are pure fruit or botrytis honey/dried fruit.","Freezing is the concentration mechanism."],"student_traps":["confusing all sweet Riesling with botrytis","missing very high acidity"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>["german_riesling_core","eiswein_purity"]</t>
+        </is>
+      </c>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW22" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10569-10582","5867-5878"],"line_reference":["10569-10582","5867-5878"],"evidence":["Eiswein is described as rare, with noble rot not a key component and focus on varietal purity.","Freezing grapes on the vine concentrates sugar in Germany and Icewine in Canada."]}</t>
+        </is>
+      </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-03-BATCH-002","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY22" t="inlineStr">
+        <is>
+          <t>22 Germany</t>
+        </is>
+      </c>
+      <c r="AZ22" t="inlineStr">
+        <is>
+          <t>Eiswein</t>
+        </is>
+      </c>
+      <c r="BA22" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>["10569-10582","5867-5878"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add Batch 003 Austria white profiles
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -5994,6 +5994,1638 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SAT_WINE_022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Blancos Austria</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Wachau Grüner Veltliner</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Concentrated dry Grüner Veltliner from steep Danube terraces</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Wachau Grüner Veltliner</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Wachau</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Niederösterreich / Danube</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Wachau</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>["Grüner Veltliner"]</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>cool continental Austrian climate with short summers and harsh winters; Wachau benefits from steep Danube exposure</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>steep, often terraced south-facing vineyards next to the Danube</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>varied terraced Danube valley soils; exposure and terraces are primary WSET markers</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>["steep terraced south-facing vineyards maximize exposure to the sun","careful growing is needed for concentration","high yields can make Grüner Veltliner fresh but unexciting"]</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>["majority fermented and stored in stainless steel","old oak casks are commonly used","some producers mature a proportion of best wines in new oak barriques"]</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>usually stainless steel or old oak; best wines may see some new oak proportion</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","white pepper","honey and toast with age"]</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","white pepper","concentrated dry palate","honey and toast with age"]</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>long in best concentrated examples</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>very good to outstanding; Wachau is renowned for high-quality dry wines from Grüner Veltliner or Riesling</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>medium to long ageing for top concentrated examples</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age","dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and stone fruit"]</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>["Grüner Veltliner is Austrias most widely planted variety","careful growing can produce full-bodied concentrated wines with naturally high acidity","Wachau is renowned for high-quality dry wines from Grüner Veltliner or Riesling"]</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>["all pepper is oak","Austria is only Riesling","full body means low acidity"]</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>["Ask whether pepper is varietal rather than oak-derived.","Use Wachau terraces as the causal structure."]</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age","dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and stone fruit","Grüner Veltliner white pepper","Wachau concentration","dry high-acid palate","terraced Danube vineyards"]</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>["do not make Wachau sweet by default","do not omit naturally high acidity"]</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Grüner Veltliner and Wachau passages; SAT colour and alcohol are standard style calibration.</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Austria - Practica 022</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Austria is best known for quality dry white wines from Grüner Veltliner and Riesling.","Wachau, Kamptal, Kremstal, Weinviertel, Burgenland and Neusiedlersee are described in the Austria chapter."],"standard_wine_knowledge":["SAT appearance, intensity, alcohol, finish and diagnostic calibration use widely accepted Austrian white wine style norms."],"derived_from_style":["Difficulty, comparisons and learning traps are derived from WSET regional and varietal contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age"],"palate":["dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and stone fruit"],"quality":["very good to outstanding when concentration, acidity and length align"],"ageing":["best examples can develop honey and toast with age"],"diagnostic_features":["Grüner Veltliner white pepper","Wachau concentration","dry high-acid palate","terraced Danube vineyards"]}</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Austrian dry white identity","Grüner Veltliner typicity","terrace and exposure effect"],"learning_objectives":["identify Grüner Veltliner versus Riesling","link Wachau terraces to concentration","separate white pepper from oak spice"],"typical_misconceptions":["all pepper is oak","Austria is only Riesling","full body means low acidity"],"mentor_focus":["ask for pepper, acidity and concentration together"],"exam_traps":["calling concentrated dry Grüner Veltliner Chardonnay","forgetting old oak is not new oak flavour by default"],"memory_hooks":["Wachau Grüner is dry, concentrated, high-acid and pepper-edged"],"comparison_styles":["Wachau Riesling","Weinviertel Grüner Veltliner","Alsace Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_025","SAT_WINE_026"],"frequently_confused_with":["SAT_WINE_023","SAT_WINE_024"],"distinguishing_features":["white pepper distinguishes from Riesling","more concentrated than Weinviertel Klassik","Wachau terrace context"]}</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Grüner Veltliner is Austrias most widely planted variety","careful growing can produce full-bodied concentrated wines with naturally high acidity","Wachau is renowned for high-quality dry wines from Grüner Veltliner or Riesling"],"mentor_hints":["Ask whether pepper is varietal rather than oak-derived.","Use Wachau terraces as the causal structure."],"student_traps":["missing Grüner Veltliner because of Riesling bias","overcalling sweetness from richness"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>["austrian_gruner_veltliner_core","wachau_dry_white_core"]</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW23" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10985-10999","11144-11154"],"line_reference":["10985-10999","11144-11154"],"evidence":["Grüner Veltliner can produce full-bodied concentrated wines with naturally high acidity, citrus or stone fruit and white pepper.","Wachau is renowned for high-quality dry wines from Grüner Veltliner or Riesling on steep terraced south-facing Danube vineyards."]}</t>
+        </is>
+      </c>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-04-BATCH-003","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY23" t="inlineStr">
+        <is>
+          <t>23 Austria</t>
+        </is>
+      </c>
+      <c r="AZ23" t="inlineStr">
+        <is>
+          <t>White Grape Varieties / Niederösterreich - Wachau</t>
+        </is>
+      </c>
+      <c r="BA23" t="inlineStr">
+        <is>
+          <t>113-114</t>
+        </is>
+      </c>
+      <c r="BB23" t="inlineStr">
+        <is>
+          <t>["10985-10999","11144-11154"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SAT_WINE_023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Blancos Austria</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Wachau Riesling</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Dry medium- to full-bodied Austrian Riesling</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Wachau Riesling</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Wachau</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Niederösterreich / Danube</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Wachau</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>cool continental Austrian climate; steep Danube terraces maximize sun exposure</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>steep, often terraced south-facing vineyards next to the Danube</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>varied terraced Danube valley soils; exposure and terraces are primary WSET markers</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>["steep terraced south-facing vineyards maximize exposure to the sun","Riesling develops highly concentrated flavours in Wachau","best Austrian Rieslings tend to come from Wachau, Kamptal and Kremstal"]</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>["usually dry","aroma-preserving white winemaking","new oak is not a diagnostic Riesling marker"]</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>typically stainless steel or neutral vessels; new oak not diagnostic</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>["ripe peach","citrus","stone fruit","honey with age"]</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>["ripe peach","citrus","stone fruit","dry mineral length"]</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>very good to outstanding; best examples capable of maturing in bottle</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>medium to long ageing in best examples</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","ripe peach","citrus","stone fruit","honey with age","dry","high acidity","medium to full body","medium to high alcohol","ripe peachy primary fruit"]</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>["Austrian Riesling is less widely planted than Grüner Veltliner","best examples tend to come from Wachau, Kamptal and Kremstal","they are usually dry and medium- to full-bodied with ripe peachy primary fruit"]</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>["all Riesling is sweet","Austrian Riesling tastes like Grüner Veltliner","dry Riesling lacks ageing potential"]</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>["Check whether the candidate is importing German sweetness assumptions.","Use ripe peach plus dry full body as a clue."]</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","ripe peach","citrus","stone fruit","honey with age","dry","high acidity","medium to full body","medium to high alcohol","ripe peachy primary fruit","dry Austrian Riesling","ripe peachy fruit","Wachau terrace concentration"]</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>["do not treat Austrian Riesling as normally sweet","do not add Grüner white pepper"]</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Austrian Riesling and Wachau passages; SAT structure uses standard dry Riesling calibration.</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Austria - Practica 023</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Austria is best known for quality dry white wines from Grüner Veltliner and Riesling.","Wachau, Kamptal, Kremstal, Weinviertel, Burgenland and Neusiedlersee are described in the Austria chapter."],"standard_wine_knowledge":["SAT appearance, intensity, alcohol, finish and diagnostic calibration use widely accepted Austrian white wine style norms."],"derived_from_style":["Difficulty, comparisons and learning traps are derived from WSET regional and varietal contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","ripe peach","citrus","stone fruit","honey with age"],"palate":["dry","high acidity","medium to full body","medium to high alcohol","ripe peachy primary fruit"],"quality":["very good to outstanding when dry concentration and acidity balance"],"ageing":["best examples can mature in bottle"],"diagnostic_features":["dry Austrian Riesling","ripe peachy fruit","medium to full body","Wachau terrace concentration"]}</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["dry Austrian Riesling","Danube terrace concentration","Riesling without German Prädikat sweetness frame"],"learning_objectives":["distinguish Austrian from German Riesling","separate Riesling from Grüner Veltliner","connect Wachau to dry concentration"],"typical_misconceptions":["all Riesling is sweet","Austrian Riesling tastes like Grüner Veltliner","dry Riesling lacks ageing potential"],"mentor_focus":["ask for dry structure and peachy primary fruit"],"exam_traps":["adding white pepper from Grüner","assuming low alcohol Mosel style"],"memory_hooks":["Wachau Riesling is dry, peachy, concentrated and ageworthy"],"comparison_styles":["Wachau Grüner Veltliner","German Rheingau Riesling","Alsace Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_013","SAT_WINE_005"],"frequently_confused_with":["SAT_WINE_022","SAT_WINE_013"],"distinguishing_features":["no white pepper unlike Grüner","drier and fuller than many Mosel styles","Austrian Wachau context"]}</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Austrian Riesling is less widely planted than Grüner Veltliner","best examples tend to come from Wachau, Kamptal and Kremstal","they are usually dry and medium- to full-bodied with ripe peachy primary fruit"],"mentor_hints":["Check whether the candidate is importing German sweetness assumptions.","Use ripe peach plus dry full body as a clue."],"student_traps":["confusing Riesling and Grüner in Wachau","forgetting bottle maturation potential"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t>["wachau_dry_white_core","german_riesling_core"]</t>
+        </is>
+      </c>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW24" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11008-11014","11144-11154"],"line_reference":["11008-11014","11144-11154"],"evidence":["Best Austrian Rieslings tend to come from Wachau, Kamptal and Kremstal and are usually dry, medium- to full-bodied with ripe peachy fruit.","Wachau has steep terraced south-facing vineyards next to the Danube."]}</t>
+        </is>
+      </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-04-BATCH-003","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY24" t="inlineStr">
+        <is>
+          <t>23 Austria</t>
+        </is>
+      </c>
+      <c r="AZ24" t="inlineStr">
+        <is>
+          <t>Riesling / Niederösterreich - Wachau</t>
+        </is>
+      </c>
+      <c r="BA24" t="inlineStr">
+        <is>
+          <t>113-114</t>
+        </is>
+      </c>
+      <c r="BB24" t="inlineStr">
+        <is>
+          <t>["11008-11014","11144-11154"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SAT_WINE_024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Blancos Austria</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Weinviertel Grüner Veltliner</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Light fresh fruity Grüner Veltliner Klassik</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Weinviertel Grüner Veltliner</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Weinviertel</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Niederösterreich</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Weinviertel DAC</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>["Grüner Veltliner"]</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>cool continental Austrian climate; more northerly areas can experience cooling winds</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>varies; DAC style is more diagnostic than altitude</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>varied Weinviertel soils; WSET focuses on DAC style rules</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>["Austria largest vine-growing area","DAC wines can only be Grüner Veltliner","yield control matters for quality"]</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>["Klassik wines are light, fresh and fruity with no discernible oak flavours","Reserve wines have higher minimum alcohol and may be matured in oak"]</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>no discernible oak for Klassik; Reserve may be oaked</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>light to medium for Klassik; fuller for Reserve</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>medium for Klassik; higher for Reserve</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>["citrus","green apple","stone fruit","white pepper"]</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>["fresh citrus","green apple","white pepper","fresh fruity finish"]</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>good to very good depending on Klassik or Reserve level</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>drink now for Klassik; Reserve may age short to medium term</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium intensity","citrus","green apple","white pepper","fresh fruit","dry","high acidity","light to medium body","medium alcohol","fresh fruity style","no discernible oak in Klassik"]</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>["Weinviertel DAC is Austria’s largest vine-growing area and first DAC","wines can only be made from Grüner Veltliner","Klassik must be light, fresh and fruity with no discernible oak flavours"]</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>["all Grüner Veltliner is full-bodied","all Reserve rules apply to Klassik","fresh fruity means low quality"]</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>["Ask whether the wine is Klassik or Reserve in style.","Use no-oak freshness to separate from richer examples."]</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium intensity","citrus","green apple","white pepper","fresh fruit","dry","high acidity","light to medium body","medium alcohol","fresh fruity style","no discernible oak in Klassik","Weinviertel DAC only Grüner Veltliner","light fresh fruity Klassik","no discernible oak"]</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>["do not assign oak to Klassik","do not confuse Weinviertel with Wachau concentration"]</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Weinviertel DAC text and Grüner Veltliner varietal passage; SAT descriptors are standard style calibration.</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Austria - Practica 024</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Austria is best known for quality dry white wines from Grüner Veltliner and Riesling.","Wachau, Kamptal, Kremstal, Weinviertel, Burgenland and Neusiedlersee are described in the Austria chapter."],"standard_wine_knowledge":["SAT appearance, intensity, alcohol, finish and diagnostic calibration use widely accepted Austrian white wine style norms."],"derived_from_style":["Difficulty, comparisons and learning traps are derived from WSET regional and varietal contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium intensity","citrus","green apple","white pepper","fresh fruit"],"palate":["dry","high acidity","light to medium body","medium alcohol","fresh fruity style","no discernible oak in Klassik"],"quality":["good to very good depending on concentration and DAC level"],"ageing":["Klassik is usually early drinking; Reserve can develop further"],"diagnostic_features":["Weinviertel DAC only Grüner Veltliner","light fresh fruity Klassik","no discernible oak","white pepper"]}</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["DAC style identity","Klassik versus Reserve","Grüner Veltliner freshness"],"learning_objectives":["distinguish Weinviertel from Wachau","connect DAC to grape/style rules","identify white pepper in lighter context"],"typical_misconceptions":["all Grüner Veltliner is full-bodied","all Reserve rules apply to Klassik","fresh fruity means low quality"],"mentor_focus":["ask for style level before quality conclusion"],"exam_traps":["adding oak to Klassik","forgetting Weinviertel can only be Grüner Veltliner"],"memory_hooks":["Weinviertel Klassik is Austria’s fresh peppery Grüner baseline"],"comparison_styles":["Wachau Grüner Veltliner","Kamptal Grüner Veltliner","Muscadet"]}</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_025","SAT_WINE_026"],"frequently_confused_with":["SAT_WINE_022"],"distinguishing_features":["lighter than Wachau","DAC grape restriction","Klassik no discernible oak"]}</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Weinviertel DAC is Austria’s largest vine-growing area and first DAC","wines can only be made from Grüner Veltliner","Klassik must be light, fresh and fruity with no discernible oak flavours"],"mentor_hints":["Ask whether the wine is Klassik or Reserve in style.","Use no-oak freshness to separate from richer examples."],"student_traps":["overstating body and oak","missing DAC restriction"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>["austrian_gruner_veltliner_core"]</t>
+        </is>
+      </c>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW25" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11156-11167"],"line_reference":["11156-11167"],"evidence":["Weinviertel DAC wines can only be made from Grüner Veltliner.","Klassik wines must be light, fresh and fruity with no discernible oak flavours."]}</t>
+        </is>
+      </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-04-BATCH-003","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY25" t="inlineStr">
+        <is>
+          <t>23 Austria</t>
+        </is>
+      </c>
+      <c r="AZ25" t="inlineStr">
+        <is>
+          <t>Weinviertel DAC</t>
+        </is>
+      </c>
+      <c r="BA25" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="BB25" t="inlineStr">
+        <is>
+          <t>["11156-11167"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SAT_WINE_025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Blancos Austria</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Kamptal Grüner Veltliner</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>High-quality dry Grüner Veltliner from Kamptal DAC</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Kamptal Grüner Veltliner</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Kamptal</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Niederösterreich</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Kamptal DAC</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>["Grüner Veltliner"]</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>cool continental Austrian climate; Kamptal lies north of Wachau and produces similar style and quality</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>varied valley and slope sites; regional proximity to Wachau is more diagnostic than exact altitude</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>varied Kamptal soils; WSET emphasizes similar style and quality to Wachau</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>["Kamptal DAC lies just north of Wachau","Grüner Veltliner develops quality dry wines when grown with care","yield control is important for concentration"]</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>["dry white winemaking","stainless steel common","old oak casks may be used; some best wines may see new oak proportion"]</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>stainless steel or old oak common; new oak possible for some best wines</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","white pepper","honey and toast with age"]</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","white pepper","concentrated dry palate"]</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>good to outstanding; Kamptal produces similar style and quality to Wachau from Grüner Veltliner or Riesling</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>medium to long ageing for best examples</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age","dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and pepper"]</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>["Kamptal DAC lies just north of Wachau","it produces wines in a similar style and quality from Grüner Veltliner or Riesling","Grüner Veltliner can be full-bodied, concentrated and naturally high in acidity"]</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>["Kamptal is lower quality by default","pepper means oak","all DACs have same rules as Weinviertel"]</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>["Ask if the profile is regional quality rather than Wachau specifically.","Use pepper plus dry high acid as the variety anchor."]</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age","dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and pepper","Kamptal DAC north of Wachau","similar style and quality to Wachau","Grüner Veltliner pepper and high acidity"]</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>["do not make Kamptal a sweet style","do not omit Grüner Veltliner pepper marker"]</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Kamptal regional line and Grüner Veltliner style paragraph; SAT details are standard calibration.</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Austria - Practica 025</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Austria is best known for quality dry white wines from Grüner Veltliner and Riesling.","Wachau, Kamptal, Kremstal, Weinviertel, Burgenland and Neusiedlersee are described in the Austria chapter."],"standard_wine_knowledge":["SAT appearance, intensity, alcohol, finish and diagnostic calibration use widely accepted Austrian white wine style norms."],"derived_from_style":["Difficulty, comparisons and learning traps are derived from WSET regional and varietal contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ26" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age"],"palate":["dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and pepper"],"quality":["good to outstanding depending on concentration and balance"],"ageing":["best examples can develop honey and toast"],"diagnostic_features":["Kamptal DAC north of Wachau","similar style and quality to Wachau","Grüner Veltliner pepper and high acidity"]}</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Kamptal DAC","Grüner Veltliner quality spectrum","dry Austrian white structure"],"learning_objectives":["compare Kamptal with Wachau and Kremstal","identify pepper and high acidity","avoid over-specific Wachau assumptions"],"typical_misconceptions":["Kamptal is lower quality by default","pepper means oak","all DACs have same rules as Weinviertel"],"mentor_focus":["train regional comparison rather than isolated recall"],"exam_traps":["calling every concentrated Austrian white Wachau","forgetting Kamptal can be Riesling or Grüner"],"memory_hooks":["Kamptal sits north of Wachau with a similar dry white quality language"],"comparison_styles":["Wachau Grüner Veltliner","Kremstal Grüner Veltliner","Weinviertel Grüner Veltliner"]}</t>
+        </is>
+      </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_022","SAT_WINE_026"],"frequently_confused_with":["SAT_WINE_022","SAT_WINE_026"],"distinguishing_features":["not as singularly Wachau-classification driven","more concentrated than basic Weinviertel","DAC region north of Wachau"]}</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Kamptal DAC lies just north of Wachau","it produces wines in a similar style and quality from Grüner Veltliner or Riesling","Grüner Veltliner can be full-bodied, concentrated and naturally high in acidity"],"mentor_hints":["Ask if the profile is regional quality rather than Wachau specifically.","Use pepper plus dry high acid as the variety anchor."],"student_traps":["overusing Wachau for all quality Austrian whites","forgetting Kamptal DAC"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>["austrian_gruner_veltliner_core"]</t>
+        </is>
+      </c>
+      <c r="AV26" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW26" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10985-10999","11151-11154"],"line_reference":["10985-10999","11151-11154"],"evidence":["Kamptal DAC lies just north of Wachau and produces similar style and quality from Grüner Veltliner or Riesling.","Grüner Veltliner can make full-bodied concentrated wines with naturally high acidity."]}</t>
+        </is>
+      </c>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-04-BATCH-003","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>23 Austria</t>
+        </is>
+      </c>
+      <c r="AZ26" t="inlineStr">
+        <is>
+          <t>Kamptal DAC</t>
+        </is>
+      </c>
+      <c r="BA26" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="BB26" t="inlineStr">
+        <is>
+          <t>["10985-10999","11151-11154"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SAT_WINE_026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Blancos Austria</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Kremstal Grüner Veltliner</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>High-quality dry Grüner Veltliner from Kremstal DAC</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Kremstal Grüner Veltliner</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Kremstal</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Niederösterreich</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Kremstal DAC</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>["Grüner Veltliner"]</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>cool continental Austrian climate; Kremstal lies north of Wachau and produces similar style and quality</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>varied Danube-adjacent and slope sites; regional style is more diagnostic than exact altitude</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>varied Kremstal soils; WSET emphasizes similar style and quality to Wachau</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>["Kremstal DAC lies just north of Wachau","quality depends on careful growing and controlled yields","Grüner Veltliner and Riesling are key varieties"]</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>["dry white winemaking","stainless steel common","old oak casks may be used; some best wines may see new oak proportion"]</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>stainless steel or old oak common; new oak possible for some best wines</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","white pepper","honey and toast with age"]</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","white pepper","concentrated dry palate"]</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>good to outstanding; Kremstal produces similar style and quality to Wachau from Grüner Veltliner or Riesling</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>medium to long ageing for best examples</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age","dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and pepper"]</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>["Kremstal DAC lies just north of Wachau","it produces wines in a similar style and quality from Grüner Veltliner or Riesling","Grüner Veltliner is naturally high in acidity and may show citrus, stone fruit and white pepper"]</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>["Kremstal is unrelated to Wachau style","full body removes acidity","pepper equals oak"]</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>["Ask whether the answer needs Kamptal/Kremstal pair recall.","Use white pepper to prevent Riesling confusion."]</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age","dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and pepper","Kremstal DAC north of Wachau","similar style and quality to Wachau","Grüner Veltliner pepper and high acidity"]</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>["do not make Kremstal sweet by default","do not omit high acidity"]</t>
+        </is>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Kremstal regional line and Grüner Veltliner style paragraph; SAT details are standard calibration.</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Austria - Practica 026</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Austria is best known for quality dry white wines from Grüner Veltliner and Riesling.","Wachau, Kamptal, Kremstal, Weinviertel, Burgenland and Neusiedlersee are described in the Austria chapter."],"standard_wine_knowledge":["SAT appearance, intensity, alcohol, finish and diagnostic calibration use widely accepted Austrian white wine style norms."],"derived_from_style":["Difficulty, comparisons and learning traps are derived from WSET regional and varietal contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ27" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","citrus","stone fruit","white pepper","honey or toast with age"],"palate":["dry","high acidity","medium to full body","medium to high alcohol","concentrated citrus and pepper"],"quality":["good to outstanding depending on concentration and balance"],"ageing":["best examples can develop honey and toast"],"diagnostic_features":["Kremstal DAC north of Wachau","similar style and quality to Wachau","Grüner Veltliner pepper and high acidity"]}</t>
+        </is>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Kremstal DAC","Grüner Veltliner concentration","dry Austrian white comparison"],"learning_objectives":["compare Kremstal with Kamptal and Wachau","identify Grüner Veltliner markers","connect high acidity to quality"],"typical_misconceptions":["Kremstal is unrelated to Wachau style","full body removes acidity","pepper equals oak"],"mentor_focus":["ask for variety marker first, then region precision"],"exam_traps":["forgetting Kremstal appears alongside Kamptal","calling it Riesling despite pepper"],"memory_hooks":["Kremstal mirrors the Wachau/Kamptal dry white language with Grüner bite"],"comparison_styles":["Kamptal Grüner Veltliner","Wachau Grüner Veltliner","Wachau Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_022","SAT_WINE_025"],"frequently_confused_with":["SAT_WINE_025","SAT_WINE_023"],"distinguishing_features":["paired with Kamptal in WSET as north of Wachau","pepper separates from Riesling","quality dry DAC context"]}</t>
+        </is>
+      </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Kremstal DAC lies just north of Wachau","it produces wines in a similar style and quality from Grüner Veltliner or Riesling","Grüner Veltliner is naturally high in acidity and may show citrus, stone fruit and white pepper"],"mentor_hints":["Ask whether the answer needs Kamptal/Kremstal pair recall.","Use white pepper to prevent Riesling confusion."],"student_traps":["collapsing Kremstal into Kamptal without naming both","missing high acidity"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>["austrian_gruner_veltliner_core"]</t>
+        </is>
+      </c>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW27" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["10985-10999","11151-11154"],"line_reference":["10985-10999","11151-11154"],"evidence":["Kremstal DAC lies just north of Wachau and produces similar style and quality from Grüner Veltliner or Riesling.","Grüner Veltliner can show citrus or stone fruit, white pepper and naturally high acidity."]}</t>
+        </is>
+      </c>
+      <c r="AX27" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-04-BATCH-003","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY27" t="inlineStr">
+        <is>
+          <t>23 Austria</t>
+        </is>
+      </c>
+      <c r="AZ27" t="inlineStr">
+        <is>
+          <t>Kremstal DAC</t>
+        </is>
+      </c>
+      <c r="BA27" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="BB27" t="inlineStr">
+        <is>
+          <t>["10985-10999","11151-11154"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SAT_WINE_027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Blancos Austria</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Neusiedlersee / Burgenland sweet Welschriesling</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Botrytised sweet white from Neusiedlersee and Burgenland</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Neusiedlersee / Burgenland Sweet Welschriesling</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Burgenland</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Neusiedlersee</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Burgenland / Neusiedlersee</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>["Welschriesling"]</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>eastern Austria warmed by easterly winds; low-lying Neusiedlersee vineyards benefit from autumn mists</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>low-lying ground near Neusiedlersee and wetland margins</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>low-lying lake-influenced vineyard land; botrytis conditions are the key source marker</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>["sweet wine vineyards are near the lake","autumn mists from lake and wetlands create ideal botrytis conditions","Welschriesling is widely used for these sweet wines"]</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>["botrytised dessert wine production","Austrian Prädikat terms mainly reserved for medium sweet and sweet wines","high sugar concentration balanced by acidity"]</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>not a diagnostic marker; botrytis and fruit concentration dominate</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>medium to full, viscous depending on concentration</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>low to medium depending on fermentation</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>gold to deep gold</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>["honey","apricot","citrus peel","dried fruit","botrytis spice"]</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>["honey","apricot","candied citrus","dried fruit","sweet-acid balance"]</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>long to very long</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>very good to outstanding; Burgenland is best known for top-quality sweet wines and red wines</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>long ageing potential for high-quality botrytised examples</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>["gold","deep gold possible","viscous tears possible","pronounced intensity","honey","apricot","citrus peel","dried fruit","botrytis spice","sweet","high acidity","medium to full body","low to medium alcohol","honeyed botrytised fruit"]</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>["Burgenland is best known for top-quality sweet wines and red wines","Neusiedlersee is key for sweet wine production","Welschriesling is one of the most widely used grapes for these sweet wines"]</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>["Welschriesling is Riesling","Austria only makes dry whites","botrytis is always a fault"]</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>["Ask whether the sweet wine is lake-botrytis driven.","Correct Welschriesling/Riesling confusion early."]</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>["gold","deep gold possible","viscous tears possible","pronounced intensity","honey","apricot","citrus peel","dried fruit","botrytis spice","sweet","high acidity","medium to full body","low to medium alcohol","honeyed botrytised fruit","Neusiedlersee autumn mists","botrytis almost guaranteed every year","Welschriesling sweet wine","not the same grape as Riesling"]</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>["do not confuse Welschriesling with Riesling","do not make Neusiedlersee sweet wines dry"]</t>
+        </is>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>Profile is included because WSET clearly supports Neusiedlersee/Burgenland sweet wine from Welschriesling and botrytis conditions.</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Austria - Practica 027</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN28" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AO28" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP28" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Austria is best known for quality dry white wines from Grüner Veltliner and Riesling.","Wachau, Kamptal, Kremstal, Weinviertel, Burgenland and Neusiedlersee are described in the Austria chapter."],"standard_wine_knowledge":["SAT appearance, intensity, alcohol, finish and diagnostic calibration use widely accepted Austrian white wine style norms."],"derived_from_style":["Difficulty, comparisons and learning traps are derived from WSET regional and varietal contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ28" t="inlineStr">
+        <is>
+          <t>{"appearance":["gold","deep gold possible","viscous tears possible"],"nose":["pronounced intensity","honey","apricot","citrus peel","dried fruit","botrytis spice"],"palate":["sweet","high acidity","medium to full body","low to medium alcohol","honeyed botrytised fruit"],"quality":["very good to outstanding when sweetness, acidity, botrytis complexity and length align"],"ageing":["high-quality examples can age for many years"],"diagnostic_features":["Neusiedlersee autumn mists","botrytis almost guaranteed every year","Welschriesling sweet wine","not the same grape as Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["botrytised Austrian sweet wine","lake-driven mesoclimate","Welschriesling distinction"],"learning_objectives":["separate Welschriesling from Riesling","connect Neusiedlersee mists to botrytis","identify sweet wine structure"],"typical_misconceptions":["Welschriesling is Riesling","Austria only makes dry whites","botrytis is always a fault"],"mentor_focus":["ask what environmental condition enables the style"],"exam_traps":["missing Neusiedlersee as key to sweet wines","confusing Burgenland sweet wine with German TBA"],"memory_hooks":["Neusiedlersee is Austria’s botrytis engine for sweet Welschriesling"],"comparison_styles":["Beerenauslese","Trockenbeerenauslese","Coteaux du Layon Chenin Blanc"]}</t>
+        </is>
+      </c>
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_019","SAT_WINE_020"],"frequently_confused_with":["SAT_WINE_020","SAT_WINE_010"],"distinguishing_features":["Austrian lake-mist botrytis context","Welschriesling not Riesling","Burgenland/Neusiedlersee source"]}</t>
+        </is>
+      </c>
+      <c r="AT28" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Burgenland is best known for top-quality sweet wines and red wines","Neusiedlersee is key for sweet wine production","Welschriesling is one of the most widely used grapes for these sweet wines"],"mentor_hints":["Ask whether the sweet wine is lake-botrytis driven.","Correct Welschriesling/Riesling confusion early."],"student_traps":["assuming Welschriesling is Riesling","forgetting botrytis can almost be guaranteed near Neusiedlersee"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>["neusiedlersee_botrytised_sweet_white","botrytised_sweet_wine"]</t>
+        </is>
+      </c>
+      <c r="AV28" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW28" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11001-11007","11173-11215"],"line_reference":["11001-11007","11173-11215"],"evidence":["Welschriesling is capable of producing high-quality dessert wines due to susceptibility to botrytis.","Neusiedlersee autumn mists and wetland margins create ideal botrytis conditions; Welschriesling is widely used for these sweet wines."]}</t>
+        </is>
+      </c>
+      <c r="AX28" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-04-BATCH-003","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY28" t="inlineStr">
+        <is>
+          <t>23 Austria</t>
+        </is>
+      </c>
+      <c r="AZ28" t="inlineStr">
+        <is>
+          <t>Burgenland / Neusiedlersee</t>
+        </is>
+      </c>
+      <c r="BA28" t="inlineStr">
+        <is>
+          <t>114-115</t>
+        </is>
+      </c>
+      <c r="BB28" t="inlineStr">
+        <is>
+          <t>["11001-11007","11173-11215"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add Batch 004 Italy white profiles
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -7626,6 +7626,2726 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SAT_WINE_028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Alto Adige Pinot Grigio</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Alpine dry Pinot Grigio with high acidity and citrus-green fruit</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Alto Adige Pinot Grigio</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Alto Adige</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Trentino-Alto Adige</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Alto Adige DOC</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>["Pinot Grigio"]</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>moderate alpine climate with short dry summers, low rainfall and large diurnal range at altitude</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>terraced south-east and south-west-facing valley sides of the River Adige</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>mountain terraces; WSET emphasizes altitude, aspect and diurnal range rather than a single soil type</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>["terraced vineyards on valley sides","altitude creates large diurnal range","conditions suit aromatic whites"]</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>["dry white winemaking","protective handling typical for Pinot Grigio","cool fermentation to preserve citrus and green fruit"]</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>typically unoaked; oak is not diagnostic</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>["citrus","green apple","pear","fresh herbs"]</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>["citrus","green fruit","crisp dry palate"]</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>good to very good; notable regional white style</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>drink young to short ageing for freshness</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium intensity","citrus","green apple","pear","fresh herbs","dry","high acidity","light to medium body","medium alcohol","citrus","green fruit","crisp dry palate"]</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>["Alto Adige is Italy's most northerly wine region","Pinot Grigio is the most notable white wine","large diurnal range supports aromatic whites"]</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>["Pinot Grigio is always simple","all Italian whites are warm-climate and low acid","green fruit means Sauvignon Blanc"]</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>["Ask whether the fruit profile is neutral-citrus rather than overtly aromatic.","Use altitude as the causal structure."]</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>["pale lemon","citrus","green apple","pear","fresh herbs","dry","high acidity","light to medium body","medium alcohol","citrus","green fruit","crisp dry palate","higher acidity than warmer valley-floor Trentino","lighter than Friuli Pinot Grigio","less floral than Gavi"]</t>
+        </is>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Trentino-Alto Adige - Alto Adige evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 028</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO29" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP29" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ29" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium intensity","citrus","green apple","pear","fresh herbs"],"palate":["dry","high acidity","light to medium body","medium alcohol","citrus","green fruit","crisp dry palate"],"quality":["good to very good; notable regional white style"],"ageing":["drink young to short ageing for freshness"],"diagnostic_features":["italian_pinot_grigio_core","cool_climate_high_acid_white","higher acidity than warmer valley-floor Trentino","lighter than Friuli Pinot Grigio"]}</t>
+        </is>
+      </c>
+      <c r="AR29" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Italian alpine white wines","Pinot Grigio freshness","altitude and diurnal range"],"learning_objectives":["identify dry high-acid Pinot Grigio","link Alto Adige to alpine freshness","avoid confusing neutral freshness with poor quality"],"typical_misconceptions":["Pinot Grigio is always simple","all Italian whites are warm-climate and low acid","green fruit means Sauvignon Blanc"],"mentor_focus":["anchor acidity, body and green fruit before naming grape"],"exam_traps":["calling it Sauvignon Blanc from green fruit alone","missing Alto Adige altitude"],"memory_hooks":["Alto Adige Pinot Grigio is mountain-fresh, dry and citrus-led"],"comparison_styles":["Trentino Pinot Grigio / Chardonnay","Friuli Pinot Grigio","Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AS29" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_029","SAT_WINE_030"],"frequently_confused_with":["SAT_WINE_009","SAT_WINE_031"],"distinguishing_features":["higher acidity than warmer valley-floor Trentino","lighter than Friuli Pinot Grigio","less floral than Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Alto Adige is Italy's most northerly wine region","Pinot Grigio is the most notable white wine","large diurnal range supports aromatic whites"],"mentor_hints":["Ask whether the fruit profile is neutral-citrus rather than overtly aromatic.","Use altitude as the causal structure."],"student_traps":["overcalling Sauvignon Blanc","forgetting Alto Adige DOC"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>["italian_pinot_grigio_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV29" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW29" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11695-11717"],"line_reference":["11695-11717"],"evidence":["Alto Adige is Italy's most northerly region with terraced valley-side vineyards and large diurnal range.","The most notable white wine is Pinot Grigio, dry, light to medium body, high acidity and citrus and green fruit flavours."]}</t>
+        </is>
+      </c>
+      <c r="AX29" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY29" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ29" t="inlineStr">
+        <is>
+          <t>Trentino-Alto Adige - Alto Adige</t>
+        </is>
+      </c>
+      <c r="BA29" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="BB29" t="inlineStr">
+        <is>
+          <t>["11695-11717"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SAT_WINE_029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Trentino Pinot Grigio / Chardonnay</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Moderate northern Italian valley white from Pinot Grigio or Chardonnay</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Trentino Pinot Grigio / Chardonnay</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Trentino</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Trentino-Alto Adige</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Trentino DOC</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>["Pinot Grigio","Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>dry summers and low rainfall; slightly warmer than Alto Adige due to southerly latitude and lower-altitude vineyards</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>valley floor and slopes on both sides of a wider valley</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>varied valley and slope sites; WSET emphasizes altitude and valley position</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>["vines on valley floor and slopes","lower altitude sites give riper fruit","higher altitude sites resemble Alto Adige whites"]</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>["fresh dry white production","cool fermentation common for fruit expression","usually stainless steel"]</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>usually unoaked or neutral; oak is not central to the style</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>["ripe stone fruit","citrus","pear"]</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>["ripe stone fruit","citrus","fresh dry palate"]</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>good to very good; regional DOC style</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>drink young to short ageing</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium intensity","ripe stone fruit","citrus","pear","dry","medium acidity","medium body","medium alcohol","ripe stone fruit","citrus","fresh dry palate"]</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>["Trentino is directly south of Alto Adige","main varieties are Chardonnay and Pinot Grigio","valley-floor wines tend to be medium-bodied with medium acidity and ripe stone fruit"]</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>["all Trentino whites are alpine and high acid","Chardonnay always shows oak","Pinot Grigio cannot show stone fruit"]</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>["Ask where the fruit sits on the green-to-stone-fruit spectrum.","Use valley position to explain structure."]</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","ripe stone fruit","citrus","pear","dry","medium acidity","medium body","medium alcohol","ripe stone fruit","citrus","fresh dry palate","riper and broader than Alto Adige","less tropical and full than Friuli","less Garganega pear and almond than Soave"]</t>
+        </is>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI30" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Trentino evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 029</t>
+        </is>
+      </c>
+      <c r="AK30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL30" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO30" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="AP30" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ30" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium intensity","ripe stone fruit","citrus","pear"],"palate":["dry","medium acidity","medium body","medium alcohol","ripe stone fruit","citrus","fresh dry palate"],"quality":["good to very good; regional DOC style"],"ageing":["drink young to short ageing"],"diagnostic_features":["italian_pinot_grigio_core","white_wine_sat_core","riper and broader than Alto Adige","less tropical and full than Friuli"]}</t>
+        </is>
+      </c>
+      <c r="AR30" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["site altitude gradient","northern Italian fresh whites","Pinot Grigio and Chardonnay overlap"],"learning_objectives":["separate Trentino valley fruit from Alto Adige freshness","recognize medium-bodied northern Italian white","avoid assuming all Pinot Grigio is high acid"],"typical_misconceptions":["all Trentino whites are alpine and high acid","Chardonnay always shows oak","Pinot Grigio cannot show stone fruit"],"mentor_focus":["ask whether acidity is medium rather than high and fruit is riper"],"exam_traps":["overcalling Alto Adige","forcing oak because Chardonnay is possible"],"memory_hooks":["Trentino sits one step warmer and riper than Alto Adige"],"comparison_styles":["Alto Adige Pinot Grigio","Friuli Pinot Grigio","Soave Classico"]}</t>
+        </is>
+      </c>
+      <c r="AS30" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_028","SAT_WINE_030"],"frequently_confused_with":["SAT_WINE_028","SAT_WINE_003"],"distinguishing_features":["riper and broader than Alto Adige","less tropical and full than Friuli","less Garganega pear and almond than Soave"]}</t>
+        </is>
+      </c>
+      <c r="AT30" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Trentino is directly south of Alto Adige","main varieties are Chardonnay and Pinot Grigio","valley-floor wines tend to be medium-bodied with medium acidity and ripe stone fruit"],"mentor_hints":["Ask where the fruit sits on the green-to-stone-fruit spectrum.","Use valley position to explain structure."],"student_traps":["treating Trentino as identical to Alto Adige","assuming Chardonnay means obvious oak"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t>["italian_pinot_grigio_core","white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV30" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW30" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11763-11800"],"line_reference":["11763-11800"],"evidence":["Trentino is slightly warmer than Alto Adige and has vines on valley floor and slopes.","Main varieties are Chardonnay and Pinot Grigio; valley-floor whites are medium-bodied with medium acidity and ripe stone fruit."]}</t>
+        </is>
+      </c>
+      <c r="AX30" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY30" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ30" t="inlineStr">
+        <is>
+          <t>Trentino</t>
+        </is>
+      </c>
+      <c r="BA30" t="inlineStr">
+        <is>
+          <t>121-122</t>
+        </is>
+      </c>
+      <c r="BB30" t="inlineStr">
+        <is>
+          <t>["11763-11800"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SAT_WINE_030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Friuli Pinot Grigio</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Rich north-east Italian Pinot Grigio from Friuli-Venezia Giulia</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Friuli Pinot Grigio</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Friuli-Venezia Giulia</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Friuli / Collio / Colli Orientali</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Friuli Grave DOC / Collio DOC / Colli Orientali DOC</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>["Pinot Grigio"]</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>moderate continental foothills in the north and warm maritime plain near the Adriatic in the south</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>foothill sites in Collio and Colli Orientali for premium concentration; plains for simpler styles</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>varied foothill and plain soils; WSET emphasizes hills versus plain</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>["large number of grape varieties planted","hills produce premium concentrated whites","plain fruit can produce simple fruity whites"]</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>["dry white winemaking","protective fermentation for fruit","premium examples may use texture-building handling"]</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>usually unoaked or neutral; oak is not the main diagnostic marker</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>["juicy peach","tropical fruit","pear","red apple"]</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>["juicy peach","tropical fruit","ripe orchard fruit","rounded dry palate"]</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>good to very good; premium hill examples can be concentrated</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>drink young to medium ageing for best concentrated whites</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium intensity","juicy peach","tropical fruit","pear","red apple","dry","medium to high acidity","medium to full body","medium to high alcohol","juicy peach","tropical fruit","ripe orchard fruit","rounded dry palate"]</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>["Pinot Grigio is prevalent in Friuli-Venezia Giulia","Friuli produces some of Italy's richest Pinot Grigio","Collio and Colli Orientali are known for premium concentrated whites"]</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>["Pinot Grigio is always light","tropical fruit means New World","Friuli is only simple Friuli Grave"]</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>["Probe body and fruit ripeness before naming Pinot Grigio.","Use the hills/plain split to explain quality."]</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","juicy peach","tropical fruit","pear","red apple","dry","medium to high acidity","medium to full body","medium to high alcohol","juicy peach","tropical fruit","ripe orchard fruit","rounded dry palate","more body and tropical fruit than Alto Adige","less floral-high-acid than Gavi","less pear-almond Garganega than Soave"]</t>
+        </is>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Friuli-Venezia Giulia evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 030</t>
+        </is>
+      </c>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP31" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ31" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium intensity","juicy peach","tropical fruit","pear","red apple"],"palate":["dry","medium to high acidity","medium to full body","medium to high alcohol","juicy peach","tropical fruit","ripe orchard fruit"],"quality":["good to very good; premium hill examples can be concentrated"],"ageing":["drink young to medium ageing for best concentrated whites"],"diagnostic_features":["friuli_rich_white_core","italian_pinot_grigio_core","more body and tropical fruit than Alto Adige","less floral-high-acid than Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AR31" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Friuli richness","Pinot Grigio style range","hill versus plain quality"],"learning_objectives":["recognize richer Pinot Grigio","contrast Friuli with Alto Adige","connect Collio and Colli Orientali to premium whites"],"typical_misconceptions":["Pinot Grigio is always light","tropical fruit means New World","Friuli is only simple Friuli Grave"],"mentor_focus":["ask whether body and fruit ripeness exceed alpine Pinot Grigio"],"exam_traps":["calling rich Pinot Grigio Chardonnay","missing Collio/Colli Orientali premium context"],"memory_hooks":["Friuli is the richer Pinot Grigio lane in Italy"],"comparison_styles":["Alto Adige Pinot Grigio","Trentino Pinot Grigio / Chardonnay","Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AS31" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_029","SAT_WINE_028"],"frequently_confused_with":["SAT_WINE_003","SAT_WINE_031"],"distinguishing_features":["more body and tropical fruit than Alto Adige","less floral-high-acid than Gavi","less pear-almond Garganega than Soave"]}</t>
+        </is>
+      </c>
+      <c r="AT31" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Pinot Grigio is prevalent in Friuli-Venezia Giulia","Friuli produces some of Italy's richest Pinot Grigio","Collio and Colli Orientali are known for premium concentrated whites"],"mentor_hints":["Probe body and fruit ripeness before naming Pinot Grigio.","Use the hills/plain split to explain quality."],"student_traps":["assuming Pinot Grigio must be neutral","confusing richness with oak"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU31" t="inlineStr">
+        <is>
+          <t>["friuli_rich_white_core","italian_pinot_grigio_core"]</t>
+        </is>
+      </c>
+      <c r="AV31" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW31" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11802-11826"],"line_reference":["11802-11826"],"evidence":["Friuli-Venezia Giulia produces some of the richest Pinot Grigio in Italy.","The medium- to full-bodied wines display juicy peach and tropical fruit flavours; Collio and Colli Orientali are premium concentrated white wine areas."]}</t>
+        </is>
+      </c>
+      <c r="AX31" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY31" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ31" t="inlineStr">
+        <is>
+          <t>Friuli-Venezia Giulia</t>
+        </is>
+      </c>
+      <c r="BA31" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="BB31" t="inlineStr">
+        <is>
+          <t>["11802-11826"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SAT_WINE_031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Soave Classico</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Foothill Garganega white from limestone, clay and volcanic soils</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Soave Classico</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Veneto</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Soave foothills</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Soave Classico DOC</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>["Garganega"]</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>warm Veneto climate moderated by altitude in the foothills and large diurnal range</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>foothills north of Soave on cooler elevated sites</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>limestone and clay with some volcanic rocks; cool soils slow ripening</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>["foothill fruit has full flavour ripeness and high acidity","plain fruit is fruitier with medium acidity","Classico indicates foothill source"]</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>["dry white production","small amounts of other white grapes may be blended","no new oak aromas or flavours typical"]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>no new oak aromas or flavours typical</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>["pear","red apple","stone fruit","white pepper","almond with age"]</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>["pear","red apple","stone fruit","subtle white pepper","almond and honey with age"]</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>good to very good; best examples can age</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>medium ageing for best Classico examples</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium intensity","pear","red apple","stone fruit","white pepper","almond with age","dry","medium to high acidity","medium body","medium alcohol","pear","red apple","stone fruit","subtle white pepper","almond and honey with age"]</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>["Soave is east of Verona","Garganega is the main variety","Soave Classico comes from foothills and best examples can age"]</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>["white pepper always means Grüner Veltliner","Soave is always simple","Italian whites all lack ageing potential"]</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>["Ask if the spice note is white pepper without oak support.","Tie Classico to foothill soils and acidity."]</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","pear","red apple","stone fruit","white pepper","almond with age","dry","medium to high acidity","medium body","medium alcohol","pear","red apple","stone fruit","subtle white pepper","almond and honey with age","more pear and almond than Pinot Grigio","less floral and lighter than Gavi","less fennel-lemon than Verdicchio"]</t>
+        </is>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Veneto - Soave evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 031</t>
+        </is>
+      </c>
+      <c r="AK32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL32" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO32" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP32" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ32" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium intensity","pear","red apple","stone fruit","white pepper","almond with age"],"palate":["dry","medium to high acidity","medium body","medium alcohol","pear","red apple","stone fruit"],"quality":["good to very good; best examples can age"],"ageing":["medium ageing for best Classico examples"],"diagnostic_features":["soave_garganega_core","central_italy_fresh_white_core","more pear and almond than Pinot Grigio","less floral and lighter than Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AR32" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Garganega identity","Classico foothill quality","no-new-oak Italian white"],"learning_objectives":["identify Soave structural markers","distinguish Classico foothills from plain Soave","separate white pepper from oak"],"typical_misconceptions":["white pepper always means Grüner Veltliner","Soave is always simple","Italian whites all lack ageing potential"],"mentor_focus":["ask for pear, apple, medium body and no new oak"],"exam_traps":["calling it Pinot Grigio from neutrality","missing Classico foothill quality"],"memory_hooks":["Soave Classico is Garganega: pear, apple, stone fruit, no new oak"],"comparison_styles":["Friuli Pinot Grigio","Gavi","Verdicchio dei Castelli di Jesi"]}</t>
+        </is>
+      </c>
+      <c r="AS32" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_030","SAT_WINE_035"],"frequently_confused_with":["SAT_WINE_030","SAT_WINE_032"],"distinguishing_features":["more pear and almond than Pinot Grigio","less floral and lighter than Gavi","less fennel-lemon than Verdicchio"]}</t>
+        </is>
+      </c>
+      <c r="AT32" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Soave is east of Verona","Garganega is the main variety","Soave Classico comes from foothills and best examples can age"],"mentor_hints":["Ask if the spice note is white pepper without oak support.","Tie Classico to foothill soils and acidity."],"student_traps":["assuming Soave means low quality","adding new oak to the tasting note"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>["soave_garganega_core","central_italy_fresh_white_core"]</t>
+        </is>
+      </c>
+      <c r="AV32" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW32" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11857-11882"],"line_reference":["11857-11882"],"evidence":["Soave foothills have limestone, clay and volcanic rocks that slow ripening, leading to full flavour ripeness and high acidity.","Garganega wines have medium to high acidity, medium body, pears, red apple, stone fruit and sometimes white pepper, without new oak; best examples age with almond and honey."]}</t>
+        </is>
+      </c>
+      <c r="AX32" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY32" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ32" t="inlineStr">
+        <is>
+          <t>Veneto - Soave</t>
+        </is>
+      </c>
+      <c r="BA32" t="inlineStr">
+        <is>
+          <t>122-123</t>
+        </is>
+      </c>
+      <c r="BB32" t="inlineStr">
+        <is>
+          <t>["11857-11882"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SAT_WINE_032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Gavi</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pale high-acid Cortese white from south-eastern Piemonte</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Gavi</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Piemonte</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>South-eastern Piemonte</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Gavi DOCG / Cortese di Gavi DOCG</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>["Cortese"]</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>moderate continental Piemonte with altitude and sea breezes in Gavi hills</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>hills where altitude supports long slow ripening</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>hillside sites; WSET emphasizes altitude and sea breezes rather than named soil</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>["altitude and sea breezes lengthen ripening","Cortese keeps natural high acidity","Gavi di Gavi can indicate grapes from the town of Gavi"]</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>["protective winemaking is the norm","cool fermentation in stainless steel","some producers use techniques for added texture"]</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>typically stainless steel; oak not diagnostic</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>["floral notes","citrus","green apple","pear"]</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>["citrus","green apple","pear","floral lift"]</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>drink young to short ageing; freshness is central</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium intensity","floral notes","citrus","green apple","pear","dry","high acidity","light body","medium alcohol","citrus","green apple","pear","floral lift"]</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>["Gavi is in south-eastern Piemonte","Cortese has natural high acidity and floral character","Gavi may be labelled Gavi DOCG or Cortese di Gavi DOCG"]</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>["Piemonte is only red wines","floral white must be aromatic Alsace","all Italian white DOCGs are full-bodied"]</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>["Ask if the profile is floral and light rather than neutral.","Use Cortese acidity as the anchor."]</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>["pale lemon","floral notes","citrus","green apple","pear","dry","high acidity","light body","medium alcohol","citrus","green apple","pear","floral lift","more floral and lighter than Soave","less fennel and almond than Verdicchio","less ripe than Friuli Pinot Grigio"]</t>
+        </is>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI33" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Piemonte - Gavi evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 032</t>
+        </is>
+      </c>
+      <c r="AK33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL33" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN33" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO33" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP33" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ33" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium intensity","floral notes","citrus","green apple","pear"],"palate":["dry","high acidity","light body","medium alcohol","citrus","green apple","pear"],"quality":["good to very good"],"ageing":["drink young to short ageing; freshness is central"],"diagnostic_features":["gavi_cortese_core","cool_climate_high_acid_white","more floral and lighter than Soave","less fennel and almond than Verdicchio"]}</t>
+        </is>
+      </c>
+      <c r="AR33" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Cortese high acidity","Piemonte white identity","protective winemaking"],"learning_objectives":["identify pale high-acid Gavi","separate Cortese from Pinot Grigio","link altitude and sea breezes to freshness"],"typical_misconceptions":["Piemonte is only red wines","floral white must be aromatic Alsace","all Italian white DOCGs are full-bodied"],"mentor_focus":["ask for pale colour, light body and high acidity together"],"exam_traps":["calling Gavi Pinot Grigio","missing DOCG/Cortese link"],"memory_hooks":["Gavi is Cortese: pale, light, floral, high-acid"],"comparison_styles":["Alto Adige Pinot Grigio","Soave Classico","Verdicchio dei Castelli di Jesi"]}</t>
+        </is>
+      </c>
+      <c r="AS33" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_028","SAT_WINE_035"],"frequently_confused_with":["SAT_WINE_031","SAT_WINE_033"],"distinguishing_features":["more floral and lighter than Soave","less fennel and almond than Verdicchio","less ripe than Friuli Pinot Grigio"]}</t>
+        </is>
+      </c>
+      <c r="AT33" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Gavi is in south-eastern Piemonte","Cortese has natural high acidity and floral character","Gavi may be labelled Gavi DOCG or Cortese di Gavi DOCG"],"mentor_hints":["Ask if the profile is floral and light rather than neutral.","Use Cortese acidity as the anchor."],"student_traps":["forgetting Piemonte whites","mistaking floral notes for Muscat"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU33" t="inlineStr">
+        <is>
+          <t>["gavi_cortese_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV33" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW33" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12114-12125"],"line_reference":["12114-12125"],"evidence":["Gavi vines grow in hills where altitude and sea breezes result in long slow ripening of Cortese, emphasizing high acidity and floral character.","Wines are pale and light-bodied, with high acidity and citrus, green apples and pears; protective winemaking and cool stainless steel are normal."]}</t>
+        </is>
+      </c>
+      <c r="AX33" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY33" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ33" t="inlineStr">
+        <is>
+          <t>Piemonte - Gavi</t>
+        </is>
+      </c>
+      <c r="BA33" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="BB33" t="inlineStr">
+        <is>
+          <t>["12114-12125"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SAT_WINE_033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Orvieto</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Fresh Umbrian white blend of Grechetto and Trebbiano</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Orvieto</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Umbria</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Orvieto</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Orvieto DOC</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>["Grechetto","Trebbiano"]</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>continental central Italian climate similar to Tuscany but without Mediterranean influence</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>hills around Orvieto; WSET emphasizes continental inland conditions</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>not specified by WSET for this style; regional inland conditions are the key marker</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>["blend led by Grechetto and Trebbiano","best examples tend to have more Grechetto","central inland freshness retained"]</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>["protective winemaking","cool fermentation in stainless steel","fresh fruit-led style"]</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>unoaked; stainless steel freshness is diagnostic</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>["ripe grapefruit","peach","citrus"]</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>["ripe grapefruit","peach","fresh citrus","clean dry finish"]</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>good; best examples with more Grechetto can be very good</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>drink young</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium intensity","ripe grapefruit","peach","citrus","dry","medium to high acidity","light body","medium alcohol","ripe grapefruit","peach","fresh citrus","clean dry finish"]</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>["Orvieto DOC is a blend of Grechetto and Trebbiano","best examples tend to have more Grechetto","cool stainless steel fermentation is used"]</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>["central Italy is only red wine","Trebbiano blends are always poor","all Italian whites are Pinot Grigio"]</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>["Ask if the blend evidence points to Grechetto/Trebbiano.","Compare with Frascati using Malvasia orange blossom."]</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>["pale lemon","ripe grapefruit","peach","citrus","dry","medium to high acidity","light body","medium alcohol","ripe grapefruit","peach","fresh citrus","clean dry finish","riper grapefruit and peach than Frascati","less floral than Malvasia-led Frascati","less high-acid and floral than Gavi"]</t>
+        </is>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Umbria - Orvieto evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 033</t>
+        </is>
+      </c>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO34" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="AP34" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ34" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium intensity","ripe grapefruit","peach","citrus"],"palate":["dry","medium to high acidity","light body","medium alcohol","ripe grapefruit","peach","fresh citrus"],"quality":["good; best examples with more Grechetto can be very good"],"ageing":["drink young"],"diagnostic_features":["central_italy_fresh_white_core","white_wine_sat_core","riper grapefruit and peach than Frascati","less floral than Malvasia-led Frascati"]}</t>
+        </is>
+      </c>
+      <c r="AR34" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["central Italian white blends","protective winemaking","Grechetto quality role"],"learning_objectives":["recognize Orvieto as a fresh blend","connect Grechetto proportion to quality","separate Orvieto from Frascati"],"typical_misconceptions":["central Italy is only red wine","Trebbiano blends are always poor","all Italian whites are Pinot Grigio"],"mentor_focus":["ask whether fruit is grapefruit-peach rather than floral-orange"],"exam_traps":["confusing Orvieto with Frascati","omitting Grechetto"],"memory_hooks":["Orvieto is Umbria freshness: Grechetto, Trebbiano, grapefruit and peach"],"comparison_styles":["Frascati","Gavi","Soave Classico"]}</t>
+        </is>
+      </c>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_034"],"frequently_confused_with":["SAT_WINE_034","SAT_WINE_032"],"distinguishing_features":["riper grapefruit and peach than Frascati","less floral than Malvasia-led Frascati","less high-acid and floral than Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AT34" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Orvieto DOC is a blend of Grechetto and Trebbiano","best examples tend to have more Grechetto","cool stainless steel fermentation is used"],"mentor_hints":["Ask if the blend evidence points to Grechetto/Trebbiano.","Compare with Frascati using Malvasia orange blossom."],"student_traps":["using Trebbiano as a synonym for low quality","missing Umbria"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>["central_italy_fresh_white_core","white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV34" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW34" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12333-12343"],"line_reference":["12333-12343"],"evidence":["Umbria is continental and known for Orvieto DOC, a blend of Grechetto, Trebbiano and often other local grapes.","Orvieto is light-bodied with medium to high acidity and ripe grapefruit and peach; made protectively with cool stainless steel fermentation."]}</t>
+        </is>
+      </c>
+      <c r="AX34" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY34" t="inlineStr">
+        <is>
+          <t>28 Central Italy</t>
+        </is>
+      </c>
+      <c r="AZ34" t="inlineStr">
+        <is>
+          <t>Umbria - Orvieto</t>
+        </is>
+      </c>
+      <c r="BA34" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="BB34" t="inlineStr">
+        <is>
+          <t>["12333-12343"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SAT_WINE_034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Frascati</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Fresh Lazio white blend of Malvasia and Trebbiano</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Frascati</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Hills south of Rome</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Frascati DOC</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>["Malvasia","Trebbiano"]</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>hills south of Rome cooled by altitude and nearby small lakes</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>hills south of Rome with altitude cooling</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>not specified by WSET; lake and altitude cooling are the key markers</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>["white grapes benefit from altitude and lake cooling","Malvasia and Trebbiano are blended","freshness is protected"]</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>["fresh unoaked style","protective white winemaking","cool fermentation typical for fresh fruit"]</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>unoaked</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>["citrus fruit","orange blossom","floral notes"]</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>["citrus","fresh dry palate","floral orange blossom nuance"]</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>drink young</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium intensity","citrus fruit","orange blossom","floral notes","dry","medium to high acidity","medium body","medium alcohol","citrus","fresh dry palate","floral orange blossom nuance"]</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>["Frascati DOC is the best-known Lazio wine","vineyards are cooled by altitude and nearby lakes","Malvasia and Trebbiano are usually made fresh and unoaked"]</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>["Frascati is always neutral","Lazio is irrelevant for WSET whites","floral notes always mean Gewurztraminer"]</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>["Use orange blossom as the Malvasia clue.","Ask whether the structure is fresh but medium-bodied."]</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>["pale lemon","citrus fruit","orange blossom","floral notes","dry","medium to high acidity","medium body","medium alcohol","citrus","fresh dry palate","floral orange blossom nuance","more floral orange blossom than Orvieto","medium body rather than Gavi light body","less pear-almond than Soave"]</t>
+        </is>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Lazio - Frascati evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 034</t>
+        </is>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL35" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO35" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="AP35" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ35" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium intensity","citrus fruit","orange blossom","floral notes"],"palate":["dry","medium to high acidity","medium body","medium alcohol","citrus","fresh dry palate","floral orange blossom nuance"],"quality":["good"],"ageing":["drink young"],"diagnostic_features":["central_italy_fresh_white_core","white_wine_sat_core","more floral orange blossom than Orvieto","medium body rather than Gavi light body"]}</t>
+        </is>
+      </c>
+      <c r="AR35" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Lazio fresh whites","Malvasia floral contribution","altitude and lake cooling"],"learning_objectives":["identify Frascati structure","separate Frascati from Orvieto","recognize Malvasia orange blossom"],"typical_misconceptions":["Frascati is always neutral","Lazio is irrelevant for WSET whites","floral notes always mean Gewurztraminer"],"mentor_focus":["ask for citrus plus orange blossom in an unoaked frame"],"exam_traps":["calling it Orvieto from Trebbiano alone","missing lake and altitude cooling"],"memory_hooks":["Frascati is Rome-hills freshness with Malvasia orange blossom"],"comparison_styles":["Orvieto","Gavi","Soave Classico"]}</t>
+        </is>
+      </c>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_033"],"frequently_confused_with":["SAT_WINE_033","SAT_WINE_032"],"distinguishing_features":["more floral orange blossom than Orvieto","medium body rather than Gavi light body","less pear-almond than Soave"]}</t>
+        </is>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Frascati DOC is the best-known Lazio wine","vineyards are cooled by altitude and nearby lakes","Malvasia and Trebbiano are usually made fresh and unoaked"],"mentor_hints":["Use orange blossom as the Malvasia clue.","Ask whether the structure is fresh but medium-bodied."],"student_traps":["forgetting Lazio in white wine study","overcalling aromatic intensity"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>["central_italy_fresh_white_core","white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV35" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW35" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12350-12359"],"line_reference":["12350-12359"],"evidence":["Frascati DOC is in hills south of Rome cooled by altitude and nearby lakes.","It is a blend of Malvasia and Trebbiano, fresh and unoaked, medium body, medium to high acidity, citrus and sometimes orange blossom."]}</t>
+        </is>
+      </c>
+      <c r="AX35" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY35" t="inlineStr">
+        <is>
+          <t>28 Central Italy</t>
+        </is>
+      </c>
+      <c r="AZ35" t="inlineStr">
+        <is>
+          <t>Lazio - Frascati</t>
+        </is>
+      </c>
+      <c r="BA35" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="BB35" t="inlineStr">
+        <is>
+          <t>["12350-12359"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SAT_WINE_035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Verdicchio dei Castelli di Jesi</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>High-acid Marche Verdicchio with lemon, fennel and almond</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Verdicchio dei Castelli di Jesi</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Marche</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Castelli di Jesi</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Verdicchio dei Castelli di Jesi DOC</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>["Verdicchio"]</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>eastern side of the Apennines with central Italian conditions; WSET emphasizes regional grape style</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>hilly central Italian sites around Castelli di Jesi</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>not specified by WSET for this style</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>["Verdicchio is the key grape","many wines are simple and fruity","best examples have concentration and can age"]</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>["fresh dry white production","protective handling for fruit","best examples may be made for bottle development"]</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>not diagnostic; almond and honey can come with bottle age</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>["green apple","lemon","fennel","almond","honey with age"]</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>["green apple","lemon","fennel","almond","honeyed notes with age"]</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>good to very good; best examples can develop complexity</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>short to medium ageing; best examples develop honey and almond</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium intensity","green apple","lemon","fennel","almond","honey with age","dry","high acidity","medium body","medium alcohol","green apple","lemon","fennel","almond","honeyed notes with age"]</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>["Marche is best known for Verdicchio whites","Verdicchio dei Castelli di Jesi is the most famous","best examples age with honey and almond"]</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>["almond always means oak","Verdicchio is only simple","central Italy is red-only"]</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>["Ask whether almond appears with freshness rather than oak.","Use fennel as the diagnostic anchor."]</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","green apple","lemon","fennel","almond","honey with age","dry","high acidity","medium body","medium alcohol","green apple","lemon","fennel","almond","honeyed notes with age","fennel and lemon more diagnostic than Soave pear","more almond-fennel than Gavi floral pear","higher acidity than Orvieto"]</t>
+        </is>
+      </c>
+      <c r="AH36" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI36" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Marche - Verdicchio evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ36" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 035</t>
+        </is>
+      </c>
+      <c r="AK36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL36" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO36" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP36" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ36" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium intensity","green apple","lemon","fennel","almond","honey with age"],"palate":["dry","high acidity","medium body","medium alcohol","green apple","lemon","fennel"],"quality":["good to very good; best examples can develop complexity"],"ageing":["short to medium ageing; best examples develop honey and almond"],"diagnostic_features":["verdicchio_core","central_italy_fresh_white_core","fennel and lemon more diagnostic than Soave pear","more almond-fennel than Gavi floral pear"]}</t>
+        </is>
+      </c>
+      <c r="AR36" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Verdicchio varietal identity","Italian white ageing beyond oak","Marche regional marker"],"learning_objectives":["identify fennel-almond Verdicchio","separate almond age notes from oak","connect Marche to Verdicchio"],"typical_misconceptions":["almond always means oak","Verdicchio is only simple","central Italy is red-only"],"mentor_focus":["ask for lemon, fennel and almond together"],"exam_traps":["calling it Soave from almond alone","missing high acidity"],"memory_hooks":["Verdicchio is lemon, fennel, almond and high acidity"],"comparison_styles":["Soave Classico","Gavi","Orvieto"]}</t>
+        </is>
+      </c>
+      <c r="AS36" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_031","SAT_WINE_032"],"frequently_confused_with":["SAT_WINE_031","SAT_WINE_033"],"distinguishing_features":["fennel and lemon more diagnostic than Soave pear","more almond-fennel than Gavi floral pear","higher acidity than Orvieto"]}</t>
+        </is>
+      </c>
+      <c r="AT36" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Marche is best known for Verdicchio whites","Verdicchio dei Castelli di Jesi is the most famous","best examples age with honey and almond"],"mentor_hints":["Ask whether almond appears with freshness rather than oak.","Use fennel as the diagnostic anchor."],"student_traps":["missing Verdicchio because it seems neutral","confusing almond with new oak"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU36" t="inlineStr">
+        <is>
+          <t>["verdicchio_core","central_italy_fresh_white_core"]</t>
+        </is>
+      </c>
+      <c r="AV36" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW36" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12361-12375"],"line_reference":["12361-12375"],"evidence":["Marche is best known for white wines made from Verdicchio, especially Verdicchio dei Castelli di Jesi DOC.","Verdicchio is high in acidity with green apples, lemons, fennel and almond; best examples develop honey and almonds with age."]}</t>
+        </is>
+      </c>
+      <c r="AX36" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY36" t="inlineStr">
+        <is>
+          <t>28 Central Italy</t>
+        </is>
+      </c>
+      <c r="AZ36" t="inlineStr">
+        <is>
+          <t>Marche - Verdicchio</t>
+        </is>
+      </c>
+      <c r="BA36" t="inlineStr">
+        <is>
+          <t>127-128</t>
+        </is>
+      </c>
+      <c r="BB36" t="inlineStr">
+        <is>
+          <t>["12361-12375"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SAT_WINE_036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Fiano di Avellino</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Medium- to full-bodied Campanian Fiano with stone fruit and ageworthy wax-honey complexity</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Fiano di Avellino</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Campania</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Avellino</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Fiano di Avellino DOCG</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>["Fiano"]</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>southern Italian region with varied mountains, valleys and coastal plains enabling quality whites</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>inland Campanian appellation with elevation influence implied by regional mountains and valleys</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>not specified by WSET for Fiano di Avellino in this passage</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>["Fiano produces some of Campania's best whites","better examples can be selected for ageing","grown in Campania and other southern regions"]</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>["often made to drink young","better examples may be matured in oak","can age in bottle"]</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>often none for youthful examples; better examples may be matured in oak</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>medium lemon</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>["stone fruit","melon","mango","wax with age","honey with age"]</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>["stone fruit","melon","mango","rounded dry palate","wax and honey with age"]</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>very good to outstanding in best DOCG examples</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>medium to long ageing for better examples</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>["medium lemon","medium intensity","stone fruit","melon","mango","wax with age","honey with age","dry","medium acidity","medium to full body","medium to high alcohol","stone fruit","melon","mango","rounded dry palate","wax and honey with age"]</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>["Fiano di Avellino DOCG is a key Campanian white","Fiano has medium acidity and medium to full body","better examples can age with wax and honey"]</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>["southern Italy only makes reds","medium acidity means low quality","oak-aged white must be Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>["Ask whether acidity is medium and body is fuller than Greco.","Use wax and honey as development markers."]</t>
+        </is>
+      </c>
+      <c r="AG37" t="inlineStr">
+        <is>
+          <t>["medium lemon","stone fruit","melon","mango","wax with age","honey with age","dry","medium acidity","medium to full body","medium to high alcohol","stone fruit","melon","mango","rounded dry palate","wax and honey with age","fuller and lower acid than Greco","more mango-melon than Friuli Pinot Grigio","more wax-honey than Soave"]</t>
+        </is>
+      </c>
+      <c r="AH37" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI37" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Campania - Fiano and Greco evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 036</t>
+        </is>
+      </c>
+      <c r="AK37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL37" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN37" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO37" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP37" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ37" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium lemon"],"nose":["medium intensity","stone fruit","melon","mango","wax with age","honey with age"],"palate":["dry","medium acidity","medium to full body","medium to high alcohol","stone fruit","melon","mango"],"quality":["very good to outstanding in best DOCG examples"],"ageing":["medium to long ageing for better examples"],"diagnostic_features":["campania_fiano_greco_core","white_wine_sat_core","fuller and lower acid than Greco","more mango-melon than Friuli Pinot Grigio"]}</t>
+        </is>
+      </c>
+      <c r="AR37" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Campanian premium whites","Fiano texture and fruit","ageworthy southern white"],"learning_objectives":["identify Fiano body and fruit profile","distinguish Fiano from Greco","connect wax-honey development to ageing"],"typical_misconceptions":["southern Italy only makes reds","medium acidity means low quality","oak-aged white must be Chardonnay"],"mentor_focus":["ask whether body and tropical-stone fruit point to Fiano"],"exam_traps":["confusing Fiano with Greco","calling oak-matured Fiano Chardonnay"],"memory_hooks":["Fiano is Campania's rounder wax-and-honey white"],"comparison_styles":["Greco di Tufo","Friuli Pinot Grigio","Soave Classico"]}</t>
+        </is>
+      </c>
+      <c r="AS37" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_037"],"frequently_confused_with":["SAT_WINE_037","SAT_WINE_030"],"distinguishing_features":["fuller and lower acid than Greco","more mango-melon than Friuli Pinot Grigio","more wax-honey than Soave"]}</t>
+        </is>
+      </c>
+      <c r="AT37" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Fiano di Avellino DOCG is a key Campanian white","Fiano has medium acidity and medium to full body","better examples can age with wax and honey"],"mentor_hints":["Ask whether acidity is medium and body is fuller than Greco.","Use wax and honey as development markers."],"student_traps":["forgetting southern Italian whites","mistaking texture for Chardonnay"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU37" t="inlineStr">
+        <is>
+          <t>["campania_fiano_greco_core","white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV37" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW37" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12431-12449"],"line_reference":["12431-12449"],"evidence":["Fiano and Greco arguably produce the best white wines in Campania; many best examples come from Fiano di Avellino DOCG and Greco di Tufo DOCG.","Fiano has medium acidity, medium to full body, stone fruit, melons and mango; better examples are matured in oak and age with wax and honey."]}</t>
+        </is>
+      </c>
+      <c r="AX37" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY37" t="inlineStr">
+        <is>
+          <t>29 Southern Italy</t>
+        </is>
+      </c>
+      <c r="AZ37" t="inlineStr">
+        <is>
+          <t>Campania - Fiano and Greco</t>
+        </is>
+      </c>
+      <c r="BA37" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="BB37" t="inlineStr">
+        <is>
+          <t>["12431-12449"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SAT_WINE_037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Blancos Italia</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Greco di Tufo</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Lean high-acid Campanian Greco with green apple, stone fruit and passion fruit</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Greco di Tufo</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Campania</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Tufo</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Greco di Tufo DOCG</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>["Greco"]</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>southern Italian region with varied mountains, valleys and coastal plains enabling quality whites</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>inland Campanian appellation with elevation influence implied by regional mountains and valleys</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>not specified by WSET for Greco di Tufo in this passage</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>["Greco produces some of Campania's best whites","best examples come from Greco di Tufo DOCG","acidity is a key structural marker"]</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>["most producers ferment in stainless steel","some use old oak","lees stirring may enhance texture"]</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>stainless steel common; some old oak may be used, not new-oak dominated</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>medium lemon</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>["green apple","stone fruit","passion fruit","honey with age","mushroom with age"]</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>["green apple","stone fruit","passion fruit","lean high-acid palate","honey and mushroom with age"]</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>very good to outstanding in best DOCG examples</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>medium ageing; best examples develop honey and mushroom</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>["medium lemon","medium intensity","green apple","stone fruit","passion fruit","honey with age","mushroom with age","dry","high acidity","medium body","medium to high alcohol","green apple","stone fruit","passion fruit","lean high-acid palate","honey and mushroom with age"]</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>["Greco di Tufo DOCG is a key Campanian white","Greco has more acidity and leaner body than Fiano","best examples can age with honey and mushroom notes"]</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>["southern whites are always low acid","Greco and Fiano are interchangeable","mushroom age notes mean fault"]</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>["Compare directly with Fiano before final identification.","Ask whether passion fruit is supported by Italian structure rather than Sauvignon Blanc aromatics."]</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>["medium lemon","green apple","stone fruit","passion fruit","honey with age","mushroom with age","dry","high acidity","medium body","medium to high alcohol","green apple","stone fruit","passion fruit","lean high-acid palate","honey and mushroom with age","higher acidity and leaner body than Fiano","more passion fruit than Gavi","less fennel-almond than Verdicchio"]</t>
+        </is>
+      </c>
+      <c r="AH38" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI38" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Campania - Fiano and Greco evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ38" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Italia - Practica 037</t>
+        </is>
+      </c>
+      <c r="AK38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL38" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN38" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO38" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP38" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Italy white wine profiles are supported by the WSET Northern, Central and Southern Italy chapters.","The selected regions and appellations are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT appearance, finish and diagnostic calibration use widely accepted Italian white wine style norms where WSET is not granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional, grape and style contrasts."],"inferred_high_confidence":["Mentor focus and memory hooks are pedagogical inferences from the WSET style descriptions."]}</t>
+        </is>
+      </c>
+      <c r="AQ38" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium lemon"],"nose":["medium intensity","green apple","stone fruit","passion fruit","honey with age","mushroom with age"],"palate":["dry","high acidity","medium body","medium to high alcohol","green apple","stone fruit","passion fruit"],"quality":["very good to outstanding in best DOCG examples"],"ageing":["medium ageing; best examples develop honey and mushroom"],"diagnostic_features":["campania_fiano_greco_core","cool_climate_high_acid_white","higher acidity and leaner body than Fiano","more passion fruit than Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AR38" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Greco high-acid structure","Campanian white comparison","lees/old-oak texture"],"learning_objectives":["distinguish Greco from Fiano","identify high-acid southern Italian white","connect stainless steel and old oak options to texture"],"typical_misconceptions":["southern whites are always low acid","Greco and Fiano are interchangeable","mushroom age notes mean fault"],"mentor_focus":["ask whether the wine is leaner and higher acid than Fiano"],"exam_traps":["calling Greco Sauvignon Blanc from passion fruit","overstating new oak"],"memory_hooks":["Greco is the leaner, higher-acid Campanian white"],"comparison_styles":["Fiano di Avellino","Gavi","Verdicchio dei Castelli di Jesi"]}</t>
+        </is>
+      </c>
+      <c r="AS38" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_036","SAT_WINE_032"],"frequently_confused_with":["SAT_WINE_036","SAT_WINE_009"],"distinguishing_features":["higher acidity and leaner body than Fiano","more passion fruit than Gavi","less fennel-almond than Verdicchio"]}</t>
+        </is>
+      </c>
+      <c r="AT38" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Greco di Tufo DOCG is a key Campanian white","Greco has more acidity and leaner body than Fiano","best examples can age with honey and mushroom notes"],"mentor_hints":["Compare directly with Fiano before final identification.","Ask whether passion fruit is supported by Italian structure rather than Sauvignon Blanc aromatics."],"student_traps":["confusing Greco and Fiano","misreading mushroom development as fault"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU38" t="inlineStr">
+        <is>
+          <t>["campania_fiano_greco_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV38" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW38" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12431-12449"],"line_reference":["12431-12449"],"evidence":["Greco has more acidity and is leaner in body than Fiano, producing green apple, stone fruit and passion fruit flavours.","Most producers ferment in stainless steel, some use old oak and lees stirring; best examples age with honey and mushrooms."]}</t>
+        </is>
+      </c>
+      <c r="AX38" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-07-BATCH-004","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY38" t="inlineStr">
+        <is>
+          <t>29 Southern Italy</t>
+        </is>
+      </c>
+      <c r="AZ38" t="inlineStr">
+        <is>
+          <t>Campania - Fiano and Greco</t>
+        </is>
+      </c>
+      <c r="BA38" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="BB38" t="inlineStr">
+        <is>
+          <t>["12431-12449"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add Batch 005 Spain Portugal Greece white profiles
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -10346,6 +10346,1638 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SAT_WINE_038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Blancos España / Portugal / Grecia</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Rueda Verdejo</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Fresh to textured Verdejo from continental Rueda</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Rueda Verdejo</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Rueda</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Castilla y Leon</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Rueda DO</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>["Verdejo"]</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>continental climate with cool summer nights</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>high inland plateau between Toro and Ribera del Duero</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>not specified by WSET; continental climate and cool nights are the key markers</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>["Rueda focuses on white wine production","cool summer nights suit Verdejo","blended whites must contain at least 50 percent Verdejo"]</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>["protective winemaking for light high-acid melon and peach styles","skin contact and barrel fermentation can make richer fuller-bodied styles","Sauvignon Blanc may be blended or labelled varietally"]</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>usually unoaked in fresh styles; richer styles may be barrel-fermented</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>["melon","peach","citrus","herbal notes"]</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>["melon","peach","citrus","fresh dry palate"]</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>good to very good; styles range from simple fruity to richer barrel-fermented versions</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>drink young to short ageing for fresh styles</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium intensity","melon","peach","citrus","herbal notes","dry","high acidity","light to medium body","medium alcohol","melon","peach","citrus","fresh dry palate"]</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>["Verdejo is highly susceptible to oxidation","Rueda focuses on white wine production","Rueda blends must contain at least 50 percent Verdejo"]</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>["Rueda is a red-wine region","Verdejo always tastes like Sauvignon Blanc","barrel fermentation means Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>["Probe whether the Sauvignon-like profile still has Verdejo melon and peach.","Ask if winemaking is protective or richer barrel-fermented."]</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>["pale lemon","melon","peach","citrus","herbal notes","dry","high acidity","light to medium body","medium alcohol","melon","peach","citrus","fresh dry palate","melon and peach rather than Albariño citrus-stone fruit","Rueda continental rather than Atlantic damp climate","possible richer barrel-fermented Verdejo style"]</t>
+        </is>
+      </c>
+      <c r="AH39" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI39" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Rueda / Verdejo evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Spain - Practica 038</t>
+        </is>
+      </c>
+      <c r="AK39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN39" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO39" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP39" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Iberian and Greek white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ39" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium intensity","melon","peach","citrus","herbal notes"],"palate":["dry","high acidity","light to medium body","medium alcohol","melon","peach","citrus"],"quality":["good to very good; styles range from simple fruity to richer barrel-fermented versions"],"ageing":["drink young to short ageing for fresh styles"],"diagnostic_features":["rueda_verdejo_core","cool_climate_high_acid_white","melon and peach rather than Albariño citrus-stone fruit","Rueda continental rather than Atlantic damp climate"]}</t>
+        </is>
+      </c>
+      <c r="AR39" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Verdejo oxidation sensitivity","Rueda white wine identity","protective versus richer winemaking"],"learning_objectives":["identify Verdejo structure","connect Rueda to white wine production","separate Verdejo from Sauvignon Blanc"],"typical_misconceptions":["Rueda is a red-wine region","Verdejo always tastes like Sauvignon Blanc","barrel fermentation means Chardonnay"],"mentor_focus":["ask whether melon-peach high-acid fruit points to Verdejo"],"exam_traps":["calling all Rueda Sauvignon Blanc","forgetting Verdejo minimum in blends"],"memory_hooks":["Rueda is Verdejo country: cool nights, melon, peach, high acidity"],"comparison_styles":["Rias Baixas Albarino","Gavi","Alto Adige Pinot Grigio"]}</t>
+        </is>
+      </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_039","SAT_WINE_032"],"frequently_confused_with":["SAT_WINE_009","SAT_WINE_028"],"distinguishing_features":["melon and peach rather than Albariño citrus-stone fruit","Rueda continental rather than Atlantic damp climate","possible richer barrel-fermented Verdejo style"]}</t>
+        </is>
+      </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Verdejo is highly susceptible to oxidation","Rueda focuses on white wine production","Rueda blends must contain at least 50 percent Verdejo"],"mentor_hints":["Probe whether the Sauvignon-like profile still has Verdejo melon and peach.","Ask if winemaking is protective or richer barrel-fermented."],"student_traps":["overcalling Sauvignon Blanc","missing Rueda as a white specialist"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU39" t="inlineStr">
+        <is>
+          <t>["rueda_verdejo_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV39" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW39" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12801-12808","13287-13302"],"line_reference":["12801-12808","13287-13302"],"evidence":["Verdejo can be made protectively into a light-bodied high-acid melon and peach style or richer with skin contact and barrel fermentation.","Rueda focuses on white wine production; its continental climate with cool summer nights is ideal for Verdejo."]}</t>
+        </is>
+      </c>
+      <c r="AX39" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-08-BATCH-005","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY39" t="inlineStr">
+        <is>
+          <t>30 Spain</t>
+        </is>
+      </c>
+      <c r="AZ39" t="inlineStr">
+        <is>
+          <t>Rueda / Verdejo</t>
+        </is>
+      </c>
+      <c r="BA39" t="inlineStr">
+        <is>
+          <t>133, 137</t>
+        </is>
+      </c>
+      <c r="BB39" t="inlineStr">
+        <is>
+          <t>["12801-12808","13287-13302"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SAT_WINE_039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Blancos España / Portugal / Grecia</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Rias Baixas Albarino</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Refreshing Atlantic Albariño with high acidity and ripe stone fruit</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Rias Baixas Albarino</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Rias Baixas</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>North-west Spain</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Rias Baixas DO</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>["Albarino"]</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>moderate damp Atlantic climate, cooler and wetter than most of Spain</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>coastal and low hill Atlantic vineyards</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>not specified by WSET; damp Atlantic setting is the key marker</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>["humid conditions make mildew and rot common","pergolas encourage air circulation","Albariño has thick skins that resist fungal disease"]</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>["most Albariño is refreshing and unoaked","some richer styles use oak or lees contact","fruit and acidity are preserved"]</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>usually unoaked; occasional touch of oak or lees in richer styles</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","peach","saline freshness"]</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>["citrus","stone fruit","ripe peach","refreshing high-acid palate"]</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>very good; among Spain's most celebrated white wines</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>drink young to short ageing; richer styles may hold longer</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium intensity","citrus","stone fruit","peach","saline freshness","dry","high acidity","medium body","medium alcohol","citrus","stone fruit","ripe peach","refreshing high-acid palate"]</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>["Rias Baixas is the most celebrated north-west Spanish white area","Albariño is naturally high in acidity","pergolas help air circulation in damp conditions"]</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>["Spain is too hot for high-acid whites","all Albariño is oaked","pergola is only for Italy"]</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>["Ask if disease pressure and pergola logic fit the region.","Use ripe stone fruit to avoid defaulting to Sauvignon Blanc."]</t>
+        </is>
+      </c>
+      <c r="AG40" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","citrus","stone fruit","peach","saline freshness","dry","high acidity","medium body","medium alcohol","citrus","stone fruit","ripe peach","refreshing high-acid palate","more Atlantic and stone-fruited than Rueda","higher alcohol and ripeness than classic Vinho Verde","less floral than Gavi"]</t>
+        </is>
+      </c>
+      <c r="AH40" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI40" t="inlineStr">
+        <is>
+          <t>Profile uses WSET North West - Rias Baixas / Albariño evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ40" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Spain - Practica 039</t>
+        </is>
+      </c>
+      <c r="AK40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL40" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM40" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN40" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO40" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP40" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Iberian and Greek white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ40" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium intensity","citrus","stone fruit","peach","saline freshness"],"palate":["dry","high acidity","medium body","medium alcohol","citrus","stone fruit","ripe peach"],"quality":["very good; among Spain's most celebrated white wines"],"ageing":["drink young to short ageing; richer styles may hold longer"],"diagnostic_features":["rias_baixas_albarino_core","cool_climate_high_acid_white","more Atlantic and stone-fruited than Rueda","higher alcohol and ripeness than classic Vinho Verde"]}</t>
+        </is>
+      </c>
+      <c r="AR40" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Atlantic Spain whites","Albariño thick skin and acidity","pergola disease management"],"learning_objectives":["identify Rias Baixas Albariño","connect damp climate to pergola training","separate Albariño from Verdejo"],"typical_misconceptions":["Spain is too hot for high-acid whites","all Albariño is oaked","pergola is only for Italy"],"mentor_focus":["ask for Atlantic freshness plus ripe stone fruit"],"exam_traps":["calling it Sauvignon Blanc from acidity alone","forgetting fungal pressure"],"memory_hooks":["Rías Baixas is Atlantic Albariño: damp, pergola, citrus-stone fruit"],"comparison_styles":["Rueda Verdejo","Vinho Verde","Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AS40" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_038","SAT_WINE_041"],"frequently_confused_with":["SAT_WINE_009","SAT_WINE_032"],"distinguishing_features":["more Atlantic and stone-fruited than Rueda","higher alcohol and ripeness than classic Vinho Verde","less floral than Gavi"]}</t>
+        </is>
+      </c>
+      <c r="AT40" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Rias Baixas is the most celebrated north-west Spanish white area","Albariño is naturally high in acidity","pergolas help air circulation in damp conditions"],"mentor_hints":["Ask if disease pressure and pergola logic fit the region.","Use ripe stone fruit to avoid defaulting to Sauvignon Blanc."],"student_traps":["forgetting north-west Spain","underestimating Albariño quality"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU40" t="inlineStr">
+        <is>
+          <t>["rias_baixas_albarino_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV40" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW40" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12810-12818","13304-13324"],"line_reference":["12810-12818","13304-13324"],"evidence":["Albariño is grown in north-west Spain, is thick-skinned, naturally high in acidity and gives citrus and stone fruit wines.","Rias Baixas has a moderate damp Atlantic climate; most Albariño is refreshing and unoaked with high acidity and ripe stone fruit."]}</t>
+        </is>
+      </c>
+      <c r="AX40" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-08-BATCH-005","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY40" t="inlineStr">
+        <is>
+          <t>30 Spain</t>
+        </is>
+      </c>
+      <c r="AZ40" t="inlineStr">
+        <is>
+          <t>North West - Rias Baixas / Albariño</t>
+        </is>
+      </c>
+      <c r="BA40" t="inlineStr">
+        <is>
+          <t>133, 137</t>
+        </is>
+      </c>
+      <c r="BB40" t="inlineStr">
+        <is>
+          <t>["12810-12818","13304-13324"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SAT_WINE_040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Blancos España / Portugal / Grecia</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>White Rioja Viura</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Viura-based white Rioja from traditional oxidative oak to modern fruit-led styles</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>White Rioja Viura</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Rioja</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Rioja Alta / Rioja Alavesa / Rioja Oriental</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Rioja DOCa</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>["Viura"]</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Rioja is protected from Atlantic weather by mountains with varied subregional influences</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>foothill and valley sites across Rioja; WSET emphasizes regional winemaking over altitude for white Rioja</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>not specified by WSET for white Rioja in this passage</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>["Viura is the most widely planted white variety in Rioja","eight white varieties are approved","regional ageing and oak culture affect style"]</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>["traditional white Rioja aged for extended periods in American oak","traditional style developed deep golden colour and nutty flavours","modern styles minimize oxygen to preserve fruit; some are barrel-fermented in a less oxidative style"]</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>American oak and barrel fermentation can be important, but modern styles may show less oxidation</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>medium lemon to gold depending on style</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>["citrus","apple","nutty notes","vanilla","subtle spice"]</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>["citrus","apple","nutty oxidative notes","spicy oak","fresh fruit in modern styles"]</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>good to very good; style depends strongly on producer and oxygen/oak choices</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>short to medium ageing; traditional oxidative styles can show developed character</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>["medium lemon to gold depending on style","medium intensity","citrus","apple","nutty notes","vanilla","subtle spice","dry","medium to high acidity","medium body","medium alcohol","citrus","apple","nutty oxidative notes","spicy oak","fresh fruit in modern styles"]</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>["Viura is the most widely planted white Rioja variety","traditional styles used extended American oak ageing","modern styles use less oxygen to preserve fruit"]</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>["Rioja only makes red wine","all white Rioja is oxidised","all oak-aged white wine is Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>["Ask whether oak is stylistic Rioja rather than Chardonnay evidence.","Separate colour from sweetness."]</t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>["medium lemon to gold depending on style","citrus","apple","nutty notes","vanilla","subtle spice","dry","medium to high acidity","medium body","medium alcohol","citrus","apple","nutty oxidative notes","spicy oak","fresh fruit in modern styles","more oak/oxygen signature than Rueda","less Garganega pear-almond than Soave","Spanish Viura identity rather than Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="AH41" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI41" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Rioja - White Rioja evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ41" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Spain - Practica 040</t>
+        </is>
+      </c>
+      <c r="AK41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL41" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO41" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="AP41" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Iberian and Greek white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ41" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium lemon to gold depending on style"],"nose":["medium intensity","citrus","apple","nutty notes","vanilla","subtle spice"],"palate":["dry","medium to high acidity","medium body","medium alcohol","citrus","apple","nutty oxidative notes"],"quality":["good to very good; style depends strongly on producer and oxygen/oak choices"],"ageing":["short to medium ageing; traditional oxidative styles can show developed character"],"diagnostic_features":["white_rioja_viura_core","white_wine_sat_core","more oak/oxygen signature than Rueda","less Garganega pear-almond than Soave"]}</t>
+        </is>
+      </c>
+      <c r="AR41" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Rioja white style range","Viura identity","oxidative versus modern winemaking"],"learning_objectives":["identify oak/oxygen choices in white Rioja","separate Viura Rioja from neutral Spanish whites","understand traditional versus modern style"],"typical_misconceptions":["Rioja only makes red wine","all white Rioja is oxidised","all oak-aged white wine is Chardonnay"],"mentor_focus":["ask whether nutty oak-derived development points to Rioja"],"exam_traps":["missing Viura","assuming deep gold means sweet"],"memory_hooks":["White Rioja is Viura shaped by oak and oxygen decisions"],"comparison_styles":["Rueda Verdejo","Soave Classico","Fiano di Avellino"]}</t>
+        </is>
+      </c>
+      <c r="AS41" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_038","SAT_WINE_031"],"frequently_confused_with":["SAT_WINE_003","SAT_WINE_036"],"distinguishing_features":["more oak/oxygen signature than Rueda","less Garganega pear-almond than Soave","Spanish Viura identity rather than Chardonnay"]}</t>
+        </is>
+      </c>
+      <c r="AT41" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Viura is the most widely planted white Rioja variety","traditional styles used extended American oak ageing","modern styles use less oxygen to preserve fruit"],"mentor_hints":["Ask whether oak is stylistic Rioja rather than Chardonnay evidence.","Separate colour from sweetness."],"student_traps":["forgetting white Rioja","overcalling oxidation as fault"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU41" t="inlineStr">
+        <is>
+          <t>["white_rioja_viura_core","white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV41" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW41" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13047-13076"],"line_reference":["13047-13076"],"evidence":["The most widely planted white variety in Rioja is Viura.","Traditional white Rioja was aged in American oak and developed deep golden colour and nutty flavours; modern styles preserve fruit and some are barrel-fermented less oxidatively."]}</t>
+        </is>
+      </c>
+      <c r="AX41" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-08-BATCH-005","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY41" t="inlineStr">
+        <is>
+          <t>30 Spain</t>
+        </is>
+      </c>
+      <c r="AZ41" t="inlineStr">
+        <is>
+          <t>Rioja - White Rioja</t>
+        </is>
+      </c>
+      <c r="BA41" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="BB41" t="inlineStr">
+        <is>
+          <t>["13047-13076"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SAT_WINE_041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Blancos España / Portugal / Grecia</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Vinho Verde</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Low-alcohol high-acid north-west Portuguese white with slight spritz</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Vinho Verde</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Vinho Verde</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>North-west Portugal</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Vinho Verde DOC</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>["Loureiro","Arinto"]</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>moderate maritime climate near the Atlantic with high annual rainfall</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>humid north-west Portuguese vineyards; altitude is not the key WSET marker</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>not specified by WSET; rainfall and Atlantic influence dominate the style</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>["high precipitation can cause excessive canopy and disease","modern vineyards moved away from traditional pergolas","spur-pruned VSP improves airflow and mechanisation"]</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>["classic whites are pale lemon, high acid and low alcohol","lower-alcohol wines are usually off-dry","traditional slight sparkling sensation enhances freshness"]</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>unoaked</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>dry to off-dry</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>["citrus","green apple","floral notes"]</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>["citrus","green apple","slight spritz","fresh high-acid palate"]</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>short to medium</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>good; freshness and drinkability are central</t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>drink young</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium intensity","citrus","green apple","floral notes","dry to off-dry","high acidity","light body","low alcohol","citrus","green apple","slight spritz","fresh high-acid palate"]</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>["Vinho Verde is in north-west Portugal","high rainfall requires canopy management","classic whites are pale, high-acid and low-alcohol with slight sparkle"]</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>["all Portuguese whites are fortified-related","spritz means sparkling wine category","off-dry means low acidity"]</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>["Ask for alcohol level before naming Albariño.","Use spritz as a clue but not as full sparkling classification."]</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr">
+        <is>
+          <t>["pale lemon","citrus","green apple","floral notes","dry to off-dry","high acidity","light body","low alcohol","citrus","green apple","slight spritz","fresh high-acid palate","lower alcohol and spritz versus Rias Baixas","more off-dry possibility than Muscadet","Atlantic Portugal rather than north-west Spain"]</t>
+        </is>
+      </c>
+      <c r="AH42" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI42" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Vinho Verde evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ42" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Portugal - Practica 041</t>
+        </is>
+      </c>
+      <c r="AK42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL42" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM42" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN42" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO42" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP42" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Iberian and Greek white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ42" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium intensity","citrus","green apple","floral notes"],"palate":["dry to off-dry","high acidity","light body","low alcohol","citrus","green apple","slight spritz"],"quality":["good; freshness and drinkability are central"],"ageing":["drink young"],"diagnostic_features":["vinho_verde_core","cool_climate_high_acid_white","lower alcohol and spritz versus Rias Baixas","more off-dry possibility than Muscadet"]}</t>
+        </is>
+      </c>
+      <c r="AR42" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Portuguese Atlantic freshness","low alcohol high acidity","spritz and off-dry balance"],"learning_objectives":["identify classic Vinho Verde","connect high rainfall to canopy management","separate Vinho Verde from Albariño"],"typical_misconceptions":["all Portuguese whites are fortified-related","spritz means sparkling wine category","off-dry means low acidity"],"mentor_focus":["ask for low alcohol, high acidity and slight spritz"],"exam_traps":["calling Vinho Verde Albariño because Alvarinho exists","missing off-dry possibility"],"memory_hooks":["Vinho Verde is pale, low-alcohol, high-acid and lightly spritzy"],"comparison_styles":["Rias Baixas Albarino","Muscadet","Rueda Verdejo"]}</t>
+        </is>
+      </c>
+      <c r="AS42" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_039"],"frequently_confused_with":["SAT_WINE_039","SAT_WINE_008"],"distinguishing_features":["lower alcohol and spritz versus Rias Baixas","more off-dry possibility than Muscadet","Atlantic Portugal rather than north-west Spain"]}</t>
+        </is>
+      </c>
+      <c r="AT42" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Vinho Verde is in north-west Portugal","high rainfall requires canopy management","classic whites are pale, high-acid and low-alcohol with slight sparkle"],"mentor_hints":["Ask for alcohol level before naming Albariño.","Use spritz as a clue but not as full sparkling classification."],"student_traps":["forgetting Portuguese still whites","overlooking low alcohol"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU42" t="inlineStr">
+        <is>
+          <t>["vinho_verde_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV42" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW42" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13446-13472"],"line_reference":["13446-13472"],"evidence":["Vinho Verde has a moderate maritime climate near the Atlantic with high rainfall and disease pressure.","Classic white Vinho Verde is pale lemon, high in acidity, low in alcohol, often off-dry at lower alcohol, and traditionally has slight spritz."]}</t>
+        </is>
+      </c>
+      <c r="AX42" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-08-BATCH-005","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY42" t="inlineStr">
+        <is>
+          <t>31 Portugal</t>
+        </is>
+      </c>
+      <c r="AZ42" t="inlineStr">
+        <is>
+          <t>Vinho Verde</t>
+        </is>
+      </c>
+      <c r="BA42" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="BB42" t="inlineStr">
+        <is>
+          <t>["13446-13472"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SAT_WINE_042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Blancos España / Portugal / Grecia</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Dao Encruzado</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Dão Encruzado from light fresh to richer barrel-fermented white</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Dao Encruzado</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Dao</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Central Portugal</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Dao DOC</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>["Encruzado"]</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>mountainous inland region with cold wet winters, warm dry summers and significant day-night temperature variation</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>vineyards on gentler hills and slopes between 200 and 400 metres</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>not specified by WSET for Encruzado; mountainous slope setting is the key marker</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>["vines planted on hills and slopes","day-night temperature variation supports quality grapes","Encruzado is the leading white variety"]</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>["styles range from light and fresh to richer barrel-fermented versions","fresh styles preserve fruit","barrel fermentation can add texture"]</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>none in fresh styles; richer examples may be barrel-fermented</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>["citrus","apple","pear","subtle toast in barrel styles"]</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>["citrus","pear","fresh dry palate","textured barrel-fermented notes"]</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>short to medium ageing for richer examples</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium intensity","citrus","apple","pear","subtle toast in barrel styles","dry","medium to high acidity","medium body","medium alcohol","citrus","pear","fresh dry palate","textured barrel-fermented notes"]</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>["Dão vineyards lie between 200 and 400 metres","day-night variation supports high-quality grapes","best Dão whites are Encruzado"]</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t>["Dão only matters for reds","Portuguese white grapes are not WSET relevant","barrel-fermented means Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>["Ask whether Portugal and barrel fermentation are both plausible.","Avoid using oak alone as a Chardonnay shortcut."]</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","citrus","apple","pear","subtle toast in barrel styles","dry","medium to high acidity","medium body","medium alcohol","citrus","pear","fresh dry palate","textured barrel-fermented notes","more medium-bodied than Vinho Verde","less Rioja oxidative oak identity","Portuguese Encruzado rather than Verdejo"]</t>
+        </is>
+      </c>
+      <c r="AH43" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI43" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Dão evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ43" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Portugal - Practica 042</t>
+        </is>
+      </c>
+      <c r="AK43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL43" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO43" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="AP43" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Iberian and Greek white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ43" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium intensity","citrus","apple","pear","subtle toast in barrel styles"],"palate":["dry","medium to high acidity","medium body","medium alcohol","citrus","pear","fresh dry palate"],"quality":["good to very good"],"ageing":["short to medium ageing for richer examples"],"diagnostic_features":["dao_encruzado_core","white_wine_sat_core","more medium-bodied than Vinho Verde","less Rioja oxidative oak identity"]}</t>
+        </is>
+      </c>
+      <c r="AR43" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Dão white identity","Encruzado style range","barrel fermentation as optional texture"],"learning_objectives":["recognize Encruzado as Dão white grape","separate fresh and barrel-fermented expressions","connect altitude range to quality"],"typical_misconceptions":["Dão only matters for reds","Portuguese white grapes are not WSET relevant","barrel-fermented means Chardonnay"],"mentor_focus":["ask whether the style range fits Encruzado rather than a single aromatic grape"],"exam_traps":["ignoring Portugal beyond Vinho Verde","overstating oak"],"memory_hooks":["Dão Encruzado can be fresh or barrel-textured from mountain slopes"],"comparison_styles":["Vinho Verde","White Rioja Viura","Rueda Verdejo"]}</t>
+        </is>
+      </c>
+      <c r="AS43" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_040"],"frequently_confused_with":["SAT_WINE_003","SAT_WINE_038"],"distinguishing_features":["more medium-bodied than Vinho Verde","less Rioja oxidative oak identity","Portuguese Encruzado rather than Verdejo"]}</t>
+        </is>
+      </c>
+      <c r="AT43" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Dão vineyards lie between 200 and 400 metres","day-night variation supports high-quality grapes","best Dão whites are Encruzado"],"mentor_hints":["Ask whether Portugal and barrel fermentation are both plausible.","Avoid using oak alone as a Chardonnay shortcut."],"student_traps":["forgetting Encruzado","collapsing all Portuguese whites into Vinho Verde"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU43" t="inlineStr">
+        <is>
+          <t>["dao_encruzado_core","white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV43" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW43" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13555-13574"],"line_reference":["13555-13574"],"evidence":["Dão is mountainous with vines between 200 and 400 metres and significant day-night temperature variation.","The best Dão whites are made from Encruzado and range from light and fresh to richer barrel-fermented versions."]}</t>
+        </is>
+      </c>
+      <c r="AX43" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-08-BATCH-005","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY43" t="inlineStr">
+        <is>
+          <t>31 Portugal</t>
+        </is>
+      </c>
+      <c r="AZ43" t="inlineStr">
+        <is>
+          <t>Dão</t>
+        </is>
+      </c>
+      <c r="BA43" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="BB43" t="inlineStr">
+        <is>
+          <t>["13555-13574"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SAT_WINE_043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Blancos España / Portugal / Grecia</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Santorini Assyrtiko</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Dry volcanic Assyrtiko with ripe citrus, stone fruit and natural high acidity</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Santorini Assyrtiko</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Greece</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Santorini</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Aegean Islands</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Santorini PDO</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>["Assyrtiko"]</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>hot Mediterranean Greece moderated by sea, altitude and strong island winds; very dry growing season</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>windswept volcanic island sites; vines are trained very low in baskets</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>volcanic island soils; WSET emphasizes Santorini as a volcanic island</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>["strong winds require basket-trained vines","fruit grows inside the low basket shape","native varieties are adapted to hot arid conditions"]</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>["dry white Assyrtiko has the highest reputation","concentrated ripe citrus and stone fruit flavours","sweet Vinsanto also exists but this profile is dry Assyrtiko"]</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>typically not a primary marker for dry Assyrtiko</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>["ripe citrus","stone fruit","mineral saline notes"]</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>["ripe citrus","stone fruit","concentrated dry palate","saline mineral finish"]</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>very good to outstanding; Santorini Assyrtiko has the highest reputation among Santorini wines</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>medium ageing for concentrated dry examples</t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium intensity","ripe citrus","stone fruit","mineral saline notes","dry","high acidity","medium to full body","medium to high alcohol","ripe citrus","stone fruit","concentrated dry palate","saline mineral finish"]</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>["Santorini is a windswept volcanic island","vines are trained low in baskets","Assyrtiko dry whites have ripe citrus, stone fruit and natural high acidity"]</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t>["hot Greece cannot make high-acid whites","Santorini only makes sweet wine","mineral saline notes identify Chablis"]</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>["Ask how a hot climate wine can retain high acidity.","Use basket training as a source clue after debrief."]</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","ripe citrus","stone fruit","mineral saline notes","dry","high acidity","medium to full body","medium to high alcohol","ripe citrus","stone fruit","concentrated dry palate","saline mineral finish","riper and more concentrated than Chablis","volcanic basket-vine context","high acidity despite hot Mediterranean setting"]</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI44" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Santorini PDO evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ44" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Greece - Practica 043</t>
+        </is>
+      </c>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL44" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN44" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO44" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP44" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Iberian and Greek white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ44" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium intensity","ripe citrus","stone fruit","mineral saline notes"],"palate":["dry","high acidity","medium to full body","medium to high alcohol","ripe citrus","stone fruit","concentrated dry palate"],"quality":["very good to outstanding; Santorini Assyrtiko has the highest reputation among Santorini wines"],"ageing":["medium ageing for concentrated dry examples"],"diagnostic_features":["santorini_assyrtiko_core","cool_climate_high_acid_white","riper and more concentrated than Chablis","volcanic basket-vine context"]}</t>
+        </is>
+      </c>
+      <c r="AR44" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Greek native varieties","Santorini volcanic island identity","high acidity in hot climate"],"learning_objectives":["identify dry Assyrtiko structure","connect wind to basket training","separate Assyrtiko from Riesling or Sauvignon Blanc"],"typical_misconceptions":["hot Greece cannot make high-acid whites","Santorini only makes sweet wine","mineral saline notes identify Chablis"],"mentor_focus":["ask whether high acidity comes with ripe citrus concentration and volcanic island context"],"exam_traps":["calling it Chablis because of acidity and minerality","forgetting basket training"],"memory_hooks":["Santorini Assyrtiko is hot-island concentration with high-acid backbone"],"comparison_styles":["Chablis","Gavi","Rueda Verdejo"]}</t>
+        </is>
+      </c>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_001","SAT_WINE_032"],"frequently_confused_with":["SAT_WINE_001","SAT_WINE_009"],"distinguishing_features":["riper and more concentrated than Chablis","volcanic basket-vine context","high acidity despite hot Mediterranean setting"]}</t>
+        </is>
+      </c>
+      <c r="AT44" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Santorini is a windswept volcanic island","vines are trained low in baskets","Assyrtiko dry whites have ripe citrus, stone fruit and natural high acidity"],"mentor_hints":["Ask how a hot climate wine can retain high acidity.","Use basket training as a source clue after debrief."],"student_traps":["confusing minerality with Chablis","missing Greece as WSET core region"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU44" t="inlineStr">
+        <is>
+          <t>["santorini_assyrtiko_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV44" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW44" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11419-11430","11505-11530"],"line_reference":["11419-11430","11505-11530"],"evidence":["Santorini is a windswept volcanic island where vines are trained low into baskets to protect them from strong winds.","White wines made from Assyrtiko have the highest reputation, with ripe citrus and stone fruit balanced by natural high acidity."]}</t>
+        </is>
+      </c>
+      <c r="AX44" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-08-BATCH-005","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY44" t="inlineStr">
+        <is>
+          <t>25 Greece</t>
+        </is>
+      </c>
+      <c r="AZ44" t="inlineStr">
+        <is>
+          <t>Santorini PDO</t>
+        </is>
+      </c>
+      <c r="BA44" t="inlineStr">
+        <is>
+          <t>118-119</t>
+        </is>
+      </c>
+      <c r="BB44" t="inlineStr">
+        <is>
+          <t>["11419-11430","11505-11530"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add Batch 006 New World white profiles
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -11978,6 +11978,2182 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SAT_WINE_044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Blancos Nuevo Mundo</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>California Chardonnay</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Broad California Chardonnay style range</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>California Chardonnay</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Statewide / coastal premium regions</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>California AVA / regional AVAs</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>["Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>wide California climate range; cooler coastal regions give more restrained premium Chardonnay</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>coastal valleys and cooler AVAs such as Los Carneros and Russian River Valley</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>varied; WSET emphasizes climate and winemaking style range</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>["Chardonnay is the most planted grape in California","cooler premium regions now make restrained examples","Central Valley gives inexpensive fruity wines"]</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>["range from inexpensive fruity wines to premium barrel-influenced styles","oak staves or chips may be used in inexpensive wines","premium styles may show oak, butter and hazelnut or more restrained less-oak handling"]</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>variable; traditional premium styles may show obvious oak, hazelnut and butter</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>medium lemon to gold</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>["peach","banana","citrus","oak","butter"]</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>["peach","banana","citrus","toasty oak","buttery texture"]</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>good to outstanding depending on region and producer</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>short to medium ageing; premium examples can age</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>["medium lemon to gold","medium to pronounced intensity","peach","banana","citrus","oak","butter","dry","medium acidity","medium to full body","medium to high alcohol","peach","banana","citrus","toasty oak","buttery texture"]</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>["Chardonnay is California's most planted grape","premium California Chardonnay formerly had full body, high alcohol, low acidity and oak/butter/hazelnut","cooler regions now produce restrained examples"]</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t>["all California Chardonnay is heavily oaked","butter always means fault","Chardonnay has one fixed style"]</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>["Ask what evidence supports Chardonnay beyond oak.","Use California style range as the teaching frame."]</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>["medium lemon to gold","peach","banana","citrus","oak","butter","dry","medium acidity","medium to full body","medium to high alcohol","peach","banana","citrus","toasty oak","buttery texture","more overt peach-banana and oak than Chablis","broader than Sonoma Coast examples","not Viura oxidative nutty Rioja"]</t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>Profile uses WSET White grape varieties - Chardonnay evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ45" t="inlineStr">
+        <is>
+          <t>Vino Blanco - USA - Practica 044</t>
+        </is>
+      </c>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO45" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP45" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected New World white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ45" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium lemon to gold"],"nose":["medium to pronounced intensity","peach","banana","citrus","oak","butter"],"palate":["dry","medium acidity","medium to full body","medium to high alcohol","peach","banana","citrus"],"quality":["good to outstanding depending on region and producer"],"ageing":["short to medium ageing; premium examples can age"],"diagnostic_features":["california_chardonnay_core","premium_chardonnay_winemaking","more overt peach-banana and oak than Chablis","broader than Sonoma Coast examples"]}</t>
+        </is>
+      </c>
+      <c r="AR45" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["California Chardonnay style range","oak and malolactic signatures","cooler premium restraint"],"learning_objectives":["identify New World Chardonnay markers","separate oak from grape identity","contrast warm and cool California styles"],"typical_misconceptions":["all California Chardonnay is heavily oaked","butter always means fault","Chardonnay has one fixed style"],"mentor_focus":["ask whether oak, body and fruit ripeness align"],"exam_traps":["overcalling Burgundy","ignoring cooler restrained California examples"],"memory_hooks":["California Chardonnay spans butter-oak tradition and cooler restraint"],"comparison_styles":["Sonoma Coast Chardonnay","White Rioja Viura","Fiano di Avellino"]}</t>
+        </is>
+      </c>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_045","SAT_WINE_040"],"frequently_confused_with":["SAT_WINE_003","SAT_WINE_036"],"distinguishing_features":["more overt peach-banana and oak than Chablis","broader than Sonoma Coast examples","not Viura oxidative nutty Rioja"]}</t>
+        </is>
+      </c>
+      <c r="AT45" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Chardonnay is California's most planted grape","premium California Chardonnay formerly had full body, high alcohol, low acidity and oak/butter/hazelnut","cooler regions now produce restrained examples"],"mentor_hints":["Ask what evidence supports Chardonnay beyond oak.","Use California style range as the teaching frame."],"student_traps":["calling all oaked whites Chardonnay","missing restrained modern styles"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU45" t="inlineStr">
+        <is>
+          <t>["california_chardonnay_core","premium_chardonnay_winemaking"]</t>
+        </is>
+      </c>
+      <c r="AV45" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW45" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13901-13913"],"line_reference":["13901-13913"],"evidence":["Chardonnay is the most planted grape in California with styles from fruity Central Valley to premium fuller oak-influenced wines.","Today California also produces restrained premium Chardonnay with less oak from cooler regions such as Los Carneros and Russian River Valley."]}</t>
+        </is>
+      </c>
+      <c r="AX45" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-09-BATCH-006","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY45" t="inlineStr">
+        <is>
+          <t>33 California</t>
+        </is>
+      </c>
+      <c r="AZ45" t="inlineStr">
+        <is>
+          <t>White grape varieties - Chardonnay</t>
+        </is>
+      </c>
+      <c r="BA45" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="BB45" t="inlineStr">
+        <is>
+          <t>["13901-13913"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SAT_WINE_045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Blancos Nuevo Mundo</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Sonoma Coast Chardonnay</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Cool Pacific-influenced premium Sonoma Chardonnay</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Sonoma Coast Chardonnay</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Sonoma Coast</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Sonoma County</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Sonoma Coast AVA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>["Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>cool Pacific-influenced Sonoma Coast climate with south-facing slopes used to maximize ripening</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>coastal slopes influenced by cold Pacific Ocean</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>not specified by WSET; Pacific influence and slope aspect are key</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>["vineyards often planted on south-facing slopes","cold Pacific Ocean strongly influences climate","nearby Sonoma AVAs include high-quality Chardonnay areas"]</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>["premium cool-climate Chardonnay production","oak and lees may be used but restraint is expected","fruit ripens slowly in cool coastal conditions"]</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>moderate, often integrated; not necessarily overt</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>pale to medium lemon</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>["citrus","green apple","peach","subtle oak","lees"]</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>["citrus","peach","fresh acidity","subtle oak texture"]</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>very good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>medium ageing for best examples</t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","medium to pronounced intensity","citrus","green apple","peach","subtle oak","lees","dry","medium to high acidity","medium body","medium alcohol","citrus","peach","fresh acidity","subtle oak texture"]</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>["Sonoma Coast is influenced by the cold Pacific Ocean","Russian River Valley is known for elegant Chardonnay","Sonoma Valley also produces high-quality Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t>["Sonoma is always warm","California Chardonnay must be full and buttery","cool climate means underripe"]</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>["Ask if fruit ripeness and oak point outside Burgundy.","Use fog/Pacific influence as debrief causal logic."]</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>["pale to medium lemon","citrus","green apple","peach","subtle oak","lees","dry","medium to high acidity","medium body","medium alcohol","citrus","peach","fresh acidity","subtle oak texture","cooler and more acid-led than generic California Chardonnay","more new-world fruit than Chablis","Pacific influence is central"]</t>
+        </is>
+      </c>
+      <c r="AH46" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI46" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Sonoma and Mendocino Counties evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ46" t="inlineStr">
+        <is>
+          <t>Vino Blanco - USA - Practica 045</t>
+        </is>
+      </c>
+      <c r="AK46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL46" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN46" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO46" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="AP46" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected New World white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ46" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium lemon"],"nose":["medium to pronounced intensity","citrus","green apple","peach","subtle oak","lees"],"palate":["dry","medium to high acidity","medium body","medium alcohol","citrus","peach","fresh acidity"],"quality":["very good to outstanding"],"ageing":["medium ageing for best examples"],"diagnostic_features":["california_chardonnay_core","premium_chardonnay_winemaking","cooler and more acid-led than generic California Chardonnay","more new-world fruit than Chablis"]}</t>
+        </is>
+      </c>
+      <c r="AR46" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["cool coastal California Chardonnay","Pacific fog and slope effect","premium restrained style"],"learning_objectives":["separate Sonoma Coast from broader California Chardonnay","identify cool-climate Chardonnay features","link Pacific influence to acidity"],"typical_misconceptions":["Sonoma is always warm","California Chardonnay must be full and buttery","cool climate means underripe"],"mentor_focus":["ask whether acidity and restrained oak suggest coastal origin"],"exam_traps":["overgeneralizing California Chardonnay","calling it Chablis from acidity alone"],"memory_hooks":["Sonoma Coast is California Chardonnay in a cooler Pacific key"],"comparison_styles":["California Chardonnay","Chablis","Margaret River Chardonnay"]}</t>
+        </is>
+      </c>
+      <c r="AS46" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_044","SAT_WINE_001"],"frequently_confused_with":["SAT_WINE_001","SAT_WINE_003"],"distinguishing_features":["cooler and more acid-led than generic California Chardonnay","more new-world fruit than Chablis","Pacific influence is central"]}</t>
+        </is>
+      </c>
+      <c r="AT46" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Sonoma Coast is influenced by the cold Pacific Ocean","Russian River Valley is known for elegant Chardonnay","Sonoma Valley also produces high-quality Chardonnay"],"mentor_hints":["Ask if fruit ripeness and oak point outside Burgundy.","Use fog/Pacific influence as debrief causal logic."],"student_traps":["assuming all California is hot","missing Sonoma Coast restraint"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU46" t="inlineStr">
+        <is>
+          <t>["california_chardonnay_core","premium_chardonnay_winemaking"]</t>
+        </is>
+      </c>
+      <c r="AV46" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW46" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["14068-14103"],"line_reference":["14068-14103"],"evidence":["Russian River Valley is cool and foggy and best known for high-quality elegant Pinot Noir and Chardonnay.","Sonoma Coast is strongly influenced by the cold Pacific Ocean with south-facing slopes to maximize ripening; Sonoma Valley produces high-quality Chardonnays."]}</t>
+        </is>
+      </c>
+      <c r="AX46" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-09-BATCH-006","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY46" t="inlineStr">
+        <is>
+          <t>33 California</t>
+        </is>
+      </c>
+      <c r="AZ46" t="inlineStr">
+        <is>
+          <t>Sonoma and Mendocino Counties</t>
+        </is>
+      </c>
+      <c r="BA46" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="BB46" t="inlineStr">
+        <is>
+          <t>["14068-14103"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SAT_WINE_046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Blancos Nuevo Mundo</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Chile Coastal Sauvignon Blanc</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Cool coastal Chilean Sauvignon Blanc with ripe fruit and high acidity</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Chile Coastal Sauvignon Blanc</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Casablanca / San Antonio</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Coastal Chile</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Casablanca Valley / San Antonio Valley</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>["Sauvignon Blanc"]</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>cooler coastal sites influenced by Pacific conditions</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>coastal valleys west of Chile's central areas</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>not specified by WSET; coastal cooling is key</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>["Sauvignon Blanc performs particularly well in cooler sites","Casablanca and San Antonio yield excellent wines","some examples gain texture from lees and oak"]</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>["cool fermentation to preserve fruit","some lees stirring and oak for richness","fresh aromatic Sauvignon Blanc style"]</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>usually unoaked; some examples use lees and oak for texture</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>["ripe apple","citrus","tropical fruit","herbaceous notes"]</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>["ripe apple","citrus","tropical fruit","fresh high-acid palate"]</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>very good; excellent examples from cooler coastal valleys</t>
+        </is>
+      </c>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>drink young to short ageing</t>
+        </is>
+      </c>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium to pronounced intensity","ripe apple","citrus","tropical fruit","herbaceous notes","dry","high acidity","medium body","medium alcohol","ripe apple","citrus","tropical fruit","fresh high-acid palate"]</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>["Sauvignon Blanc performs well in Casablanca and San Antonio","wines have high acidity and intense fruity flavours","some examples gain texture from lees stirring and oak"]</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
+          <t>["all Chile is warm Central Valley","herbaceous always means Loire","lees texture means Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>["Ask if the fruit is Chile-ripe rather than Marlborough-pungent.","Use coastal valley names after reveal."]</t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>["pale lemon","ripe apple","citrus","tropical fruit","herbaceous notes","dry","high acidity","medium body","medium alcohol","ripe apple","citrus","tropical fruit","fresh high-acid palate","riper apple and tropical fruit than Sancerre","less benchmark elderflower/passionfruit than Marlborough","cool coastal Chile context"]</t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI47" t="inlineStr">
+        <is>
+          <t>Profile uses WSET White varieties evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ47" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Chile - Practica 046</t>
+        </is>
+      </c>
+      <c r="AK47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL47" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN47" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO47" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP47" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected New World white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ47" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium to pronounced intensity","ripe apple","citrus","tropical fruit","herbaceous notes"],"palate":["dry","high acidity","medium body","medium alcohol","ripe apple","citrus","tropical fruit"],"quality":["very good; excellent examples from cooler coastal valleys"],"ageing":["drink young to short ageing"],"diagnostic_features":["chile_coastal_sauvignon_core","cool_climate_high_acid_white","riper apple and tropical fruit than Sancerre","less benchmark elderflower/passionfruit than Marlborough"]}</t>
+        </is>
+      </c>
+      <c r="AR47" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["coastal Chile freshness","Sauvignon Blanc fruit spectrum","lees/oak texture option"],"learning_objectives":["identify Chilean Sauvignon Blanc","separate Chile from New Zealand Sauvignon","connect cool coastal valleys to acidity"],"typical_misconceptions":["all Chile is warm Central Valley","herbaceous always means Loire","lees texture means Chardonnay"],"mentor_focus":["ask for ripe apple/citrus/tropical plus high acidity"],"exam_traps":["calling it Marlborough automatically","missing Casablanca/San Antonio"],"memory_hooks":["Chile coastal Sauvignon is ripe-fruited and high-acid"],"comparison_styles":["Marlborough Sauvignon Blanc","Sancerre","Rueda Verdejo"]}</t>
+        </is>
+      </c>
+      <c r="AS47" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_051","SAT_WINE_009"],"frequently_confused_with":["SAT_WINE_051","SAT_WINE_038"],"distinguishing_features":["riper apple and tropical fruit than Sancerre","less benchmark elderflower/passionfruit than Marlborough","cool coastal Chile context"]}</t>
+        </is>
+      </c>
+      <c r="AT47" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Sauvignon Blanc performs well in Casablanca and San Antonio","wines have high acidity and intense fruity flavours","some examples gain texture from lees stirring and oak"],"mentor_hints":["Ask if the fruit is Chile-ripe rather than Marlborough-pungent.","Use coastal valley names after reveal."],"student_traps":["defaulting all Sauvignon to Marlborough","ignoring lees/oak texture"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU47" t="inlineStr">
+        <is>
+          <t>["chile_coastal_sauvignon_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV47" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW47" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["14584-14599"],"line_reference":["14584-14599"],"evidence":["Chile's white plantings are dominated by Sauvignon Blanc and Chardonnay.","Sauvignon Blanc performs particularly well in cooler Casablanca and San Antonio Valleys, giving high acidity, intense fruity flavours, ripe apple, citrus, tropical fruit and sometimes herbaceous notes."]}</t>
+        </is>
+      </c>
+      <c r="AX47" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-09-BATCH-006","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY47" t="inlineStr">
+        <is>
+          <t>36 Chile</t>
+        </is>
+      </c>
+      <c r="AZ47" t="inlineStr">
+        <is>
+          <t>White varieties</t>
+        </is>
+      </c>
+      <c r="BA47" t="inlineStr">
+        <is>
+          <t>153</t>
+        </is>
+      </c>
+      <c r="BB47" t="inlineStr">
+        <is>
+          <t>["14584-14599"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SAT_WINE_047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Blancos Nuevo Mundo</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Salta Torrontes</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>High-altitude aromatic Argentine Torrontes</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Salta Torrontes</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Salta</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Cafayate</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Salta / Cafayate GI</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>["Torrontes"]</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>high-altitude arid Argentine vineyards near Cafayate</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>very high-altitude vineyards close to Cafayate in Salta Province</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>not specified by WSET; altitude is the key quality driver</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>["many best Torrontes examples come from high-altitude Cafayate","aromatic variety harvested for freshness","released in the year of harvest"]</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>["inert temperature-controlled fermentation","early release","aroma preservation is central"]</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>unoaked</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>["floral perfume","stone fruit","melon","grape blossom"]</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>["stone fruit","melon","floral dry palate"]</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>good to very good; best high-altitude examples are concentrated and pure</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>drink young</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium to pronounced intensity","floral perfume","stone fruit","melon","grape blossom","dry","medium acidity","medium body","medium alcohol","stone fruit","melon","floral dry palate"]</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>["Torrontes is Argentina's white signature variety","best examples come from high-altitude Cafayate","wines are aromatic and usually fermented in inert vessels"]</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>["Argentina is only Malbec","floral dry whites must be Muscat","Torrontes is sweet by default"]</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>["Ask whether aroma is floral but palate is dry and medium-acid.","Use altitude to explain purity."]</t>
+        </is>
+      </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>["pale lemon","floral perfume","stone fruit","melon","grape blossom","dry","medium acidity","medium body","medium alcohol","stone fruit","melon","floral dry palate","more stone fruit and melon than Muscat","medium acidity rather than Assyrtiko high acidity","Salta altitude context"]</t>
+        </is>
+      </c>
+      <c r="AH48" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI48" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Torrontes / Salta evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ48" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Argentina - Practica 047</t>
+        </is>
+      </c>
+      <c r="AK48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL48" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO48" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP48" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected New World white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ48" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium to pronounced intensity","floral perfume","stone fruit","melon","grape blossom"],"palate":["dry","medium acidity","medium body","medium alcohol","stone fruit","melon","floral dry palate"],"quality":["good to very good; best high-altitude examples are concentrated and pure"],"ageing":["drink young"],"diagnostic_features":["argentina_torrontes_core","white_wine_sat_core","more stone fruit and melon than Muscat","medium acidity rather than Assyrtiko high acidity"]}</t>
+        </is>
+      </c>
+      <c r="AR48" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Argentina white signature","high-altitude aromatic freshness","inert winemaking"],"learning_objectives":["identify Torrontes aromatics","connect Salta altitude to purity","avoid confusing perfume with Muscat"],"typical_misconceptions":["Argentina is only Malbec","floral dry whites must be Muscat","Torrontes is sweet by default"],"mentor_focus":["ask for floral perfume with medium acidity"],"exam_traps":["calling it Gewurztraminer","assuming sweetness from perfume"],"memory_hooks":["Torrontes is Argentina's floral high-altitude white"],"comparison_styles":["Muscat d'Alsace","Frascati","Santorini Assyrtiko"]}</t>
+        </is>
+      </c>
+      <c r="AS48" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_011","SAT_WINE_034"],"frequently_confused_with":["SAT_WINE_011","SAT_WINE_043"],"distinguishing_features":["more stone fruit and melon than Muscat","medium acidity rather than Assyrtiko high acidity","Salta altitude context"]}</t>
+        </is>
+      </c>
+      <c r="AT48" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Torrontes is Argentina's white signature variety","best examples come from high-altitude Cafayate","wines are aromatic and usually fermented in inert vessels"],"mentor_hints":["Ask whether aroma is floral but palate is dry and medium-acid.","Use altitude to explain purity."],"student_traps":["assuming aromatic means sweet","forgetting Argentina whites"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU48" t="inlineStr">
+        <is>
+          <t>["argentina_torrontes_core","white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV48" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW48" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["15081-15097","15124-15135"],"line_reference":["15081-15097","15124-15135"],"evidence":["Torrontes is Argentina's white signature variety and many best examples come from high-altitude vineyards in Cafayate, Salta.","It has intense fruity floral perfume, medium body and acidity, stone fruit and melon, usually fermented in inert temperature-controlled vessels and released young."]}</t>
+        </is>
+      </c>
+      <c r="AX48" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-09-BATCH-006","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY48" t="inlineStr">
+        <is>
+          <t>37 Argentina</t>
+        </is>
+      </c>
+      <c r="AZ48" t="inlineStr">
+        <is>
+          <t>Torrontes / Salta</t>
+        </is>
+      </c>
+      <c r="BA48" t="inlineStr">
+        <is>
+          <t>157-158</t>
+        </is>
+      </c>
+      <c r="BB48" t="inlineStr">
+        <is>
+          <t>["15081-15097","15124-15135"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SAT_WINE_048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Blancos Nuevo Mundo</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>South Africa Chenin Blanc</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>South African Chenin Blanc from easy stone fruit to old-vine textured styles</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>South Africa Chenin Blanc</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Western Cape / Swartland</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Cape wine regions</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Western Cape WO / Swartland WO</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>["Chenin Blanc"]</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>warm South African climate moderated in cooler sites; old bush vines and dry farming can concentrate fruit</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>old bush-vine sites, especially Swartland, may be dry-farmed</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>not specified by WSET; old vines and dry farming are key markers</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>["Chenin Blanc is South Africa's most widely planted variety","old bush vines give concentration and complexity","Swartland is recognized for old vine Chenin"]</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>["dry and sweet styles possible","basic wines are easy-drinking stone fruit","barrel fermentation and ageing can add body and toasty oak"]</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>variable; premium wines may use barrel fermentation and ageing</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>medium lemon</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>["stone fruit","apple","honey","toasty oak"]</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>["stone fruit","apple","textured palate","toasty oak in premium examples"]</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>good to outstanding; old bush-vine examples can be concentrated and complex</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>medium ageing for concentrated examples</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>["medium lemon","medium to pronounced intensity","stone fruit","apple","honey","toasty oak","dry","medium to high acidity","medium to full body","medium alcohol","stone fruit","apple","textured palate","toasty oak in premium examples"]</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>["Chenin Blanc is South Africa's most widely planted variety","old bush vines can give concentration and complexity","barrel fermentation and ageing can add body and toasty oak"]</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>["South Africa is only Sauvignon or red blends","Chenin is always simple","oak texture means Chardonnay"]</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>["Ask whether acidity and texture fit Chenin rather than Chardonnay.","Use old vines as a quality explanation."]</t>
+        </is>
+      </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>["medium lemon","stone fruit","apple","honey","toasty oak","dry","medium to high acidity","medium to full body","medium alcohol","stone fruit","apple","textured palate","toasty oak in premium examples","more New World stone fruit than Loire Chenin","less varietal Chardonnay oak signature","old bush-vine South Africa context"]</t>
+        </is>
+      </c>
+      <c r="AH49" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI49" t="inlineStr">
+        <is>
+          <t>Profile uses WSET White varieties / Swartland evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ49" t="inlineStr">
+        <is>
+          <t>Vino Blanco - South Africa - Practica 048</t>
+        </is>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL49" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM49" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO49" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP49" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected New World white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ49" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium lemon"],"nose":["medium to pronounced intensity","stone fruit","apple","honey","toasty oak"],"palate":["dry","medium to high acidity","medium to full body","medium alcohol","stone fruit","apple","textured palate"],"quality":["good to outstanding; old bush-vine examples can be concentrated and complex"],"ageing":["medium ageing for concentrated examples"],"diagnostic_features":["south_africa_chenin_core","white_wine_sat_core","more New World stone fruit than Loire Chenin","less varietal Chardonnay oak signature"]}</t>
+        </is>
+      </c>
+      <c r="AR49" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["South African Chenin identity","old bush-vine concentration","barrel texture option"],"learning_objectives":["identify South African Chenin","separate Chenin from Chardonnay","connect old vines to concentration"],"typical_misconceptions":["South Africa is only Sauvignon or red blends","Chenin is always simple","oak texture means Chardonnay"],"mentor_focus":["ask whether stone fruit and texture could be Chenin"],"exam_traps":["calling premium Chenin Chardonnay","ignoring old bush vine clue"],"memory_hooks":["South African Chenin moves from easy stone fruit to old-vine texture"],"comparison_styles":["Vouvray Chenin Blanc","Fiano di Avellino","California Chardonnay"]}</t>
+        </is>
+      </c>
+      <c r="AS49" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_007","SAT_WINE_036"],"frequently_confused_with":["SAT_WINE_044","SAT_WINE_007"],"distinguishing_features":["more New World stone fruit than Loire Chenin","less varietal Chardonnay oak signature","old bush-vine South Africa context"]}</t>
+        </is>
+      </c>
+      <c r="AT49" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Chenin Blanc is South Africa's most widely planted variety","old bush vines can give concentration and complexity","barrel fermentation and ageing can add body and toasty oak"],"mentor_hints":["Ask whether acidity and texture fit Chenin rather than Chardonnay.","Use old vines as a quality explanation."],"student_traps":["overlooking Chenin as South Africa core","confusing all barrel texture with Chardonnay"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU49" t="inlineStr">
+        <is>
+          <t>["south_africa_chenin_core","white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV49" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW49" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["15357-15367","15591-15604"],"line_reference":["15357-15367","15591-15604"],"evidence":["Chenin Blanc is South Africa's most widely planted variety and producers make great wines in sweet and dry styles.","Old bush vines can offer more concentrated complex flavours and fuller texture; Swartland is a source of old vine Chenin."]}</t>
+        </is>
+      </c>
+      <c r="AX49" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-09-BATCH-006","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY49" t="inlineStr">
+        <is>
+          <t>38 South Africa</t>
+        </is>
+      </c>
+      <c r="AZ49" t="inlineStr">
+        <is>
+          <t>White varieties / Swartland</t>
+        </is>
+      </c>
+      <c r="BA49" t="inlineStr">
+        <is>
+          <t>161-162</t>
+        </is>
+      </c>
+      <c r="BB49" t="inlineStr">
+        <is>
+          <t>["15357-15367","15591-15604"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SAT_WINE_049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Blancos Nuevo Mundo</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Hunter Valley Semillon</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Early-harvest unoaked Hunter Valley Semillon built for bottle age</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Hunter Valley Semillon</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Hunter Valley</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>New South Wales</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Hunter Valley GI</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>["Semillon"]</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>hot humid Hunter Valley climate</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>low-altitude Hunter Valley vineyards</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>not specified by WSET; early harvest and winemaking define style</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>["Semillon is the most planted Hunter Valley grape","harvested early at low sugar and high acidity","style is unique to Australia"]</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>["oxygen contact kept to a minimum","inert vessels for fermentation and storage","bottled young almost neutral then develops with age"]</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>unoaked</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>["lemon","grass","neutral young fruit","honey with age","toast with age"]</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>["lemon","neutral young palate","high-acid light body","honey and toast with age"]</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>long with age</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>very good to outstanding; best examples can age 20 years or more</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>very long ageing for best examples</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium to pronounced intensity","lemon","grass","neutral young fruit","honey with age","toast with age","dry","high acidity","light body","low alcohol","lemon","neutral young palate","high-acid light body","honey and toast with age"]</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>["Hunter Semillon is harvested early","oxygen is minimized and inert vessels are used","best examples develop honey and toast and can age 20 years or more"]</t>
+        </is>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>["toast always means oak","Hunter Valley is only Shiraz","neutral young wine means low quality"]</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>["Ask if toast could be bottle age rather than barrel.","Use low alcohol as a decisive clue."]</t>
+        </is>
+      </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>["pale lemon","lemon","grass","neutral young fruit","honey with age","toast with age","dry","high acidity","light body","low alcohol","lemon","neutral young palate","high-acid light body","honey and toast with age","lower alcohol than most Chardonnay","toast develops without oak","unique Hunter early-harvest Semillon style"]</t>
+        </is>
+      </c>
+      <c r="AH50" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI50" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Semillon / Hunter Valley evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ50" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Australia - Practica 049</t>
+        </is>
+      </c>
+      <c r="AK50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL50" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM50" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN50" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO50" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="AP50" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected New World white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ50" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium to pronounced intensity","lemon","grass","neutral young fruit","honey with age","toast with age"],"palate":["dry","high acidity","light body","low alcohol","lemon","neutral young palate","high-acid light body"],"quality":["very good to outstanding; best examples can age 20 years or more"],"ageing":["very long ageing for best examples"],"diagnostic_features":["hunter_semillon_core","cool_climate_high_acid_white","lower alcohol than most Chardonnay","toast develops without oak"]}</t>
+        </is>
+      </c>
+      <c r="AR50" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Australian unique Semillon","age transformation without oak","early harvest structure"],"learning_objectives":["identify Hunter Semillon","separate age-derived toast from oak","connect low alcohol and high acidity"],"typical_misconceptions":["toast always means oak","Hunter Valley is only Shiraz","neutral young wine means low quality"],"mentor_focus":["ask whether low alcohol and high acidity can explain longevity"],"exam_traps":["calling it oaked Chardonnay with age","missing Semillon despite neutrality"],"memory_hooks":["Hunter Semillon starts quiet and ages into honeyed toast"],"comparison_styles":["Australian Riesling","Muscadet","White Bordeaux"]}</t>
+        </is>
+      </c>
+      <c r="AS50" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_050","SAT_WINE_008"],"frequently_confused_with":["SAT_WINE_044","SAT_WINE_008"],"distinguishing_features":["lower alcohol than most Chardonnay","toast develops without oak","unique Hunter early-harvest Semillon style"]}</t>
+        </is>
+      </c>
+      <c r="AT50" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Hunter Semillon is harvested early","oxygen is minimized and inert vessels are used","best examples develop honey and toast and can age 20 years or more"],"mentor_hints":["Ask if toast could be bottle age rather than barrel.","Use low alcohol as a decisive clue."],"student_traps":["mistaking bottle-aged Semillon for oaked Chardonnay","undervaluing neutral young examples"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU50" t="inlineStr">
+        <is>
+          <t>["hunter_semillon_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV50" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW50" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["15916-15930","16306-16318"],"line_reference":["15916-15930","16306-16318"],"evidence":["Hunter Valley is the classic region for Australian Semillon, harvested early with low sugar and high acidity.","Inert vessels and minimal oxygen produce low-alcohol almost neutral young wines that develop honey and toast with bottle age; best can age 20 years or more."]}</t>
+        </is>
+      </c>
+      <c r="AX50" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-09-BATCH-006","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY50" t="inlineStr">
+        <is>
+          <t>39 Australia</t>
+        </is>
+      </c>
+      <c r="AZ50" t="inlineStr">
+        <is>
+          <t>Semillon / Hunter Valley</t>
+        </is>
+      </c>
+      <c r="BA50" t="inlineStr">
+        <is>
+          <t>165, 169</t>
+        </is>
+      </c>
+      <c r="BB50" t="inlineStr">
+        <is>
+          <t>["15916-15930","16306-16318"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SAT_WINE_050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Blancos Nuevo Mundo</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Clare Valley Riesling</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Dry high-acid lime-led Australian Riesling</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Clare Valley Riesling</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Clare Valley</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>South Australia</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Clare Valley GI</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>["Riesling"]</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>South Australian region suited to dry high-acid Riesling</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>elevated Clare Valley sites within South Australia</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>not specified by WSET; regional suitability and style are key</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>["Clare Valley is a classic Riesling region","Riesling is the regional speciality","dry high-acid style is central"]</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>["unoaked Riesling production","dry or slightly off-dry styles","bottle ageing develops toast, honey and petrol"]</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>unoaked</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>dry to slightly off-dry</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>["lime","lemon","grapefruit","petrol with age","honey with age"]</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>["lime","lemon","grapefruit","high-acid dry palate","toast and honey with age"]</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>very good to outstanding; classic Australian Riesling region</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>medium to long ageing</t>
+        </is>
+      </c>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium to pronounced intensity","lime","lemon","grapefruit","petrol with age","honey with age","dry to slightly off-dry","high acidity","light to medium body","medium alcohol","lime","lemon","grapefruit","high-acid dry palate","toast and honey with age"]</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>["Australian Riesling is unoaked and high acid","classic regions include Clare and Eden Valleys","Clare Valley Riesling is a speciality"]</t>
+        </is>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>["all Riesling is sweet","petrol is a fault","Australia only makes full-bodied whites"]</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>["Ask whether sweetness is assumed or observed.","Use lime intensity as the memory anchor."]</t>
+        </is>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>["pale lemon","lime","lemon","grapefruit","petrol with age","honey with age","dry to slightly off-dry","high acidity","light to medium body","medium alcohol","lime","lemon","grapefruit","high-acid dry palate","toast and honey with age","drier and more lime-driven than Kabinett","less full than Wachau dry Riesling","Australian regional identity"]</t>
+        </is>
+      </c>
+      <c r="AH51" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI51" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Riesling / Clare Valley evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ51" t="inlineStr">
+        <is>
+          <t>Vino Blanco - Australia - Practica 050</t>
+        </is>
+      </c>
+      <c r="AK51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN51" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO51" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP51" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected New World white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ51" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium to pronounced intensity","lime","lemon","grapefruit","petrol with age","honey with age"],"palate":["dry to slightly off-dry","high acidity","light to medium body","medium alcohol","lime","lemon","grapefruit"],"quality":["very good to outstanding; classic Australian Riesling region"],"ageing":["medium to long ageing"],"diagnostic_features":["australian_riesling_core","cool_climate_high_acid_white","drier and more lime-driven than Kabinett","less full than Wachau dry Riesling"]}</t>
+        </is>
+      </c>
+      <c r="AR51" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Australian dry Riesling","citrus intensity and age development","Clare regional identity"],"learning_objectives":["identify lime-led Australian Riesling","separate dry Riesling from German sweetness","connect petrol/toast to bottle age"],"typical_misconceptions":["all Riesling is sweet","petrol is a fault","Australia only makes full-bodied whites"],"mentor_focus":["ask for lime, dry palate and high acidity"],"exam_traps":["calling it German Kabinett","assuming petrol means old faulty wine"],"memory_hooks":["Clare Riesling is dry lime lightning with ageworthy petrol-honey"],"comparison_styles":["Eden Valley Riesling","Wachau Riesling","Riesling Kabinett"]}</t>
+        </is>
+      </c>
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_023","SAT_WINE_016"],"frequently_confused_with":["SAT_WINE_016","SAT_WINE_023"],"distinguishing_features":["drier and more lime-driven than Kabinett","less full than Wachau dry Riesling","Australian regional identity"]}</t>
+        </is>
+      </c>
+      <c r="AT51" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Australian Riesling is unoaked and high acid","classic regions include Clare and Eden Valleys","Clare Valley Riesling is a speciality"],"mentor_hints":["Ask whether sweetness is assumed or observed.","Use lime intensity as the memory anchor."],"student_traps":["defaulting to Germany","missing dry Australian Riesling"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU51" t="inlineStr">
+        <is>
+          <t>["australian_riesling_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV51" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW51" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["15932-15942","16000-16002"],"line_reference":["15932-15942","16000-16002"],"evidence":["Australian Riesling has lime, lemon and grapefruit in youth, developing toast, honey and petrol; it is unoaked, high acid and usually dry or slightly off-dry.","Classic regions include Eden and Clare Valleys; Riesling is the speciality of Clare Valley."]}</t>
+        </is>
+      </c>
+      <c r="AX51" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-09-BATCH-006","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY51" t="inlineStr">
+        <is>
+          <t>39 Australia</t>
+        </is>
+      </c>
+      <c r="AZ51" t="inlineStr">
+        <is>
+          <t>Riesling / Clare Valley</t>
+        </is>
+      </c>
+      <c r="BA51" t="inlineStr">
+        <is>
+          <t>165-166</t>
+        </is>
+      </c>
+      <c r="BB51" t="inlineStr">
+        <is>
+          <t>["15932-15942","16000-16002"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SAT_WINE_051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Blancos Nuevo Mundo</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Marlborough Sauvignon Blanc</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Pungent high-acid Marlborough Sauvignon Blanc</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Marlborough Sauvignon Blanc</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Marlborough</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>South Island</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Marlborough GI</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>["Sauvignon Blanc"]</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>sunny South Island climate with Wairau and Awatere valley contrasts; Awatere is drier, cooler and windier</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Wairau and Awatere estuary valleys with varied aspects and altitudes</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>not specified by WSET; valley and climate differences are key</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>["Sauvignon Blanc makes up the majority of Marlborough plantings","Wairau can show tropical fruit","Awatere gives higher acidity and herbaceous character"]</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>["cool inert fermentation preserves fruity aromas","some producers make oak-matured styles","benchmark aromatic Sauvignon style"]</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>usually unoaked; some oak-matured styles exist</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>["elderflower","passion fruit","green bell pepper","gooseberry","citrus"]</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>["passion fruit","gooseberry","green bell pepper","high-acid dry palate"]</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>very good to outstanding; global benchmark for Sauvignon Blanc</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr">
+        <is>
+          <t>drink young to short ageing; oak-matured styles may hold longer</t>
+        </is>
+      </c>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>["pale lemon","medium to pronounced intensity","elderflower","passion fruit","green bell pepper","gooseberry","citrus","dry","high acidity","medium body","medium alcohol","passion fruit","gooseberry","green bell pepper","high-acid dry palate"]</t>
+        </is>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>["Sauvignon Blanc is New Zealand's flagship grape","Marlborough is the major centre and Sauvignon Blanc majority planting","Awatere Sauvignon has higher acidity and herbaceous character"]</t>
+        </is>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>["all Sauvignon Blanc is Loire","Marlborough always only passion fruit","oak-matured Sauvignon is impossible"]</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>["Ask if the aromatic intensity is truly pungent Sauvignon.","Use Wairau/Awatere contrast in debrief."]</t>
+        </is>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>["pale lemon","elderflower","passion fruit","green bell pepper","gooseberry","citrus","dry","high acidity","medium body","medium alcohol","passion fruit","gooseberry","green bell pepper","high-acid dry palate","more pungent elderflower/passion fruit than Chile","more gooseberry and bell pepper than Rueda","global benchmark Sauvignon profile"]</t>
+        </is>
+      </c>
+      <c r="AH52" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI52" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Sauvignon Blanc / Marlborough evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ52" t="inlineStr">
+        <is>
+          <t>Vino Blanco - New Zealand - Practica 051</t>
+        </is>
+      </c>
+      <c r="AK52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL52" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN52" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO52" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="AP52" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected New World white profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ52" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon"],"nose":["medium to pronounced intensity","elderflower","passion fruit","green bell pepper","gooseberry","citrus"],"palate":["dry","high acidity","medium body","medium alcohol","passion fruit","gooseberry","green bell pepper"],"quality":["very good to outstanding; global benchmark for Sauvignon Blanc"],"ageing":["drink young to short ageing; oak-matured styles may hold longer"],"diagnostic_features":["marlborough_sauvignon_core","cool_climate_high_acid_white","more pungent elderflower/passion fruit than Chile","more gooseberry and bell pepper than Rueda"]}</t>
+        </is>
+      </c>
+      <c r="AR52" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["New Zealand benchmark Sauvignon","Marlborough valley contrast","cool inert fermentation"],"learning_objectives":["identify Marlborough Sauvignon Blanc","separate Wairau tropical and Awatere herbaceous styles","contrast with Chile Sauvignon"],"typical_misconceptions":["all Sauvignon Blanc is Loire","Marlborough always only passion fruit","oak-matured Sauvignon is impossible"],"mentor_focus":["ask for pungent aromatics and high acidity"],"exam_traps":["calling every aromatic high-acid white Marlborough","missing Awatere herbaceous profile"],"memory_hooks":["Marlborough Sauvignon is elderflower, passionfruit, gooseberry and acid"],"comparison_styles":["Chile Coastal Sauvignon Blanc","Sancerre","Rueda Verdejo"]}</t>
+        </is>
+      </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_046","SAT_WINE_009"],"frequently_confused_with":["SAT_WINE_046","SAT_WINE_038"],"distinguishing_features":["more pungent elderflower/passion fruit than Chile","more gooseberry and bell pepper than Rueda","global benchmark Sauvignon profile"]}</t>
+        </is>
+      </c>
+      <c r="AT52" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Sauvignon Blanc is New Zealand's flagship grape","Marlborough is the major centre and Sauvignon Blanc majority planting","Awatere Sauvignon has higher acidity and herbaceous character"],"mentor_hints":["Ask if the aromatic intensity is truly pungent Sauvignon.","Use Wairau/Awatere contrast in debrief."],"student_traps":["overusing Marlborough as a default answer","ignoring Chile as a comparator"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU52" t="inlineStr">
+        <is>
+          <t>["marlborough_sauvignon_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV52" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW52" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["16454-16467","16576-16598"],"line_reference":["16454-16467","16576-16598"],"evidence":["New Zealand Sauvignon Blanc is the flagship grape with elderflower, passion fruit and high acidity, often fermented cool in inert vessels.","Marlborough is the major grape-growing centre; Sauvignon Blanc is the majority, with Awatere examples higher in acidity and herbaceous character."]}</t>
+        </is>
+      </c>
+      <c r="AX52" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-09-BATCH-006","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY52" t="inlineStr">
+        <is>
+          <t>40 New Zealand</t>
+        </is>
+      </c>
+      <c r="AZ52" t="inlineStr">
+        <is>
+          <t>Sauvignon Blanc / Marlborough</t>
+        </is>
+      </c>
+      <c r="BA52" t="inlineStr">
+        <is>
+          <t>170-172</t>
+        </is>
+      </c>
+      <c r="BB52" t="inlineStr">
+        <is>
+          <t>["16454-16467","16576-16598"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add Batch 007 France red profiles
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -14154,6 +14154,1638 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SAT_WINE_052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Tintos Francia</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Left Bank Bordeaux</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Cabernet Sauvignon-dominant structured Bordeaux from Médoc and Graves</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Left Bank Bordeaux</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Bordeaux</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Médoc / Graves</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Haut-Médoc / Pauillac / Margaux / Pessac-Léognan</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>["Cabernet Sauvignon","Merlot","Cabernet Franc"]</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>moderate maritime climate with vintage variation</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>gravelly Left Bank sites including Haut-Médoc and Graves</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>gravel soils suited to Cabernet Sauvignon</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>["Cabernet Sauvignon dominates in Haut-Médoc","gravel soils aid drainage and warmth","top châteaux use careful vineyard selection"]</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>["top-quality red Bordeaux aged in small oak casks","blending balances ripening differences","long-term wines often use traditional fermentation and extraction"]</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>small oak casks, often with new oak in top wines</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>deep ruby</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>["blackcurrant","black cherry","cedar","vanilla","tobacco"]</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>["black fruit","cedar","firm tannin","oak spice"]</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>very good to outstanding; top communes have high reputation</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>["deep ruby","medium to pronounced intensity","blackcurrant","black cherry","cedar","vanilla","tobacco","dry","medium to high acidity","medium to full body","medium to high alcohol","medium to high tannin","black fruit","cedar","firm tannin","oak spice"]</t>
+        </is>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>["Cabernet Sauvignon dominates in Haut-Médoc","top-quality red Bordeaux is aged in small oak casks","Left Bank includes Médoc, Graves and Sauternes"]</t>
+        </is>
+      </c>
+      <c r="AE53" t="inlineStr">
+        <is>
+          <t>["all Bordeaux is Merlot-dominant","oak spice means Rioja","high tannin always means Italy"]</t>
+        </is>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>["Ask what points to Cabernet rather than Merlot.","Use bank geography only after commitment."]</t>
+        </is>
+      </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>["deep ruby","blackcurrant","black cherry","cedar","vanilla","tobacco","dry","medium to high acidity","medium to full body","medium to high alcohol","medium to high tannin","black fruit","cedar","firm tannin","oak spice","more Cabernet structure than Right Bank","firmer tannin than Merlot-led styles","gravel Left Bank source"]</t>
+        </is>
+      </c>
+      <c r="AH53" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI53" t="inlineStr">
+        <is>
+          <t>Profile uses WSET The Reds of Médoc and Graves evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ53" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Francia - Practica 052</t>
+        </is>
+      </c>
+      <c r="AK53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL53" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM53" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN53" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO53" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP53" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected French red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ53" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby"],"nose":["medium to pronounced intensity","blackcurrant","black cherry","cedar","vanilla","tobacco"],"palate":["dry","medium to high acidity","medium to full body","medium to high alcohol","medium to high tannin","black fruit","cedar","firm tannin"],"quality":["very good to outstanding; top communes have high reputation"],"ageing":["long ageing potential"],"diagnostic_features":["left_bank_bordeaux_core","more Cabernet structure than Right Bank","firmer tannin than Merlot-led styles"]}</t>
+        </is>
+      </c>
+      <c r="AR53" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Cabernet-led Bordeaux structure","Left Bank gravel and tannin","oak-aged ageworthy claret"],"learning_objectives":["identify Cabernet-led Bordeaux","connect gravel soils to Cabernet Sauvignon","separate Left Bank from Right Bank"],"typical_misconceptions":["all Bordeaux is Merlot-dominant","oak spice means Rioja","high tannin always means Italy"],"mentor_focus":["ask whether tannin, black fruit and cedar point to Cabernet-led Bordeaux"],"exam_traps":["confusing Left and Right Bank","missing oak ageing role"],"memory_hooks":["Left Bank is Cabernet on gravel: black fruit, cedar, tannin"],"comparison_styles":["Right Bank Bordeaux","Rioja Reserva","Napa Cabernet"]}</t>
+        </is>
+      </c>
+      <c r="AS53" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_053"],"frequently_confused_with":["SAT_WINE_053"],"distinguishing_features":["more Cabernet structure than Right Bank","firmer tannin than Merlot-led styles","gravel Left Bank source"]}</t>
+        </is>
+      </c>
+      <c r="AT53" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Cabernet Sauvignon dominates in Haut-Médoc","top-quality red Bordeaux is aged in small oak casks","Left Bank includes Médoc, Graves and Sauternes"],"mentor_hints":["Ask what points to Cabernet rather than Merlot.","Use bank geography only after commitment."],"student_traps":["mixing up Left and Right Bank","overcalling new oak"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU53" t="inlineStr">
+        <is>
+          <t>["left_bank_bordeaux_core"]</t>
+        </is>
+      </c>
+      <c r="AV53" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW53" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["7766-7880","8077-8106"],"line_reference":["7766-7880","8077-8106"],"evidence":["Cabernet Sauvignon dominates in the Haut-Médoc and top-quality red Bordeaux is aged in small oak casks.","The highest reputation Left Bank communes include Saint-Estèphe, Pauillac, Saint-Julien and Margaux; Pessac-Léognan has gravelly soils suited to Cabernet Sauvignon."]}</t>
+        </is>
+      </c>
+      <c r="AX53" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-10-BATCH-007","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY53" t="inlineStr">
+        <is>
+          <t>13 Bordeaux</t>
+        </is>
+      </c>
+      <c r="AZ53" t="inlineStr">
+        <is>
+          <t>The Reds of Médoc and Graves</t>
+        </is>
+      </c>
+      <c r="BA53" t="inlineStr">
+        <is>
+          <t>78-80</t>
+        </is>
+      </c>
+      <c r="BB53" t="inlineStr">
+        <is>
+          <t>["7766-7880","8077-8106"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SAT_WINE_053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Tintos Francia</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Right Bank Bordeaux</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Merlot-dominant Saint-Émilion and Pomerol red Bordeaux</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Right Bank Bordeaux</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Bordeaux</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Saint-Émilion / Pomerol</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Saint-Émilion Grand Cru / Pomerol</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>["Merlot","Cabernet Franc","Cabernet Sauvignon"]</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>moderate maritime Bordeaux climate with Right Bank ripening differences</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>plateau and slope sites in Saint-Émilion and Pomerol</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>warm well-drained gravel, clay and limestone sites</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>["Merlot is most important in Saint-Émilion and Pomerol","Cabernet Franc is widely used in Saint-Émilion","best sites differ by drainage and warmth"]</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>["blended red Bordeaux production","small oak cask ageing for top wines","Merlot-led wines can be richer and spicier"]</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>small oak casks in top wines</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>deep ruby</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>["plum","black cherry","spice","cedar","chocolate"]</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>["plum","black cherry","spice","rounded tannin"]</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>very good to outstanding; Pomerol and Saint-Émilion have high reputation</t>
+        </is>
+      </c>
+      <c r="AB54" t="inlineStr">
+        <is>
+          <t>medium to long ageing</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>["deep ruby","medium to pronounced intensity","plum","black cherry","spice","cedar","chocolate","dry","medium acidity","medium to full body","medium to high alcohol","medium to high tannin","plum","black cherry","spice","rounded tannin"]</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>["Merlot is key in Saint-Émilion and Pomerol","Cabernet Franc is widely used in Saint-Émilion","Pomerol wines tend to be richer and spicier"]</t>
+        </is>
+      </c>
+      <c r="AE54" t="inlineStr">
+        <is>
+          <t>["all Bordeaux tastes like Cabernet","Pomerol is a classification not place","Merlot lacks ageing potential"]</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>["Ask if structure is firm Cabernet or plush Merlot.","Use Saint-Émilion/Pomerol as debrief anchors."]</t>
+        </is>
+      </c>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>["deep ruby","plum","black cherry","spice","cedar","chocolate","dry","medium acidity","medium to full body","medium to high alcohol","medium to high tannin","plum","black cherry","spice","rounded tannin","plummier and rounder than Left Bank","more Merlot and Cabernet Franc emphasis","Right Bank Saint-Émilion/Pomerol source"]</t>
+        </is>
+      </c>
+      <c r="AH54" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI54" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Saint-Émilion and Pomerol evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ54" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Francia - Practica 053</t>
+        </is>
+      </c>
+      <c r="AK54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL54" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN54" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO54" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP54" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected French red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ54" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby"],"nose":["medium to pronounced intensity","plum","black cherry","spice","cedar","chocolate"],"palate":["dry","medium acidity","medium to full body","medium to high alcohol","medium to high tannin","plum","black cherry","spice"],"quality":["very good to outstanding; Pomerol and Saint-Émilion have high reputation"],"ageing":["medium to long ageing"],"diagnostic_features":["right_bank_bordeaux_core","plummier and rounder than Left Bank","more Merlot and Cabernet Franc emphasis"]}</t>
+        </is>
+      </c>
+      <c r="AR54" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Merlot-led Bordeaux","Right Bank appellation logic","Cabernet Franc support"],"learning_objectives":["identify Merlot-dominant Bordeaux","distinguish Right Bank from Left Bank","connect Pomerol richness to style"],"typical_misconceptions":["all Bordeaux tastes like Cabernet","Pomerol is a classification not place","Merlot lacks ageing potential"],"mentor_focus":["ask whether tannins are rounder and fruit is plummy"],"exam_traps":["calling Right Bank Left Bank from Bordeaux label alone","missing Cabernet Franc"],"memory_hooks":["Right Bank is Merlot generosity with Bordeaux structure"],"comparison_styles":["Left Bank Bordeaux","Pomerol","Saint-Émilion"]}</t>
+        </is>
+      </c>
+      <c r="AS54" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_052"],"frequently_confused_with":["SAT_WINE_052"],"distinguishing_features":["plummier and rounder than Left Bank","more Merlot and Cabernet Franc emphasis","Right Bank Saint-Émilion/Pomerol source"]}</t>
+        </is>
+      </c>
+      <c r="AT54" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Merlot is key in Saint-Émilion and Pomerol","Cabernet Franc is widely used in Saint-Émilion","Pomerol wines tend to be richer and spicier"],"mentor_hints":["Ask if structure is firm Cabernet or plush Merlot.","Use Saint-Émilion/Pomerol as debrief anchors."],"student_traps":["assuming all Bordeaux is Cabernet","forgetting Cabernet Franc"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU54" t="inlineStr">
+        <is>
+          <t>["right_bank_bordeaux_core"]</t>
+        </is>
+      </c>
+      <c r="AV54" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW54" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["7815-7836","8112-8143"],"line_reference":["7815-7836","8112-8143"],"evidence":["Merlot is most widely planted in Bordeaux and is particularly important in Saint-Émilion and Pomerol; Cabernet Franc is widely used in Saint-Émilion.","Pomerol wines tend to be richer, spicier and fuller-bodied."]}</t>
+        </is>
+      </c>
+      <c r="AX54" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-10-BATCH-007","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY54" t="inlineStr">
+        <is>
+          <t>13 Bordeaux</t>
+        </is>
+      </c>
+      <c r="AZ54" t="inlineStr">
+        <is>
+          <t>Saint-Émilion and Pomerol</t>
+        </is>
+      </c>
+      <c r="BA54" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="BB54" t="inlineStr">
+        <is>
+          <t>["7815-7836","8112-8143"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SAT_WINE_054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Tintos Francia</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Cote d'Or Red Burgundy</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Côte d'Or Pinot Noir with red fruit, site expression and moderate structure</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Cote d'Or Red Burgundy</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Burgundy</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Côte d'Or</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Village / Premier Cru / Grand Cru Côte d'Or</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>["Pinot Noir"]</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>cool to moderate continental Burgundy climate</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>east and south-east facing limestone slopes in the Côte d'Or</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>varied limestone-rich Burgundy soils</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>["Pinot Noir is the important black grape in Côte d'Or","site hierarchy drives quality","best vineyards have favourable aspect and drainage"]</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>["red Burgundy may use oak maturation","extraction must respect Pinot Noir structure","quality depends strongly on site and producer"]</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>often old or new oak depending on producer and level</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>low to medium</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>pale to medium ruby</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>["red cherry","raspberry","violet","earth","sweet spice"]</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>["red cherry","raspberry","earth","fine tannin"]</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>very good to outstanding at higher site levels</t>
+        </is>
+      </c>
+      <c r="AB55" t="inlineStr">
+        <is>
+          <t>medium to long ageing for best sites</t>
+        </is>
+      </c>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>["pale to medium ruby","medium to pronounced intensity","red cherry","raspberry","violet","earth","sweet spice","dry","medium to high acidity","medium body","medium alcohol","low to medium tannin","red cherry","raspberry","earth","fine tannin"]</t>
+        </is>
+      </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>["Burgundy is the home of Pinot Noir","Côte d'Or is the heartland of Burgundy","appellation hierarchy is based on quality"]</t>
+        </is>
+      </c>
+      <c r="AE55" t="inlineStr">
+        <is>
+          <t>["all pale red wine is simple","Burgundy is only Chardonnay","low tannin means low quality"]</t>
+        </is>
+      </c>
+      <c r="AF55" t="inlineStr">
+        <is>
+          <t>["Ask whether pale colour is Pinot or Gamay.","Use hierarchy as quality reasoning."]</t>
+        </is>
+      </c>
+      <c r="AG55" t="inlineStr">
+        <is>
+          <t>["pale to medium ruby","red cherry","raspberry","violet","earth","sweet spice","dry","medium to high acidity","medium body","medium alcohol","low to medium tannin","red cherry","raspberry","earth","fine tannin","more tannic and complex than Beaujolais","Pinot Noir rather than Gamay","earth and site hierarchy are central"]</t>
+        </is>
+      </c>
+      <c r="AH55" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI55" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Côte d'Or / Burgundy appellation hierarchy evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ55" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Francia - Practica 054</t>
+        </is>
+      </c>
+      <c r="AK55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL55" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM55" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN55" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO55" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP55" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected French red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ55" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium ruby"],"nose":["medium to pronounced intensity","red cherry","raspberry","violet","earth","sweet spice"],"palate":["dry","medium to high acidity","medium body","medium alcohol","low to medium tannin","red cherry","raspberry","earth"],"quality":["very good to outstanding at higher site levels"],"ageing":["medium to long ageing for best sites"],"diagnostic_features":["red_burgundy_pinot_core","more tannic and complex than Beaujolais","Pinot Noir rather than Gamay"]}</t>
+        </is>
+      </c>
+      <c r="AR55" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Pinot Noir site expression","Burgundy hierarchy","Côte d'Or red-fruit structure"],"learning_objectives":["identify red Burgundy structure","connect appellation hierarchy to quality","separate Pinot Noir from Gamay"],"typical_misconceptions":["all pale red wine is simple","Burgundy is only Chardonnay","low tannin means low quality"],"mentor_focus":["ask for red fruit, fine tannin and site-derived complexity"],"exam_traps":["calling Burgundy Beaujolais from pale colour","overstating tannin"],"memory_hooks":["Côte d'Or Pinot is red fruit plus place precision"],"comparison_styles":["Beaujolais Villages / Cru","Sonoma Pinot Noir","Loire Cabernet Franc"]}</t>
+        </is>
+      </c>
+      <c r="AS55" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_055"],"frequently_confused_with":["SAT_WINE_055"],"distinguishing_features":["more tannic and complex than Beaujolais","Pinot Noir rather than Gamay","earth and site hierarchy are central"]}</t>
+        </is>
+      </c>
+      <c r="AT55" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Burgundy is the home of Pinot Noir","Côte d'Or is the heartland of Burgundy","appellation hierarchy is based on quality"],"mentor_hints":["Ask whether pale colour is Pinot or Gamay.","Use hierarchy as quality reasoning."],"student_traps":["equating pale colour with low quality","forgetting village hierarchy"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU55" t="inlineStr">
+        <is>
+          <t>["red_burgundy_pinot_core"]</t>
+        </is>
+      </c>
+      <c r="AV55" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW55" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["8354-8450","8563-8674"],"line_reference":["8354-8450","8563-8674"],"evidence":["Burgundy is the home of Pinot Noir and Chardonnay; most important plantings are in the Côte d'Or.","The vineyards of the Côte d'Or form the heartland of Burgundy and appellations form a hierarchy based on quality."]}</t>
+        </is>
+      </c>
+      <c r="AX55" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-10-BATCH-007","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY55" t="inlineStr">
+        <is>
+          <t>15 Burgundy</t>
+        </is>
+      </c>
+      <c r="AZ55" t="inlineStr">
+        <is>
+          <t>Côte d'Or / Burgundy appellation hierarchy</t>
+        </is>
+      </c>
+      <c r="BA55" t="inlineStr">
+        <is>
+          <t>85-88</t>
+        </is>
+      </c>
+      <c r="BB55" t="inlineStr">
+        <is>
+          <t>["8354-8450","8563-8674"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SAT_WINE_055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Tintos Francia</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Beaujolais Villages / Cru</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Gamay-based Beaujolais from fruity Villages to more concentrated crus</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Beaujolais Villages / Cru</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Beaujolais</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Beaujolais Villages / Crus</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Beaujolais Villages / Beaujolais Cru</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>["Gamay"]</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>moderate continental climate south of Burgundy</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>hilly northern Beaujolais for villages and crus</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>not specified by WSET here; granite soils are standard regional knowledge for crus</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>["production is overwhelmingly red","Gamay gives fragrant raspberry wines","cru villages sit at top of hierarchy"]</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>["whole-bunch or semi-carbonic methods common in fruity styles","crus may use more traditional fermentation","made for fruit purity and early drinkability to medium ageing"]</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>usually little new oak; large or neutral vessels may be used</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>pale to medium ruby</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>["raspberry","red cherry","banana","violet","pepper"]</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>["raspberry","red cherry","juicy fruit","low tannin"]</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>good to very good; crus can be more concentrated</t>
+        </is>
+      </c>
+      <c r="AB56" t="inlineStr">
+        <is>
+          <t>drink young to medium ageing for crus</t>
+        </is>
+      </c>
+      <c r="AC56" t="inlineStr">
+        <is>
+          <t>["pale to medium ruby","medium to pronounced intensity","raspberry","red cherry","banana","violet","pepper","dry","medium to high acidity","light to medium body","medium alcohol","low tannin","raspberry","red cherry","juicy fruit","low tannin"]</t>
+        </is>
+      </c>
+      <c r="AD56" t="inlineStr">
+        <is>
+          <t>["Gamay gives fragrant raspberry wines","Beaujolais hierarchy culminates in crus","Beaujolais and Nouveau are light-bodied and fruity"]</t>
+        </is>
+      </c>
+      <c r="AE56" t="inlineStr">
+        <is>
+          <t>["Beaujolais is only Nouveau","banana is required in every Gamay","low tannin means poor quality"]</t>
+        </is>
+      </c>
+      <c r="AF56" t="inlineStr">
+        <is>
+          <t>["Ask if tannin level supports Gamay.","Use hierarchy to avoid dismissing crus."]</t>
+        </is>
+      </c>
+      <c r="AG56" t="inlineStr">
+        <is>
+          <t>["pale to medium ruby","raspberry","red cherry","banana","violet","pepper","dry","medium to high acidity","light to medium body","medium alcohol","low tannin","raspberry","red cherry","juicy fruit","low tannin","fruitier and lower tannin than red Burgundy","Gamay rather than Pinot Noir","cru hierarchy gives concentration"]</t>
+        </is>
+      </c>
+      <c r="AH56" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI56" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Beaujolais Villages and Crus evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ56" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Francia - Practica 055</t>
+        </is>
+      </c>
+      <c r="AK56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL56" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM56" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN56" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO56" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP56" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected French red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ56" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium ruby"],"nose":["medium to pronounced intensity","raspberry","red cherry","banana","violet","pepper"],"palate":["dry","medium to high acidity","light to medium body","medium alcohol","low tannin","raspberry","red cherry","juicy fruit"],"quality":["good to very good; crus can be more concentrated"],"ageing":["drink young to medium ageing for crus"],"diagnostic_features":["beaujolais_gamay_core","fruitier and lower tannin than red Burgundy","Gamay rather than Pinot Noir"]}</t>
+        </is>
+      </c>
+      <c r="AR56" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Gamay fruitiness","Beaujolais hierarchy","low-tannin red identification"],"learning_objectives":["identify Gamay markers","separate Beaujolais from red Burgundy","understand Villages versus Cru"],"typical_misconceptions":["Beaujolais is only Nouveau","banana is required in every Gamay","low tannin means poor quality"],"mentor_focus":["ask whether juicy raspberry and low tannin point to Gamay"],"exam_traps":["calling Beaujolais Pinot Noir","missing cru concentration"],"memory_hooks":["Beaujolais is Gamay joy: raspberry, light body, low tannin"],"comparison_styles":["Cote d'Or Red Burgundy","Loire Cabernet Franc","Valpolicella"]}</t>
+        </is>
+      </c>
+      <c r="AS56" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_054"],"frequently_confused_with":["SAT_WINE_054"],"distinguishing_features":["fruitier and lower tannin than red Burgundy","Gamay rather than Pinot Noir","cru hierarchy gives concentration"]}</t>
+        </is>
+      </c>
+      <c r="AT56" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Gamay gives fragrant raspberry wines","Beaujolais hierarchy culminates in crus","Beaujolais and Nouveau are light-bodied and fruity"],"mentor_hints":["Ask if tannin level supports Gamay.","Use hierarchy to avoid dismissing crus."],"student_traps":["treating all Beaujolais as Nouveau","confusing Gamay and Pinot Noir"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU56" t="inlineStr">
+        <is>
+          <t>["beaujolais_gamay_core"]</t>
+        </is>
+      </c>
+      <c r="AV56" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW56" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["8843-8877","8891-8937"],"line_reference":["8843-8877","8891-8937"],"evidence":["Beaujolais production is overwhelmingly red and Gamay gives fragrant wines with raspberry aromas.","The hierarchy moves from Beaujolais to Beaujolais Villages and then individual crus; Beaujolais and Nouveau are light-bodied."]}</t>
+        </is>
+      </c>
+      <c r="AX56" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-10-BATCH-007","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY56" t="inlineStr">
+        <is>
+          <t>16 Beaujolais</t>
+        </is>
+      </c>
+      <c r="AZ56" t="inlineStr">
+        <is>
+          <t>Beaujolais Villages and Crus</t>
+        </is>
+      </c>
+      <c r="BA56" t="inlineStr">
+        <is>
+          <t>90-91</t>
+        </is>
+      </c>
+      <c r="BB56" t="inlineStr">
+        <is>
+          <t>["8843-8877","8891-8937"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SAT_WINE_056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Tintos Francia</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Northern Rhone Syrah</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Syrah from steep northern Rhône slopes with black fruit, pepper and firm structure</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Northern Rhone Syrah</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Northern Rhône</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Côte-Rôtie / Hermitage / Crozes-Hermitage</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Northern Rhône AOCs</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>["Syrah"]</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>continental Rhône valley at the cool limit for Syrah with mistral influence</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>steep south-facing slopes in best sites</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>steep granitic and mixed slope sites; WSET emphasizes slope exposure</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>["Syrah is the only black variety permitted in Northern Rhône","best sites have southerly exposures on steep slopes","Hermitage is a steep south-facing slope"]</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>["red Syrah fermentation and oak maturation depending on appellation","some traditional co-fermentation with white varieties exists but is now rare","top wines are structured and ageworthy"]</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>oak maturation possible; not dominated by new oak aromatics</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>deep ruby</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>["blackberry","black pepper","violet","smoke","meat"]</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>["black fruit","pepper","firm tannin","savoury spice"]</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>very good to outstanding; Hermitage and Côte-Rôtie are benchmarks</t>
+        </is>
+      </c>
+      <c r="AB57" t="inlineStr">
+        <is>
+          <t>long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC57" t="inlineStr">
+        <is>
+          <t>["deep ruby","medium to pronounced intensity","blackberry","black pepper","violet","smoke","meat","dry","medium to high acidity","full body","medium to high alcohol","high tannin","black fruit","pepper","firm tannin","savoury spice"]</t>
+        </is>
+      </c>
+      <c r="AD57" t="inlineStr">
+        <is>
+          <t>["Syrah is the only black variety in Northern Rhône","best sites have southerly exposure and steep slopes","Hermitage is full-bodied and ageworthy"]</t>
+        </is>
+      </c>
+      <c r="AE57" t="inlineStr">
+        <is>
+          <t>["all Rhône reds are Grenache","pepper means oak","Syrah cannot be elegant"]</t>
+        </is>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>["Ask if black pepper is varietal Syrah evidence.","Use Northern versus Southern Rhône as a comparison drill."]</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t>["deep ruby","blackberry","black pepper","violet","smoke","meat","dry","medium to high acidity","full body","medium to high alcohol","high tannin","black fruit","pepper","firm tannin","savoury spice","more peppery and Syrah-driven than Southern Rhône","firmer and darker than Beaujolais","slope exposure is diagnostic"]</t>
+        </is>
+      </c>
+      <c r="AH57" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI57" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Syrah / Hermitage / Crozes-Hermitage evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ57" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Francia - Practica 056</t>
+        </is>
+      </c>
+      <c r="AK57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL57" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM57" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN57" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO57" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP57" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected French red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ57" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby"],"nose":["medium to pronounced intensity","blackberry","black pepper","violet","smoke","meat"],"palate":["dry","medium to high acidity","full body","medium to high alcohol","high tannin","black fruit","pepper","firm tannin"],"quality":["very good to outstanding; Hermitage and Côte-Rôtie are benchmarks"],"ageing":["long ageing potential"],"diagnostic_features":["northern_rhone_syrah_core","more peppery and Syrah-driven than Southern Rhône","firmer and darker than Beaujolais"]}</t>
+        </is>
+      </c>
+      <c r="AR57" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Northern Rhône Syrah identity","slope exposure and ripeness","pepper and savoury structure"],"learning_objectives":["identify Syrah versus Grenache blend","connect steep slopes to ripening","separate Northern and Southern Rhône"],"typical_misconceptions":["all Rhône reds are Grenache","pepper means oak","Syrah cannot be elegant"],"mentor_focus":["ask for black fruit, pepper and firm tannin"],"exam_traps":["calling it Shiraz without origin reasoning","confusing Crozes with Hermitage quality"],"memory_hooks":["Northern Rhône is Syrah on steep slopes at its cool limit"],"comparison_styles":["Chateauneuf-du-Pape Rouge","Australian Shiraz","Left Bank Bordeaux"]}</t>
+        </is>
+      </c>
+      <c r="AS57" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_057"],"frequently_confused_with":["SAT_WINE_057"],"distinguishing_features":["more peppery and Syrah-driven than Southern Rhône","firmer and darker than Beaujolais","slope exposure is diagnostic"]}</t>
+        </is>
+      </c>
+      <c r="AT57" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Syrah is the only black variety in Northern Rhône","best sites have southerly exposure and steep slopes","Hermitage is full-bodied and ageworthy"],"mentor_hints":["Ask if black pepper is varietal Syrah evidence.","Use Northern versus Southern Rhône as a comparison drill."],"student_traps":["mixing Northern and Southern Rhône","overlooking appellation hierarchy"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU57" t="inlineStr">
+        <is>
+          <t>["northern_rhone_syrah_core"]</t>
+        </is>
+      </c>
+      <c r="AV57" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW57" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["9673-9688","9790-9805","9862-9888"],"line_reference":["9673-9688","9790-9805","9862-9888"],"evidence":["Syrah is the only black variety permitted in the Northern Rhône and is at the northern limit of where it can ripen.","Hermitage is on a steep south-facing slope and red Hermitage is generally the fullest-bodied; Crozes-Hermitage reds are made from Syrah."]}</t>
+        </is>
+      </c>
+      <c r="AX57" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-10-BATCH-007","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY57" t="inlineStr">
+        <is>
+          <t>17 Northern Rhône</t>
+        </is>
+      </c>
+      <c r="AZ57" t="inlineStr">
+        <is>
+          <t>Syrah / Hermitage / Crozes-Hermitage</t>
+        </is>
+      </c>
+      <c r="BA57" t="inlineStr">
+        <is>
+          <t>99-101</t>
+        </is>
+      </c>
+      <c r="BB57" t="inlineStr">
+        <is>
+          <t>["9673-9688","9790-9805","9862-9888"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SAT_WINE_057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Tintos Francia</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Chateauneuf-du-Pape Rouge</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Full-bodied Grenache-dominant Southern Rhône blend</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Chateauneuf-du-Pape Rouge</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Southern Rhône</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Châteauneuf-du-Pape</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Châteauneuf-du-Pape AOC</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>["Grenache","Syrah","Mourvedre"]</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>warm Southern Rhône climate with mistral wind and sunny summers</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>east bank of Rhône; warm sites around Châteauneuf-du-Pape</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>varied stones and soils; WSET emphasizes warmth and mistral</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>["Grenache dominates Southern Rhône reds","Syrah and Mourvèdre support Grenache","bush vines are used to protect from wind and benefit from soil warmth"]</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>["Grenache-led blending","large vessels often used because new oak can overwhelm Grenache","producers vary from 100 percent Grenache to more Syrah/Mourvèdre"]</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>usually large vessels; new oak is not a dominant marker</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>deep ruby</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>["red plum","strawberry","baked red fruit","garrigue","sweet spice"]</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>["ripe red fruit","spice","full body","warming alcohol"]</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>very good to outstanding in best examples; variable producer quality</t>
+        </is>
+      </c>
+      <c r="AB58" t="inlineStr">
+        <is>
+          <t>medium to long ageing</t>
+        </is>
+      </c>
+      <c r="AC58" t="inlineStr">
+        <is>
+          <t>["deep ruby","medium to pronounced intensity","red plum","strawberry","baked red fruit","garrigue","sweet spice","dry","medium acidity","full body","high alcohol","medium to high tannin","ripe red fruit","spice","full body","warming alcohol"]</t>
+        </is>
+      </c>
+      <c r="AD58" t="inlineStr">
+        <is>
+          <t>["Grenache dominates Southern Rhône reds","Châteauneuf-du-Pape is most famous for red wine","Syrah and Mourvèdre support Grenache"]</t>
+        </is>
+      </c>
+      <c r="AE58" t="inlineStr">
+        <is>
+          <t>["all Rhône red is Syrah","high alcohol means New World","new oak is required for premium red"]</t>
+        </is>
+      </c>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>["Ask if alcohol and red fruit point to Grenache.","Use Northern/Southern contrast in mentor mode."]</t>
+        </is>
+      </c>
+      <c r="AG58" t="inlineStr">
+        <is>
+          <t>["deep ruby","red plum","strawberry","baked red fruit","garrigue","sweet spice","dry","medium acidity","full body","high alcohol","medium to high tannin","ripe red fruit","spice","full body","warming alcohol","warmer and red-fruited than Northern Rhône Syrah","Grenache-dominant rather than Syrah-only","large vessel rather than new oak focus"]</t>
+        </is>
+      </c>
+      <c r="AH58" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI58" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Châteauneuf-du-Pape / Grenache blends evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ58" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Francia - Practica 057</t>
+        </is>
+      </c>
+      <c r="AK58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL58" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM58" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO58" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP58" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected French red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ58" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby"],"nose":["medium to pronounced intensity","red plum","strawberry","baked red fruit","garrigue","sweet spice"],"palate":["dry","medium acidity","full body","high alcohol","medium to high tannin","ripe red fruit","spice","full body"],"quality":["very good to outstanding in best examples; variable producer quality"],"ageing":["medium to long ageing"],"diagnostic_features":["southern_rhone_grenache_core","warmer and red-fruited than Northern Rhône Syrah","Grenache-dominant rather than Syrah-only"]}</t>
+        </is>
+      </c>
+      <c r="AR58" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Southern Rhône Grenache blends","warm-climate full body","large-vessel Grenache handling"],"learning_objectives":["identify Châteauneuf structure","separate Southern Rhône from Northern Rhône","connect Grenache to alcohol and red fruit"],"typical_misconceptions":["all Rhône red is Syrah","high alcohol means New World","new oak is required for premium red"],"mentor_focus":["ask for full body, warm alcohol and red-fruit spice"],"exam_traps":["calling it Northern Rhône from Rhône label alone","missing Grenache dominance"],"memory_hooks":["Châteauneuf is warm Grenache generosity with Syrah/Mourvèdre support"],"comparison_styles":["Northern Rhone Syrah","Garnacha Spain","Barossa Shiraz"]}</t>
+        </is>
+      </c>
+      <c r="AS58" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_056"],"frequently_confused_with":["SAT_WINE_056"],"distinguishing_features":["warmer and red-fruited than Northern Rhône Syrah","Grenache-dominant rather than Syrah-only","large vessel rather than new oak focus"]}</t>
+        </is>
+      </c>
+      <c r="AT58" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Grenache dominates Southern Rhône reds","Châteauneuf-du-Pape is most famous for red wine","Syrah and Mourvèdre support Grenache"],"mentor_hints":["Ask if alcohol and red fruit point to Grenache.","Use Northern/Southern contrast in mentor mode."],"student_traps":["confusing Rhône north and south","overstating oak"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU58" t="inlineStr">
+        <is>
+          <t>["southern_rhone_grenache_core"]</t>
+        </is>
+      </c>
+      <c r="AV58" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW58" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["9896-9960","10018-10042"],"line_reference":["9896-9960","10018-10042"],"evidence":["Grenache dominates most Southern Rhône red wines and Syrah and Mourvèdre play supporting roles.","Châteauneuf-du-Pape is most famous for red wine, Grenache dominates, and some successful wines are 100 percent Grenache while others use more Syrah and Mourvèdre."]}</t>
+        </is>
+      </c>
+      <c r="AX58" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-10-BATCH-007","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY58" t="inlineStr">
+        <is>
+          <t>18 Southern Rhône</t>
+        </is>
+      </c>
+      <c r="AZ58" t="inlineStr">
+        <is>
+          <t>Châteauneuf-du-Pape / Grenache blends</t>
+        </is>
+      </c>
+      <c r="BA58" t="inlineStr">
+        <is>
+          <t>102-103</t>
+        </is>
+      </c>
+      <c r="BB58" t="inlineStr">
+        <is>
+          <t>["9896-9960","10018-10042"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add Batch 008 Italy red profiles
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -15786,6 +15786,2182 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>SAT_WINE_058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Tintos Italia</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Valpolicella</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Fresh high-acid Corvina-based Veneto red</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Valpolicella</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Veneto</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Valpolicella</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Valpolicella DOC / Valpolicella Classico DOC</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>["Corvina"]</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>warm Veneto climate with foothill and plain contrasts</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>foothills north-west of Verona and flatter southern sites</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>limestone, clay and volcanic foothills; gravel and sand in warmer flatter south</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>["Corvina is the main grape","foothill fruit has more acidity","plain fruit is fruitier with less acidity"]</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>["simple fruity red winemaking","rarely oaked","made to drink immediately"]</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>rarely oaked</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>low to medium</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>pale to medium ruby</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>["red cherry","red plum","fresh herbs"]</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>["red cherry","fresh red fruit","light tannin"]</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>short to medium</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>good; simple fruity styles predominate</t>
+        </is>
+      </c>
+      <c r="AB59" t="inlineStr">
+        <is>
+          <t>drink young</t>
+        </is>
+      </c>
+      <c r="AC59" t="inlineStr">
+        <is>
+          <t>["pale to medium ruby","medium to pronounced intensity","red cherry","red plum","fresh herbs","dry","high acidity","light to medium body","medium alcohol","low to medium tannin","red cherry","fresh red fruit","light tannin"]</t>
+        </is>
+      </c>
+      <c r="AD59" t="inlineStr">
+        <is>
+          <t>["Corvina is the main grape of Valpolicella","Valpolicella is simple and fruity with light tannins","wines are made to drink immediately"]</t>
+        </is>
+      </c>
+      <c r="AE59" t="inlineStr">
+        <is>
+          <t>["Valpolicella is always full-bodied","all Veneto red is Amarone","pale colour means Pinot Noir"]</t>
+        </is>
+      </c>
+      <c r="AF59" t="inlineStr">
+        <is>
+          <t>["Compare structure directly against Amarone.","Ask whether tannin and body are too light for passito."]</t>
+        </is>
+      </c>
+      <c r="AG59" t="inlineStr">
+        <is>
+          <t>["pale to medium ruby","red cherry","red plum","fresh herbs","dry","high acidity","light to medium body","medium alcohol","low to medium tannin","red cherry","fresh red fruit","light tannin","lighter and fresher than Amarone","more cherry-acid Corvina than Gamay raspberry","rarely oaked"]</t>
+        </is>
+      </c>
+      <c r="AH59" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI59" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Veneto - Valpolicella evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ59" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Italia - Practica 058</t>
+        </is>
+      </c>
+      <c r="AK59" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL59" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM59" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN59" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AO59" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="AP59" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Italian red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ59" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale to medium ruby"],"nose":["medium to pronounced intensity","red cherry","red plum","fresh herbs"],"palate":["dry","high acidity","light to medium body","medium alcohol","low to medium tannin","red cherry","fresh red fruit","light tannin"],"quality":["good; simple fruity styles predominate"],"ageing":["drink young"],"diagnostic_features":["valpolicella_corvina_core","lighter and fresher than Amarone","more cherry-acid Corvina than Gamay raspberry"]}</t>
+        </is>
+      </c>
+      <c r="AR59" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Corvina freshness","Valpolicella immediacy","Veneto red baseline"],"learning_objectives":["identify Valpolicella structure","separate simple Valpolicella from Amarone","connect Corvina to high acidity"],"typical_misconceptions":["Valpolicella is always full-bodied","all Veneto red is Amarone","pale colour means Pinot Noir"],"mentor_focus":["ask for red cherry, high acidity and light tannin"],"exam_traps":["calling simple Valpolicella Beaujolais","overstating oak"],"memory_hooks":["Valpolicella is fresh Corvina red cherry"],"comparison_styles":["Amarone della Valpolicella","Beaujolais Villages / Cru"]}</t>
+        </is>
+      </c>
+      <c r="AS59" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_059","SAT_WINE_055"],"frequently_confused_with":["SAT_WINE_055","SAT_WINE_059"],"distinguishing_features":["lighter and fresher than Amarone","more cherry-acid Corvina than Gamay raspberry","rarely oaked"]}</t>
+        </is>
+      </c>
+      <c r="AT59" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Corvina is the main grape of Valpolicella","Valpolicella is simple and fruity with light tannins","wines are made to drink immediately"],"mentor_hints":["Compare structure directly against Amarone.","Ask whether tannin and body are too light for passito."],"student_traps":["confusing Valpolicella with Amarone","missing high acidity"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU59" t="inlineStr">
+        <is>
+          <t>["valpolicella_corvina_core"]</t>
+        </is>
+      </c>
+      <c r="AV59" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW59" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11884-11901"],"line_reference":["11884-11901"],"evidence":["Valpolicella is north-west of Verona; Corvina is the main grape with moderate colour, low to medium tannin and high acidity.","The wines are simple and fruity with light tannins and red cherry flavours, rarely oaked and made to drink immediately."]}</t>
+        </is>
+      </c>
+      <c r="AX59" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-11-BATCH-008","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY59" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ59" t="inlineStr">
+        <is>
+          <t>Veneto - Valpolicella</t>
+        </is>
+      </c>
+      <c r="BA59" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="BB59" t="inlineStr">
+        <is>
+          <t>["11884-11901"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SAT_WINE_059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Tintos Italia</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Amarone della Valpolicella</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Full-bodied dry or off-dry passito red from Veneto</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Amarone della Valpolicella</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Veneto</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Valpolicella</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Amarone della Valpolicella DOCG</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>["Corvina"]</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>warm Veneto with grapes picked early for passito drying</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Valpolicella drying-fruit source vineyards</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>varied Veneto soils; drying process is the diagnostic marker</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>["grapes picked early while still high in acidity","grapes dried indoors to concentrate sugars and flavours","fruit must be healthy for drying"]</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>["passito method","fermentation starts in winter","usually aged in large oak casks"]</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>usually large oak casks</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>dry to off-dry</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>deep ruby to garnet</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>["dried cherry","red berry","spice","raisins","chocolate"]</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>["concentrated red berry","spice","dried fruit","warming alcohol"]</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>very good to outstanding; iconic passito dry red</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
+        <is>
+          <t>long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>["deep ruby to garnet","medium to pronounced intensity","dried cherry","red berry","spice","raisins","chocolate","dry to off-dry","medium to high acidity","full body","high alcohol","medium to high tannin","concentrated red berry","spice","dried fruit","warming alcohol"]</t>
+        </is>
+      </c>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>["Amarone is dry or off-dry","passito dries grapes indoors","Amarone is full-bodied and high alcohol"]</t>
+        </is>
+      </c>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>["Amarone is sweet like Recioto","all dried-grape wines are dessert wines","high alcohol means New World"]</t>
+        </is>
+      </c>
+      <c r="AF60" t="inlineStr">
+        <is>
+          <t>["Ask whether sweetness is residual or perceived from alcohol/dried fruit.","Use passito as the causal link."]</t>
+        </is>
+      </c>
+      <c r="AG60" t="inlineStr">
+        <is>
+          <t>["deep ruby to garnet","dried cherry","red berry","spice","raisins","chocolate","dry to off-dry","medium to high acidity","full body","high alcohol","medium to high tannin","concentrated red berry","spice","dried fruit","warming alcohol","much fuller than Valpolicella","dried fruit passito signature","not fortified like Port"]</t>
+        </is>
+      </c>
+      <c r="AH60" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI60" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Veneto - Passito method / Amarone evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ60" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Italia - Practica 059</t>
+        </is>
+      </c>
+      <c r="AK60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL60" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN60" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO60" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP60" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Italian red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ60" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby to garnet"],"nose":["medium to pronounced intensity","dried cherry","red berry","spice","raisins","chocolate"],"palate":["dry to off-dry","medium to high acidity","full body","high alcohol","medium to high tannin","concentrated red berry","spice","dried fruit"],"quality":["very good to outstanding; iconic passito dry red"],"ageing":["long ageing potential"],"diagnostic_features":["amarone_passito_core","much fuller than Valpolicella","dried fruit passito signature"]}</t>
+        </is>
+      </c>
+      <c r="AR60" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["passito concentration","dry/off-dry high-alcohol red","Veneto Amarone identity"],"learning_objectives":["identify Amarone structure","connect drying to concentration","separate Amarone from Recioto and Valpolicella"],"typical_misconceptions":["Amarone is sweet like Recioto","all dried-grape wines are dessert wines","high alcohol means New World"],"mentor_focus":["ask if dried fruit and alcohol are structural not just age"],"exam_traps":["calling Amarone Port","missing acidity retained by early harvest"],"memory_hooks":["Amarone is dried-grape power, not fortified sweetness"],"comparison_styles":["Valpolicella","Chateauneuf-du-Pape Rouge","Vintage Port"]}</t>
+        </is>
+      </c>
+      <c r="AS60" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_058","SAT_WINE_057"],"frequently_confused_with":["SAT_WINE_058","SAT_WINE_057"],"distinguishing_features":["much fuller than Valpolicella","dried fruit passito signature","not fortified like Port"]}</t>
+        </is>
+      </c>
+      <c r="AT60" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Amarone is dry or off-dry","passito dries grapes indoors","Amarone is full-bodied and high alcohol"],"mentor_hints":["Ask whether sweetness is residual or perceived from alcohol/dried fruit.","Use passito as the causal link."],"student_traps":["assuming Amarone is fortified","confusing Amarone and Recioto"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU60" t="inlineStr">
+        <is>
+          <t>["amarone_passito_core"]</t>
+        </is>
+      </c>
+      <c r="AV60" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW60" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["11903-11920"],"line_reference":["11903-11920"],"evidence":["Amarone della Valpolicella DOCG wines are dry or off-dry, full-bodied, high alcohol, medium to high tannin and intensely concentrated red berry and spice flavours.","The passito method dries grapes indoors, concentrating sugars and flavours; Amarone is usually aged in large oak casks."]}</t>
+        </is>
+      </c>
+      <c r="AX60" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-11-BATCH-008","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY60" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ60" t="inlineStr">
+        <is>
+          <t>Veneto - Passito method / Amarone</t>
+        </is>
+      </c>
+      <c r="BA60" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="BB60" t="inlineStr">
+        <is>
+          <t>["11903-11920"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>SAT_WINE_060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Tintos Italia</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Barolo</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Structured ageworthy Nebbiolo from south-facing Piemonte slopes</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Barolo</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Piemonte</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Barolo</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Barolo DOCG</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>["Nebbiolo"]</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>moderate continental Piemonte with fog and hillside variation</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>300 to 500 metre south-facing slopes</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>hillside sites with aspect and altitude differences</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>["Barolo must be entirely Nebbiolo","Nebbiolo ripens slowly at altitude","best wines can come from named vineyards or crus"]</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>["aged three years before release with 18 months in oak","traditional large oak or modern shorter oak choices","benefits from bottle ageing"]</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>oak ageing required; large casks or smaller barrels depending on producer</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>pale garnet to medium ruby</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>["sour cherry","herbs","dried flowers","tar","leather"]</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>["sour cherry","herbs","firm tannin","earthy complexity"]</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>outstanding for top sites and vintages</t>
+        </is>
+      </c>
+      <c r="AB61" t="inlineStr">
+        <is>
+          <t>long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC61" t="inlineStr">
+        <is>
+          <t>["pale garnet to medium ruby","medium to pronounced intensity","sour cherry","herbs","dried flowers","tar","leather","dry","high acidity","full body","medium to high alcohol","high tannin","sour cherry","herbs","firm tannin","earthy complexity"]</t>
+        </is>
+      </c>
+      <c r="AD61" t="inlineStr">
+        <is>
+          <t>["Barolo must be 100 percent Nebbiolo","Barolo must be aged three years before release","all Barolo benefits from bottle ageing"]</t>
+        </is>
+      </c>
+      <c r="AE61" t="inlineStr">
+        <is>
+          <t>["pale colour means light body","Nebbiolo lacks tannin","all Piemonte red is Barolo"]</t>
+        </is>
+      </c>
+      <c r="AF61" t="inlineStr">
+        <is>
+          <t>["Ask if colour misleads the student away from tannin.","Use legal ageing as a memory peg."]</t>
+        </is>
+      </c>
+      <c r="AG61" t="inlineStr">
+        <is>
+          <t>["pale garnet to medium ruby","sour cherry","herbs","dried flowers","tar","leather","dry","high acidity","full body","medium to high alcohol","high tannin","sour cherry","herbs","firm tannin","earthy complexity","higher altitude and longer ageing than Barbaresco","more Nebbiolo perfume than Sangiovese","pale colour with high tannin"]</t>
+        </is>
+      </c>
+      <c r="AH61" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI61" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Piemonte - Barolo evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ61" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Italia - Practica 060</t>
+        </is>
+      </c>
+      <c r="AK61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL61" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM61" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AO61" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="AP61" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Italian red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ61" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale garnet to medium ruby"],"nose":["medium to pronounced intensity","sour cherry","herbs","dried flowers","tar","leather"],"palate":["dry","high acidity","full body","medium to high alcohol","high tannin","sour cherry","herbs","firm tannin"],"quality":["outstanding for top sites and vintages"],"ageing":["long ageing potential"],"diagnostic_features":["barolo_nebbiolo_core","higher altitude and longer ageing than Barbaresco","more Nebbiolo perfume than Sangiovese"]}</t>
+        </is>
+      </c>
+      <c r="AR61" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Nebbiolo structure","Barolo ageing law","site and cru identity"],"learning_objectives":["identify Barolo tannin-acid profile","connect ageing to tar/leather complexity","separate Barolo from Barbaresco"],"typical_misconceptions":["pale colour means light body","Nebbiolo lacks tannin","all Piemonte red is Barolo"],"mentor_focus":["ask whether tannin and acidity are both high despite pale colour"],"exam_traps":["calling Barolo Pinot Noir from colour","missing ageing requirement"],"memory_hooks":["Barolo is pale but fierce: acid, tannin, tar and time"],"comparison_styles":["Barbaresco","Brunello di Montalcino","Left Bank Bordeaux"]}</t>
+        </is>
+      </c>
+      <c r="AS61" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_061","SAT_WINE_064"],"frequently_confused_with":["SAT_WINE_061","SAT_WINE_052"],"distinguishing_features":["higher altitude and longer ageing than Barbaresco","more Nebbiolo perfume than Sangiovese","pale colour with high tannin"]}</t>
+        </is>
+      </c>
+      <c r="AT61" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Barolo must be 100 percent Nebbiolo","Barolo must be aged three years before release","all Barolo benefits from bottle ageing"],"mentor_hints":["Ask if colour misleads the student away from tannin.","Use legal ageing as a memory peg."],"student_traps":["underestimating tannin because colour is pale","confusing Barolo and Barbaresco"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU61" t="inlineStr">
+        <is>
+          <t>["barolo_nebbiolo_core"]</t>
+        </is>
+      </c>
+      <c r="AV61" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW61" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12029-12066"],"line_reference":["12029-12066"],"evidence":["Barolo DOCG must be entirely Nebbiolo from steep south-facing slopes; Nebbiolo has high acidity and tannins with sour cherry, herbs and sometimes dried flowers.","Barolo must be aged three years, including 18 months in oak, and benefits from bottle ageing developing truffle, tar and leather."]}</t>
+        </is>
+      </c>
+      <c r="AX61" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-11-BATCH-008","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY61" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ61" t="inlineStr">
+        <is>
+          <t>Piemonte - Barolo</t>
+        </is>
+      </c>
+      <c r="BA61" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="BB61" t="inlineStr">
+        <is>
+          <t>["12029-12066"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>SAT_WINE_061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Tintos Italia</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Barbaresco</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Nebbiolo from lower-altitude Piemonte slopes with earlier ripening fruit</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Barbaresco</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Piemonte</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Barbaresco</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Barbaresco DOCG</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>["Nebbiolo"]</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>moderate continental Piemonte with lower-altitude Barbaresco sites</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>200 to 400 metre south-facing slopes</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>slope sites near local river influence</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>["Nebbiolo ripens earlier than Barolo here","lower altitude gives fruitier less perfumed wines","wines have acidity and tannin to age"]</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>["aged two years before release with nine months in oak","fewer village mentions than Barolo","single vineyard or cru may indicate higher quality"]</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>oak ageing required</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>pale garnet to medium ruby</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>["red cherry","sour cherry","herbs","rose","earth"]</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>["red cherry","herbs","firm tannin","savoury finish"]</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>very good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB62" t="inlineStr">
+        <is>
+          <t>medium to long ageing</t>
+        </is>
+      </c>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>["pale garnet to medium ruby","medium to pronounced intensity","red cherry","sour cherry","herbs","rose","earth","dry","high acidity","medium to full body","medium to high alcohol","high tannin","red cherry","herbs","firm tannin","savoury finish"]</t>
+        </is>
+      </c>
+      <c r="AD62" t="inlineStr">
+        <is>
+          <t>["Barbaresco has lower altitude than Barolo","Nebbiolo ripens earlier here","Barbaresco must age two years before release"]</t>
+        </is>
+      </c>
+      <c r="AE62" t="inlineStr">
+        <is>
+          <t>["Barbaresco is simple Barolo","lower altitude means no ageing","Nebbiolo always smells the same"]</t>
+        </is>
+      </c>
+      <c r="AF62" t="inlineStr">
+        <is>
+          <t>["Ask if the student can explain why it is not Barolo.","Use lower altitude as the causal hook."]</t>
+        </is>
+      </c>
+      <c r="AG62" t="inlineStr">
+        <is>
+          <t>["pale garnet to medium ruby","red cherry","sour cherry","herbs","rose","earth","dry","high acidity","medium to full body","medium to high alcohol","high tannin","red cherry","herbs","firm tannin","savoury finish","fruitier and less perfumed than Barolo","shorter ageing requirement","same Nebbiolo acid-tannin spine"]</t>
+        </is>
+      </c>
+      <c r="AH62" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI62" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Piemonte - Barbaresco evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ62" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Italia - Practica 061</t>
+        </is>
+      </c>
+      <c r="AK62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL62" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM62" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN62" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO62" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP62" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Italian red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ62" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale garnet to medium ruby"],"nose":["medium to pronounced intensity","red cherry","sour cherry","herbs","rose","earth"],"palate":["dry","high acidity","medium to full body","medium to high alcohol","high tannin","red cherry","herbs","firm tannin"],"quality":["very good to outstanding"],"ageing":["medium to long ageing"],"diagnostic_features":["barbaresco_nebbiolo_core","fruitier and less perfumed than Barolo","shorter ageing requirement"]}</t>
+        </is>
+      </c>
+      <c r="AR62" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Barbaresco versus Barolo","Nebbiolo fruit and structure","legal ageing contrast"],"learning_objectives":["distinguish Barbaresco from Barolo","identify Nebbiolo despite fruitier profile","connect lower altitude to earlier ripening"],"typical_misconceptions":["Barbaresco is simple Barolo","lower altitude means no ageing","Nebbiolo always smells the same"],"mentor_focus":["ask whether Nebbiolo structure is present with a fruitier tone"],"exam_traps":["overcalling Barolo","ignoring legal ageing contrast"],"memory_hooks":["Barbaresco is Nebbiolo a little earlier and fruitier"],"comparison_styles":["Barolo","Red Burgundy","Brunello di Montalcino"]}</t>
+        </is>
+      </c>
+      <c r="AS62" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_060"],"frequently_confused_with":["SAT_WINE_060","SAT_WINE_054"],"distinguishing_features":["fruitier and less perfumed than Barolo","shorter ageing requirement","same Nebbiolo acid-tannin spine"]}</t>
+        </is>
+      </c>
+      <c r="AT62" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Barbaresco has lower altitude than Barolo","Nebbiolo ripens earlier here","Barbaresco must age two years before release"],"mentor_hints":["Ask if the student can explain why it is not Barolo.","Use lower altitude as the causal hook."],"student_traps":["collapsing all Nebbiolo into Barolo","missing Barbaresco ageing law"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU62" t="inlineStr">
+        <is>
+          <t>["barbaresco_nebbiolo_core"]</t>
+        </is>
+      </c>
+      <c r="AV62" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW62" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12068-12080"],"line_reference":["12068-12080"],"evidence":["Barbaresco is renowned for Nebbiolo, with lower altitude than Barolo, earlier ripening, fruitier and less perfumed wines.","Barbaresco has similar acidity and tannin levels and must be aged two years with nine months in oak."]}</t>
+        </is>
+      </c>
+      <c r="AX62" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-11-BATCH-008","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY62" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ62" t="inlineStr">
+        <is>
+          <t>Piemonte - Barbaresco</t>
+        </is>
+      </c>
+      <c r="BA62" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="BB62" t="inlineStr">
+        <is>
+          <t>["12068-12080"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>SAT_WINE_062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Tintos Italia</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Barbera d'Asti</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>High-acid low-tannin Barbera from Piemonte</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Barbera d'Asti</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Piemonte</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Asti</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Barbera d'Asti DOCG</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>["Barbera"]</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>moderate continental Piemonte</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>hills around Asti and Alba</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>not specified by WSET; grape and appellation are key</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>["Barbera is the most widely planted black grape in Asti/Alba area","Barbera is late ripening","Barbera d'Asti is often regarded as higher quality than Barbera d'Alba"]</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>["youthful fruity no-oak style or barrel-aged spicy style","oak may add spice","drunk young or aged several years for best examples"]</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>none in youthful styles; barrel-aged versions show spice</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>low to medium</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>medium ruby</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>["red cherry","plum","black pepper","spice"]</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>["red cherry","plum","high-acid palate","soft tannin"]</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>good to very good; Barbera d'Asti often higher quality</t>
+        </is>
+      </c>
+      <c r="AB63" t="inlineStr">
+        <is>
+          <t>short to medium ageing for best examples</t>
+        </is>
+      </c>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>["medium ruby","medium to pronounced intensity","red cherry","plum","black pepper","spice","dry","high acidity","medium body","medium alcohol","low to medium tannin","red cherry","plum","high-acid palate","soft tannin"]</t>
+        </is>
+      </c>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t>["Barbera is the most widely planted black grape around Asti and Alba","Barbera d'Asti is often regarded as higher quality","Barbera has high acidity and low to medium tannin"]</t>
+        </is>
+      </c>
+      <c r="AE63" t="inlineStr">
+        <is>
+          <t>["high acidity means high tannin","all Piemonte red is Nebbiolo","Barbera cannot age"]</t>
+        </is>
+      </c>
+      <c r="AF63" t="inlineStr">
+        <is>
+          <t>["Ask for tannin-acid contrast.","Use Barbera as the Piemonte non-Nebbiolo foil."]</t>
+        </is>
+      </c>
+      <c r="AG63" t="inlineStr">
+        <is>
+          <t>["medium ruby","red cherry","plum","black pepper","spice","dry","high acidity","medium body","medium alcohol","low to medium tannin","red cherry","plum","high-acid palate","soft tannin","lower tannin than Nebbiolo","more plum-cherry than Sangiovese herbs","higher acidity than Valpolicella with deeper colour"]</t>
+        </is>
+      </c>
+      <c r="AH63" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI63" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Piemonte - Asti and Alba evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ63" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Italia - Practica 062</t>
+        </is>
+      </c>
+      <c r="AK63" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL63" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM63" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN63" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO63" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP63" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Italian red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ63" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium ruby"],"nose":["medium to pronounced intensity","red cherry","plum","black pepper","spice"],"palate":["dry","high acidity","medium body","medium alcohol","low to medium tannin","red cherry","plum","high-acid palate"],"quality":["good to very good; Barbera d'Asti often higher quality"],"ageing":["short to medium ageing for best examples"],"diagnostic_features":["barbera_asti_core","lower tannin than Nebbiolo","more plum-cherry than Sangiovese herbs"]}</t>
+        </is>
+      </c>
+      <c r="AR63" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Barbera acid-tannin contrast","Asti quality cue","oak style choice"],"learning_objectives":["identify high-acid low-tannin Barbera","separate Barbera from Nebbiolo","understand youthful versus barrel-aged styles"],"typical_misconceptions":["high acidity means high tannin","all Piemonte red is Nebbiolo","Barbera cannot age"],"mentor_focus":["ask whether acidity is high but tannin is relatively soft"],"exam_traps":["calling Barbera Nebbiolo","missing low tannin"],"memory_hooks":["Barbera is Piemonte red with acid turned up and tannin turned down"],"comparison_styles":["Barolo","Chianti Classico","Valpolicella"]}</t>
+        </is>
+      </c>
+      <c r="AS63" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_060","SAT_WINE_063"],"frequently_confused_with":["SAT_WINE_060","SAT_WINE_063"],"distinguishing_features":["lower tannin than Nebbiolo","more plum-cherry than Sangiovese herbs","higher acidity than Valpolicella with deeper colour"]}</t>
+        </is>
+      </c>
+      <c r="AT63" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Barbera is the most widely planted black grape around Asti and Alba","Barbera d'Asti is often regarded as higher quality","Barbera has high acidity and low to medium tannin"],"mentor_hints":["Ask for tannin-acid contrast.","Use Barbera as the Piemonte non-Nebbiolo foil."],"student_traps":["assuming Piemonte equals Nebbiolo","overcalling tannin"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU63" t="inlineStr">
+        <is>
+          <t>["barbera_asti_core"]</t>
+        </is>
+      </c>
+      <c r="AV63" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW63" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12082-12105"],"line_reference":["12082-12105"],"evidence":["Barbera is the most widely planted black grape in the Asti and Alba area and Barbera d'Asti DOCG is often regarded as higher quality.","It has medium to deep colour, low to medium tannins, high acidity, red cherries, plums and sometimes black pepper; styles can be youthful fruity or barrel-aged spicy."]}</t>
+        </is>
+      </c>
+      <c r="AX63" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-11-BATCH-008","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY63" t="inlineStr">
+        <is>
+          <t>27 Northern Italy</t>
+        </is>
+      </c>
+      <c r="AZ63" t="inlineStr">
+        <is>
+          <t>Piemonte - Asti and Alba</t>
+        </is>
+      </c>
+      <c r="BA63" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="BB63" t="inlineStr">
+        <is>
+          <t>["12082-12105"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>SAT_WINE_063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Tintos Italia</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Chianti Classico</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>High-acid Sangiovese from elevated Chianti Classico vineyards</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Chianti Classico</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Tuscany</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Chianti Classico</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Chianti Classico DOCG</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>["Sangiovese"]</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>warm central Italian climate moderated by altitude in Apennine foothills</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>higher-altitude Chianti Classico vineyards</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>not specified by WSET; elevation and foothill setting are key</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>["Chianti is based on Sangiovese","Chianti Classico vineyards are at higher altitudes than Chianti DOCG","higher altitude slows ripening and increases acidity and herbal aromas"]</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>["red fermentation with ageing depending on level","Riserva and Gran Selezione have higher ageing/designation expectations","large and small oak use varies"]</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>variable oak depending on producer and category</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>medium ruby</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>["red cherry","red plum","dried herbs","violet","earth"]</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>["sour cherry","red plum","herbal notes","firm acidity"]</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>very good to outstanding for top Classico levels</t>
+        </is>
+      </c>
+      <c r="AB64" t="inlineStr">
+        <is>
+          <t>medium to long ageing for Riserva and Gran Selezione</t>
+        </is>
+      </c>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>["medium ruby","medium to pronounced intensity","red cherry","red plum","dried herbs","violet","earth","dry","high acidity","medium body","medium to high alcohol","medium to high tannin","sour cherry","red plum","herbal notes","firm acidity"]</t>
+        </is>
+      </c>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t>["Chianti is based on Sangiovese","Chianti Classico has its own DOCG","higher altitude gives greater acidity and herbal aromas"]</t>
+        </is>
+      </c>
+      <c r="AE64" t="inlineStr">
+        <is>
+          <t>["Chianti Classico is just a sub-zone of Chianti","all Sangiovese is full-bodied","herbal notes mean underripe"]</t>
+        </is>
+      </c>
+      <c r="AF64" t="inlineStr">
+        <is>
+          <t>["Ask whether high acidity comes with Sangiovese tannin/herbs.","Use Classico geography in debrief."]</t>
+        </is>
+      </c>
+      <c r="AG64" t="inlineStr">
+        <is>
+          <t>["medium ruby","red cherry","red plum","dried herbs","violet","earth","dry","high acidity","medium body","medium to high alcohol","medium to high tannin","sour cherry","red plum","herbal notes","firm acidity","more herbal and Sangiovese than Barbera","less full-bodied than Brunello","Classico higher-altitude source"]</t>
+        </is>
+      </c>
+      <c r="AH64" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI64" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Tuscany - Chianti / Chianti Classico evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ64" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Italia - Practica 063</t>
+        </is>
+      </c>
+      <c r="AK64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL64" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM64" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN64" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO64" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP64" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Italian red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ64" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium ruby"],"nose":["medium to pronounced intensity","red cherry","red plum","dried herbs","violet","earth"],"palate":["dry","high acidity","medium body","medium to high alcohol","medium to high tannin","sour cherry","red plum","herbal notes"],"quality":["very good to outstanding for top Classico levels"],"ageing":["medium to long ageing for Riserva and Gran Selezione"],"diagnostic_features":["chianti_classico_sangiovese_core","more herbal and Sangiovese than Barbera","less full-bodied than Brunello"]}</t>
+        </is>
+      </c>
+      <c r="AR64" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Sangiovese acidity","Chianti Classico altitude","Tuscan classification"],"learning_objectives":["identify Chianti Classico markers","connect altitude to acidity and herbs","separate Sangiovese from Barbera"],"typical_misconceptions":["Chianti Classico is just a sub-zone of Chianti","all Sangiovese is full-bodied","herbal notes mean underripe"],"mentor_focus":["ask for sour cherry, herbs and high acidity"],"exam_traps":["calling it Barbera from acidity alone","missing Classico status"],"memory_hooks":["Chianti Classico is Sangiovese lifted by altitude"],"comparison_styles":["Brunello di Montalcino","Barbera d'Asti","Vino Nobile di Montepulciano"]}</t>
+        </is>
+      </c>
+      <c r="AS64" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_064","SAT_WINE_062"],"frequently_confused_with":["SAT_WINE_062","SAT_WINE_064"],"distinguishing_features":["more herbal and Sangiovese than Barbera","less full-bodied than Brunello","Classico higher-altitude source"]}</t>
+        </is>
+      </c>
+      <c r="AT64" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Chianti is based on Sangiovese","Chianti Classico has its own DOCG","higher altitude gives greater acidity and herbal aromas"],"mentor_hints":["Ask whether high acidity comes with Sangiovese tannin/herbs.","Use Classico geography in debrief."],"student_traps":["confusing Chianti and Chianti Classico","overlooking Sangiovese acidity"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU64" t="inlineStr">
+        <is>
+          <t>["chianti_classico_sangiovese_core"]</t>
+        </is>
+      </c>
+      <c r="AV64" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW64" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12190-12225"],"line_reference":["12190-12225"],"evidence":["Chianti is based on Sangiovese; Chianti Classico DOCG is separate and its higher altitude vineyards slow ripening, giving greater acidity and more herbal aromas.","Chianti Classico Riserva and Gran Selezione are higher designations."]}</t>
+        </is>
+      </c>
+      <c r="AX64" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-11-BATCH-008","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY64" t="inlineStr">
+        <is>
+          <t>28 Central Italy</t>
+        </is>
+      </c>
+      <c r="AZ64" t="inlineStr">
+        <is>
+          <t>Tuscany - Chianti / Chianti Classico</t>
+        </is>
+      </c>
+      <c r="BA64" t="inlineStr">
+        <is>
+          <t>126-127</t>
+        </is>
+      </c>
+      <c r="BB64" t="inlineStr">
+        <is>
+          <t>["12190-12225"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SAT_WINE_064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Tintos Italia</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Brunello di Montalcino</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Fuller-bodied ageworthy Sangiovese from Montalcino</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Brunello di Montalcino</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Tuscany</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Montalcino</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Brunello di Montalcino DOCG</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>["Sangiovese"]</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>warmer southern Tuscany moderated by altitude and sea breezes</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>hills around Montalcino</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>not specified by WSET; warmth and hill exposure matter</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>["Montalcino conditions create more intense fuller Sangiovese","Brunello regulations require long ageing","style is more powerful than Chianti"]</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>["must be aged for five years before sale","two years must be in oak","long maturation supports complexity"]</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>oak ageing required; two years in oak</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>medium to deep ruby to garnet</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>["red cherry","plum","dried herbs","leather","spice"]</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>["red cherry","plum","firm tannin","savoury oak complexity"]</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>outstanding in top examples</t>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr">
+        <is>
+          <t>long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>["medium to deep ruby to garnet","medium to pronounced intensity","red cherry","plum","dried herbs","leather","spice","dry","high acidity","full body","high alcohol","high tannin","red cherry","plum","firm tannin","savoury oak complexity"]</t>
+        </is>
+      </c>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t>["Brunello is fuller-bodied than Chianti","Brunello must age before sale","two years must be in oak"]</t>
+        </is>
+      </c>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>["Brunello is a separate grape","all Sangiovese is medium-bodied","oak means Bordeaux"]</t>
+        </is>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>["Ask if the power level exceeds Chianti Classico.","Use legal ageing as a diagnostic anchor."]</t>
+        </is>
+      </c>
+      <c r="AG65" t="inlineStr">
+        <is>
+          <t>["medium to deep ruby to garnet","red cherry","plum","dried herbs","leather","spice","dry","high acidity","full body","high alcohol","high tannin","red cherry","plum","firm tannin","savoury oak complexity","fuller than Chianti Classico","Sangiovese red cherry and herbs rather than Nebbiolo tar","mandatory long ageing"]</t>
+        </is>
+      </c>
+      <c r="AH65" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI65" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Tuscany - Brunello di Montalcino evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ65" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Italia - Practica 064</t>
+        </is>
+      </c>
+      <c r="AK65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL65" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM65" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN65" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO65" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP65" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Italian red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ65" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium to deep ruby to garnet"],"nose":["medium to pronounced intensity","red cherry","plum","dried herbs","leather","spice"],"palate":["dry","high acidity","full body","high alcohol","high tannin","red cherry","plum","firm tannin"],"quality":["outstanding in top examples"],"ageing":["long ageing potential"],"diagnostic_features":["brunello_sangiovese_core","fuller than Chianti Classico","Sangiovese red cherry and herbs rather than Nebbiolo tar"]}</t>
+        </is>
+      </c>
+      <c r="AR65" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["powerful Sangiovese","Brunello ageing law","Montalcino versus Chianti"],"learning_objectives":["distinguish Brunello from Chianti Classico","identify full-bodied Sangiovese","connect oak ageing to complexity"],"typical_misconceptions":["Brunello is a separate grape","all Sangiovese is medium-bodied","oak means Bordeaux"],"mentor_focus":["ask whether Sangiovese acidity is carried by more body and tannin"],"exam_traps":["calling Brunello Chianti","forgetting ageing requirements"],"memory_hooks":["Brunello is Sangiovese turned fuller and longer-aged"],"comparison_styles":["Chianti Classico","Barolo","Taurasi"]}</t>
+        </is>
+      </c>
+      <c r="AS65" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_063","SAT_WINE_060"],"frequently_confused_with":["SAT_WINE_063","SAT_WINE_060"],"distinguishing_features":["fuller than Chianti Classico","Sangiovese red cherry and herbs rather than Nebbiolo tar","mandatory long ageing"]}</t>
+        </is>
+      </c>
+      <c r="AT65" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Brunello is fuller-bodied than Chianti","Brunello must age before sale","two years must be in oak"],"mentor_hints":["Ask if the power level exceeds Chianti Classico.","Use legal ageing as a diagnostic anchor."],"student_traps":["thinking Brunello is a grape","missing Sangiovese identity"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU65" t="inlineStr">
+        <is>
+          <t>["brunello_sangiovese_core"]</t>
+        </is>
+      </c>
+      <c r="AV65" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW65" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12238-12249"],"line_reference":["12238-12249"],"evidence":["Brunello di Montalcino is more intense and fuller-bodied than Chianti.","Regulations stipulate long ageing before sale, two years of which must be in oak."]}</t>
+        </is>
+      </c>
+      <c r="AX65" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-11-BATCH-008","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY65" t="inlineStr">
+        <is>
+          <t>28 Central Italy</t>
+        </is>
+      </c>
+      <c r="AZ65" t="inlineStr">
+        <is>
+          <t>Tuscany - Brunello di Montalcino</t>
+        </is>
+      </c>
+      <c r="BA65" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="BB65" t="inlineStr">
+        <is>
+          <t>["12238-12249"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>SAT_WINE_065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Tintos Italia</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Taurasi</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Prestigious ageworthy Aglianico from Campania</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Taurasi</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Campania</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Taurasi</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Taurasi DOCG</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>["Aglianico"]</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>southern Italy with varied mountains, valleys and coastal plains enabling quality reds</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>inland Campanian sites suited to Aglianico</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>not specified by WSET; grape prestige and appellation are key</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>["Aglianico is the most prestigious black grape of southern Italy","it is at its best in Taurasi DOCG","late-ripening structured grape"]</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>["structured red winemaking","oak maturation commonly used for premium ageworthy styles","requires time to soften tannin"]</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>oak commonly used in premium styles</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>deep ruby to garnet</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>["black cherry","black plum","earth","smoke","dried herbs"]</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>["black fruit","earth","firm tannin","savoury spice"]</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>very good to outstanding; Taurasi is the benchmark for Aglianico</t>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t>long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>["deep ruby to garnet","medium to pronounced intensity","black cherry","black plum","earth","smoke","dried herbs","dry","high acidity","full body","medium to high alcohol","high tannin","black fruit","earth","firm tannin","savoury spice"]</t>
+        </is>
+      </c>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t>["Aglianico is the most prestigious black grape of southern Italy","Taurasi DOCG is its best expression","Aglianico is a key Campanian red"]</t>
+        </is>
+      </c>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>["southern Italy only makes soft fruity reds","Aglianico is low acid","all Italian ageworthy reds are Nebbiolo"]</t>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t>["Ask if the student can name a southern Italian ageworthy red.","Use Taurasi as the Aglianico anchor."]</t>
+        </is>
+      </c>
+      <c r="AG66" t="inlineStr">
+        <is>
+          <t>["deep ruby to garnet","black cherry","black plum","earth","smoke","dried herbs","dry","high acidity","full body","medium to high alcohol","high tannin","black fruit","earth","firm tannin","savoury spice","darker and more southern than Nebbiolo","more black-fruited than Sangiovese","Aglianico benchmark Taurasi"]</t>
+        </is>
+      </c>
+      <c r="AH66" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI66" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Campania - Aglianico / Taurasi evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ66" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Italia - Practica 065</t>
+        </is>
+      </c>
+      <c r="AK66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL66" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM66" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN66" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AO66" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="AP66" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Italian red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ66" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby to garnet"],"nose":["medium to pronounced intensity","black cherry","black plum","earth","smoke","dried herbs"],"palate":["dry","high acidity","full body","medium to high alcohol","high tannin","black fruit","earth","firm tannin"],"quality":["very good to outstanding; Taurasi is the benchmark for Aglianico"],"ageing":["long ageing potential"],"diagnostic_features":["taurasi_aglianico_core","darker and more southern than Nebbiolo","more black-fruited than Sangiovese"]}</t>
+        </is>
+      </c>
+      <c r="AR66" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["southern Italian premium red","Aglianico structure","Taurasi benchmark"],"learning_objectives":["identify Aglianico power","separate Taurasi from Sangiovese and Nebbiolo","connect southern Italy to ageworthy reds"],"typical_misconceptions":["southern Italy only makes soft fruity reds","Aglianico is low acid","all Italian ageworthy reds are Nebbiolo"],"mentor_focus":["ask for high tannin and acidity with dark fruit"],"exam_traps":["calling Taurasi Barolo from tannin alone","forgetting Campania reds"],"memory_hooks":["Taurasi is southern Italy's stern Aglianico benchmark"],"comparison_styles":["Barolo","Brunello di Montalcino","Left Bank Bordeaux"]}</t>
+        </is>
+      </c>
+      <c r="AS66" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_060","SAT_WINE_064"],"frequently_confused_with":["SAT_WINE_060","SAT_WINE_064"],"distinguishing_features":["darker and more southern than Nebbiolo","more black-fruited than Sangiovese","Aglianico benchmark Taurasi"]}</t>
+        </is>
+      </c>
+      <c r="AT66" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Aglianico is the most prestigious black grape of southern Italy","Taurasi DOCG is its best expression","Aglianico is a key Campanian red"],"mentor_hints":["Ask if the student can name a southern Italian ageworthy red.","Use Taurasi as the Aglianico anchor."],"student_traps":["forgetting Taurasi","confusing all high-tannin Italian reds with Barolo"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU66" t="inlineStr">
+        <is>
+          <t>["taurasi_aglianico_core"]</t>
+        </is>
+      </c>
+      <c r="AV66" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW66" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["12451-12456"],"line_reference":["12451-12456"],"evidence":["Aglianico is the most prestigious black grape of the south.","Aglianico is grown in a number of regions but is at its best in Taurasi DOCG."]}</t>
+        </is>
+      </c>
+      <c r="AX66" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-11-BATCH-008","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY66" t="inlineStr">
+        <is>
+          <t>29 Southern Italy</t>
+        </is>
+      </c>
+      <c r="AZ66" t="inlineStr">
+        <is>
+          <t>Campania - Aglianico / Taurasi</t>
+        </is>
+      </c>
+      <c r="BA66" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="BB66" t="inlineStr">
+        <is>
+          <t>["12451-12456"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add Batch 009 Spain Portugal red profiles
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -17962,6 +17962,1366 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SAT_WINE_066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Tintos España / Portugal</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Rioja Reserva</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Rioja Reserva</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Rioja Reserva</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Rioja</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Rioja Alta / Rioja Alavesa / Rioja Oriental</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Rioja DOCa</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>["Tempranillo","Garnacha","Mazuelo","Graciano"]</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>moderated by Atlantic influence in western Rioja with warmer Rioja Oriental</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>500 to 800 metre vineyards in western subregions</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>not specified by WSET; subregion and altitude are key</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>["Tempranillo is main component of most blends","Garnacha adds body and alcohol","Mazuelo and Graciano support blends"]</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>["traditional fermentation for long-term wines","oak maturation has defining role","American oak traditionally gives vanilla"]</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>American oak traditional; French and other European oak increasingly used</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>medium ruby to garnet</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>["red cherry","strawberry","vanilla","dill","leather"]</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>["red fruit","vanilla oak","spice","smooth tannin"]</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>very good to outstanding for top aged Rioja</t>
+        </is>
+      </c>
+      <c r="AB67" t="inlineStr">
+        <is>
+          <t>medium to long ageing</t>
+        </is>
+      </c>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>["medium ruby to garnet","medium to pronounced intensity","red cherry","strawberry","vanilla","dill","leather","dry","medium to high acidity","medium to full body","medium to high alcohol","medium tannin","red fruit","vanilla oak","spice","smooth tannin"]</t>
+        </is>
+      </c>
+      <c r="AD67" t="inlineStr">
+        <is>
+          <t>["Tempranillo is the main Rioja component","Garnacha adds body and alcohol","oak maturation is defining in Rioja"]</t>
+        </is>
+      </c>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t>["all Spanish Tempranillo tastes identical","vanilla means New World","Garnacha is never in Rioja"]</t>
+        </is>
+      </c>
+      <c r="AF67" t="inlineStr">
+        <is>
+          <t>["Ask if oak character is American vanilla or modern spice.","Use blend roles as debrief."]</t>
+        </is>
+      </c>
+      <c r="AG67" t="inlineStr">
+        <is>
+          <t>["medium ruby to garnet","red cherry","strawberry","vanilla","dill","leather","dry","medium to high acidity","medium to full body","medium to high alcohol","medium tannin","red fruit","vanilla oak","spice","smooth tannin","more vanilla-oak and red-fruited than Ribera","less black-fruited and tannic than Priorat","Rioja subregion blend context"]</t>
+        </is>
+      </c>
+      <c r="AH67" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI67" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Rioja evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ67" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Spain - Practica 066</t>
+        </is>
+      </c>
+      <c r="AK67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL67" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM67" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN67" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO67" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP67" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Spain and Portugal red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ67" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium ruby to garnet"],"nose":["medium to pronounced intensity","red cherry","strawberry","vanilla","dill","leather"],"palate":["dry","medium to high acidity","medium to full body","medium to high alcohol","medium tannin","red fruit","vanilla oak","spice"],"quality":["very good to outstanding for top aged Rioja"],"ageing":["medium to long ageing"],"diagnostic_features":["rioja_tempranillo_core","more vanilla-oak and red-fruited than Ribera","less black-fruited and tannic than Priorat"]}</t>
+        </is>
+      </c>
+      <c r="AR67" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Rioja oak identity","Tempranillo blend structure","Spanish age category logic"],"learning_objectives":["identify oak-aged Rioja","separate Rioja from Ribera del Duero","connect American oak to vanilla"],"typical_misconceptions":["all Spanish Tempranillo tastes identical","vanilla means New World","Garnacha is never in Rioja"],"mentor_focus":["ask whether red fruit and vanilla oak point to Rioja"],"exam_traps":["calling Rioja Ribera from Tempranillo alone","overlooking blend roles"],"memory_hooks":["Rioja is Tempranillo red fruit framed by oak"],"comparison_styles":["Ribera del Duero","Barbera d'Asti"]}</t>
+        </is>
+      </c>
+      <c r="AS67" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_067"],"frequently_confused_with":["SAT_WINE_067"],"distinguishing_features":["more vanilla-oak and red-fruited than Ribera","less black-fruited and tannic than Priorat","Rioja subregion blend context"]}</t>
+        </is>
+      </c>
+      <c r="AT67" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Tempranillo is the main Rioja component","Garnacha adds body and alcohol","oak maturation is defining in Rioja"],"mentor_hints":["Ask if oak character is American vanilla or modern spice.","Use blend roles as debrief."],"student_traps":["confusing Rioja with Ribera","ignoring oak maturation"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU67" t="inlineStr">
+        <is>
+          <t>["rioja_tempranillo_core"]</t>
+        </is>
+      </c>
+      <c r="AV67" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW67" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13026-13064"],"line_reference":["13026-13064"],"evidence":["Tempranillo is the main component of most Rioja blends giving red fruit and medium tannin; Garnacha adds body and alcohol.","Oak maturation has a defining role in Rioja, traditionally American oak with pronounced vanilla."]}</t>
+        </is>
+      </c>
+      <c r="AX67" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-12-BATCH-009","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY67" t="inlineStr">
+        <is>
+          <t>30 Spain</t>
+        </is>
+      </c>
+      <c r="AZ67" t="inlineStr">
+        <is>
+          <t>Rioja</t>
+        </is>
+      </c>
+      <c r="BA67" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="BB67" t="inlineStr">
+        <is>
+          <t>["13026-13064"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>SAT_WINE_067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Tintos España / Portugal</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Ribera del Duero</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Ribera del Duero</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Ribera del Duero</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Ribera del Duero</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Duero Valley</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Ribera del Duero DO</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>["Tempranillo"]</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>continental, cut off from maritime influence with hot dry summers and very cold winters</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>high Meseta Central vineyards, some over 850 metres</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>not specified by WSET; altitude and continental isolation are key</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>["DO for red and rosé only","Tempranillo is dominant and often sole grape in best reds","cool nights retain acidity and fresh fruit"]</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>["long macerations accentuate concentration and tannin","shorter ageing in new oak barrels increasingly French","deeply coloured concentrated style"]</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>new oak, increasingly French</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>deep ruby</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>["black cherry","blackberry","plum","vanilla","toast"]</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>["black fruit","firm tannin","new oak spice","fresh acidity"]</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>very good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB68" t="inlineStr">
+        <is>
+          <t>long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>["deep ruby","medium to pronounced intensity","black cherry","blackberry","plum","vanilla","toast","dry","medium to high acidity","full body","medium to high alcohol","high tannin","black fruit","firm tannin","new oak spice","fresh acidity"]</t>
+        </is>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>["Ribera is mainly red wine","Tempranillo is dominant","best wines are dark with high tannin"]</t>
+        </is>
+      </c>
+      <c r="AE68" t="inlineStr">
+        <is>
+          <t>["Ribera is just Rioja without oak","high alcohol means low acidity","Tempranillo always has medium tannin"]</t>
+        </is>
+      </c>
+      <c r="AF68" t="inlineStr">
+        <is>
+          <t>["Ask if fruit/tannin profile is darker than Rioja.","Use altitude as the balancing clue."]</t>
+        </is>
+      </c>
+      <c r="AG68" t="inlineStr">
+        <is>
+          <t>["deep ruby","black cherry","blackberry","plum","vanilla","toast","dry","medium to high acidity","full body","medium to high alcohol","high tannin","black fruit","firm tannin","new oak spice","fresh acidity","darker and more tannic than Rioja","Tempranillo-dominant rather than Garnacha/Cariñena Priorat","high Meseta altitude"]</t>
+        </is>
+      </c>
+      <c r="AH68" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI68" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Ribera del Duero evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ68" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Spain - Practica 067</t>
+        </is>
+      </c>
+      <c r="AK68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL68" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM68" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN68" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO68" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP68" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Spain and Portugal red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ68" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby"],"nose":["medium to pronounced intensity","black cherry","blackberry","plum","vanilla","toast"],"palate":["dry","medium to high acidity","full body","medium to high alcohol","high tannin","black fruit","firm tannin","new oak spice"],"quality":["very good to outstanding"],"ageing":["long ageing potential"],"diagnostic_features":["ribera_tempranillo_core","darker and more tannic than Rioja","Tempranillo-dominant rather than Garnacha/Cariñena Priorat"]}</t>
+        </is>
+      </c>
+      <c r="AR68" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["high-altitude Tempranillo","Ribera concentration","new-oak structure"],"learning_objectives":["identify Ribera del Duero","separate Ribera from Rioja","link altitude to freshness"],"typical_misconceptions":["Ribera is just Rioja without oak","high alcohol means low acidity","Tempranillo always has medium tannin"],"mentor_focus":["ask whether darker fruit and tannin exceed Rioja"],"exam_traps":["calling all Tempranillo Rioja","missing altitude"],"memory_hooks":["Ribera is high-altitude Tempranillo with grip"],"comparison_styles":["Rioja Reserva","Priorat"]}</t>
+        </is>
+      </c>
+      <c r="AS68" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_066","SAT_WINE_068"],"frequently_confused_with":["SAT_WINE_066","SAT_WINE_068"],"distinguishing_features":["darker and more tannic than Rioja","Tempranillo-dominant rather than Garnacha/Cariñena Priorat","high Meseta altitude"]}</t>
+        </is>
+      </c>
+      <c r="AT68" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Ribera is mainly red wine","Tempranillo is dominant","best wines are dark with high tannin"],"mentor_hints":["Ask if fruit/tannin profile is darker than Rioja.","Use altitude as the balancing clue."],"student_traps":["defaulting to Rioja","forgetting Ribera's altitude"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU68" t="inlineStr">
+        <is>
+          <t>["ribera_tempranillo_core"]</t>
+        </is>
+      </c>
+      <c r="AV68" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW68" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13241-13274"],"line_reference":["13241-13274"],"evidence":["Ribera del Duero has high-altitude vineyards with cool nights that retain acidity and fresh fruit.","Tempranillo dominates the best reds, typically dark in colour with high tannin; many use long maceration and new oak."]}</t>
+        </is>
+      </c>
+      <c r="AX68" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-12-BATCH-009","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY68" t="inlineStr">
+        <is>
+          <t>30 Spain</t>
+        </is>
+      </c>
+      <c r="AZ68" t="inlineStr">
+        <is>
+          <t>Ribera del Duero</t>
+        </is>
+      </c>
+      <c r="BA68" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="BB68" t="inlineStr">
+        <is>
+          <t>["13241-13274"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SAT_WINE_068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Tintos España / Portugal</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Priorat</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Priorat</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Priorat</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Priorat</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Catalunya inland hills</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Priorat DOCa</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>["Garnacha","Carinena"]</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>long hot dry summers and very low rainfall</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>steep inland hills from Tarragona</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>llicorella red slate with mica</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>["old Garnacha and Cariñena vines","bush vines and steep slopes make mechanisation difficult","low nutrient soils and old vines give low yields"]</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>["concentrated red winemaking","new French oak commonly gives toasty aromas","some Cabernet Sauvignon may be added"]</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>new French oak common</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>deep ruby</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>["black fruit","dried herbs","spice","toast","mineral"]</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>["concentrated black fruit","firm tannin","toasty oak","warm alcohol"]</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>very good to outstanding; intense and rarely cheap</t>
+        </is>
+      </c>
+      <c r="AB69" t="inlineStr">
+        <is>
+          <t>long ageing potential</t>
+        </is>
+      </c>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>["deep ruby","medium to pronounced intensity","black fruit","dried herbs","spice","toast","mineral","dry","medium to high acidity","full body","high alcohol","high tannin","concentrated black fruit","firm tannin","toasty oak","warm alcohol"]</t>
+        </is>
+      </c>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>["Priorat uses old Garnacha and Cariñena","llicorella soils help ripening and water retention","red Priorat is deep, tannic and concentrated"]</t>
+        </is>
+      </c>
+      <c r="AE69" t="inlineStr">
+        <is>
+          <t>["Priorat is just Garnacha like simple Spain","new French oak means Bordeaux","all Catalunya reds are light"]</t>
+        </is>
+      </c>
+      <c r="AF69" t="inlineStr">
+        <is>
+          <t>["Ask if the structure is Priorat intensity rather than Ribera Tempranillo.","Use llicorella as a memory hook."]</t>
+        </is>
+      </c>
+      <c r="AG69" t="inlineStr">
+        <is>
+          <t>["deep ruby","black fruit","dried herbs","spice","toast","mineral","dry","medium to high acidity","full body","high alcohol","high tannin","concentrated black fruit","firm tannin","toasty oak","warm alcohol","Garnacha/Cariñena rather than Tempranillo","llicorella slate clue","more black-fruit and new French oak intensity"]</t>
+        </is>
+      </c>
+      <c r="AH69" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI69" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Priorat evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ69" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Spain - Practica 068</t>
+        </is>
+      </c>
+      <c r="AK69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL69" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM69" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN69" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO69" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="AP69" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Spain and Portugal red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ69" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby"],"nose":["medium to pronounced intensity","black fruit","dried herbs","spice","toast","mineral"],"palate":["dry","medium to high acidity","full body","high alcohol","high tannin","concentrated black fruit","firm tannin","toasty oak"],"quality":["very good to outstanding; intense and rarely cheap"],"ageing":["long ageing potential"],"diagnostic_features":["priorat_core","Garnacha/Cariñena rather than Tempranillo","llicorella slate clue"]}</t>
+        </is>
+      </c>
+      <c r="AR69" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Priorat intensity","llicorella soils","old-vine Garnacha/Cariñena"],"learning_objectives":["identify Priorat structure","connect low yields to intensity","separate Priorat from Ribera"],"typical_misconceptions":["Priorat is just Garnacha like simple Spain","new French oak means Bordeaux","all Catalunya reds are light"],"mentor_focus":["ask for deep colour, high tannin, black fruit and heat"],"exam_traps":["calling Priorat Ribera","missing Cariñena role"],"memory_hooks":["Priorat is slate, old vines and concentrated black fruit"],"comparison_styles":["Ribera del Duero","Chateauneuf-du-Pape Rouge"]}</t>
+        </is>
+      </c>
+      <c r="AS69" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_067","SAT_WINE_057"],"frequently_confused_with":["SAT_WINE_067","SAT_WINE_057"],"distinguishing_features":["Garnacha/Cariñena rather than Tempranillo","llicorella slate clue","more black-fruit and new French oak intensity"]}</t>
+        </is>
+      </c>
+      <c r="AT69" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Priorat uses old Garnacha and Cariñena","llicorella soils help ripening and water retention","red Priorat is deep, tannic and concentrated"],"mentor_hints":["Ask if the structure is Priorat intensity rather than Ribera Tempranillo.","Use llicorella as a memory hook."],"student_traps":["missing Cariñena","overlooking soil clue"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU69" t="inlineStr">
+        <is>
+          <t>["priorat_core"]</t>
+        </is>
+      </c>
+      <c r="AV69" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW69" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13158-13238"],"line_reference":["13158-13238"],"evidence":["Priorat has old Garnacha and Cariñena vines, llicorella red slate soils, steep slopes and low yields.","Red Priorat is deeply coloured, high in tannins, medium to high alcohol, concentrated black fruit and often toasty new French oak."]}</t>
+        </is>
+      </c>
+      <c r="AX69" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-12-BATCH-009","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY69" t="inlineStr">
+        <is>
+          <t>30 Spain</t>
+        </is>
+      </c>
+      <c r="AZ69" t="inlineStr">
+        <is>
+          <t>Priorat</t>
+        </is>
+      </c>
+      <c r="BA69" t="inlineStr">
+        <is>
+          <t>135-136</t>
+        </is>
+      </c>
+      <c r="BB69" t="inlineStr">
+        <is>
+          <t>["13158-13238"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SAT_WINE_069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Tintos España / Portugal</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Douro Red</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Douro Red</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Douro Red</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Douro</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Douro Valley</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Douro DOC</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>["Touriga Nacional","Touriga Franca","Tinta Roriz"]</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>hot inland valley east of Porto with Port-influenced viticulture</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>steep Douro valley vineyards</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>not specified here; Douro slope context is key</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>["same principal varieties as Port","Touriga Nacional is highest-quality and low yielding","unfortified wines have always been made"]</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>["dry red winemaking from Port varieties","best examples may mature in new oak","full-bodied black-fruited style"]</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>new oak often gives subtle toasty aromas in best examples</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>deep ruby</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>["blackberry","black plum","violet","toast","spice"]</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>["rich black fruit","ripe tannin","toasty oak","full body"]</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>very good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB70" t="inlineStr">
+        <is>
+          <t>medium to long ageing</t>
+        </is>
+      </c>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t>["deep ruby","medium to pronounced intensity","blackberry","black plum","violet","toast","spice","dry","medium to high acidity","full body","high alcohol","high tannin","rich black fruit","ripe tannin","toasty oak","full body"]</t>
+        </is>
+      </c>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>["Douro is oldest demarcated region","unfortified reds rely on Port varieties","red Douro is deep, full and tannic"]</t>
+        </is>
+      </c>
+      <c r="AE70" t="inlineStr">
+        <is>
+          <t>["Douro only makes Port","Touriga Nacional is only for fortified wine","Portugal reds are light"]</t>
+        </is>
+      </c>
+      <c r="AF70" t="inlineStr">
+        <is>
+          <t>["Ask if alcohol/fortification is observed or assumed.","Use Touriga Nacional as anchor."]</t>
+        </is>
+      </c>
+      <c r="AG70" t="inlineStr">
+        <is>
+          <t>["deep ruby","blackberry","black plum","violet","toast","spice","dry","medium to high acidity","full body","high alcohol","high tannin","rich black fruit","ripe tannin","toasty oak","full body","fuller and blacker than Dão","Portuguese varieties rather than Priorat Garnacha/Cariñena","not fortified"]</t>
+        </is>
+      </c>
+      <c r="AH70" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI70" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Douro evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ70" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Portugal - Practica 069</t>
+        </is>
+      </c>
+      <c r="AK70" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AL70" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM70" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AN70" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO70" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="AP70" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Spain and Portugal red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ70" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby"],"nose":["medium to pronounced intensity","blackberry","black plum","violet","toast","spice"],"palate":["dry","medium to high acidity","full body","high alcohol","high tannin","rich black fruit","ripe tannin","toasty oak"],"quality":["very good to outstanding"],"ageing":["medium to long ageing"],"diagnostic_features":["douro_red_core","fuller and blacker than Dão","Portuguese varieties rather than Priorat Garnacha/Cariñena"]}</t>
+        </is>
+      </c>
+      <c r="AR70" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Portuguese dry red from Port varieties","Touriga Nacional quality","Douro black-fruit structure"],"learning_objectives":["identify Douro red","separate dry Douro from Port","connect varieties to structure"],"typical_misconceptions":["Douro only makes Port","Touriga Nacional is only for fortified wine","Portugal reds are light"],"mentor_focus":["ask whether full dry red uses Port grapes"],"exam_traps":["calling Douro Port","forgetting unfortified Douro"],"memory_hooks":["Douro red is dry table wine from Port's powerhouse grapes"],"comparison_styles":["Dao Red","Priorat"]}</t>
+        </is>
+      </c>
+      <c r="AS70" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_070","SAT_WINE_068"],"frequently_confused_with":["SAT_WINE_070","SAT_WINE_068"],"distinguishing_features":["fuller and blacker than Dão","Portuguese varieties rather than Priorat Garnacha/Cariñena","not fortified"]}</t>
+        </is>
+      </c>
+      <c r="AT70" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Douro is oldest demarcated region","unfortified reds rely on Port varieties","red Douro is deep, full and tannic"],"mentor_hints":["Ask if alcohol/fortification is observed or assumed.","Use Touriga Nacional as anchor."],"student_traps":["assuming all Douro is Port","missing dry red category"],"revision_priority":"high"}</t>
+        </is>
+      </c>
+      <c r="AU70" t="inlineStr">
+        <is>
+          <t>["douro_red_core"]</t>
+        </is>
+      </c>
+      <c r="AV70" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW70" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13529-13550"],"line_reference":["13529-13550"],"evidence":["Douro unfortified reds rely on the same principal varieties as Port, including Touriga Nacional, Touriga Franca and Tinta Roriz.","Red Douro wines are deeply coloured, full-bodied, high in ripe tannins and rich black fruit, with best examples showing new oak toast."]}</t>
+        </is>
+      </c>
+      <c r="AX70" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-12-BATCH-009","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY70" t="inlineStr">
+        <is>
+          <t>31 Portugal</t>
+        </is>
+      </c>
+      <c r="AZ70" t="inlineStr">
+        <is>
+          <t>Douro</t>
+        </is>
+      </c>
+      <c r="BA70" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="BB70" t="inlineStr">
+        <is>
+          <t>["13529-13550"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SAT_WINE_070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Tintos España / Portugal</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Dao Red</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Dao Red</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Dao Red</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>TINTO</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Dao</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Central Portugal</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Dao DOC</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>["Touriga Nacional","Tinta Roriz","Jaen","Alfrocheiro"]</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>mountainous area with cold wet winters, warm dry summers and significant day-night variation</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>gentle hills and slopes between 200 and 400 metres</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>not specified by WSET; mountain slope setting is key</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>["vineyards lie between 200 and 400 metres","day-night variation provides excellent grape conditions","new high-quality plantings include Touriga Nacional, Tinta Roriz, Jaen and Alfrocheiro"]</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>["dry red winemaking preserving delicate red fruit","oak may be used but delicacy is central","softer tannin style than Douro"]</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>variable; oak not the defining marker</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>soft to medium</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>medium ruby</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>["red cherry","red plum","strawberry","blackberry"]</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>["delicate red fruit","high acidity","soft tannin","fresh finish"]</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t>short to medium ageing</t>
+        </is>
+      </c>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>["medium ruby","medium to pronounced intensity","red cherry","red plum","strawberry","blackberry","dry","high acidity","medium body","medium alcohol","soft to medium tannin","delicate red fruit","high acidity","soft tannin","fresh finish"]</t>
+        </is>
+      </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>["Dão lies at 200 to 400 metres","Dão reds show delicate red fruit, soft tannin and high acidity","Touriga Nacional, Tinta Roriz, Jaen and Alfrocheiro are planted"]</t>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr">
+        <is>
+          <t>["Portuguese reds are all full-bodied Douro","soft tannin means low quality","Dão is only white Encruzado"]</t>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t>["Ask if tannin is actually ripe-high or soft-medium.","Use Dão as the Portuguese elegance contrast."]</t>
+        </is>
+      </c>
+      <c r="AG71" t="inlineStr">
+        <is>
+          <t>["medium ruby","red cherry","red plum","strawberry","blackberry","dry","high acidity","medium body","medium alcohol","soft to medium tannin","delicate red fruit","high acidity","soft tannin","fresh finish","lighter and softer than Douro","higher acidity and delicate red fruit","mountainous Dão source"]</t>
+        </is>
+      </c>
+      <c r="AH71" t="inlineStr">
+        <is>
+          <t>["do not expose identity fields in blind render profiles","do not add markers that contradict WSET style evidence"]</t>
+        </is>
+      </c>
+      <c r="AI71" t="inlineStr">
+        <is>
+          <t>Profile uses WSET Dão evidence; SAT sensory calibration uses standard style knowledge where WSET is less granular.</t>
+        </is>
+      </c>
+      <c r="AJ71" t="inlineStr">
+        <is>
+          <t>Vino Tinto - Portugal - Practica 070</t>
+        </is>
+      </c>
+      <c r="AK71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AL71" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM71" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AN71" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO71" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="AP71" t="inlineStr">
+        <is>
+          <t>{"wset_primary":["Selected Spain and Portugal red profiles are explicitly described in WSET3_rebuilt.md."],"standard_wine_knowledge":["SAT sensory calibration uses accepted style norms where WSET is less granular."],"derived_from_style":["Difficulty and comparisons derive from WSET regional and grape contrasts."],"inferred_high_confidence":["Mentor hints and memory hooks are pedagogical inferences."]}</t>
+        </is>
+      </c>
+      <c r="AQ71" t="inlineStr">
+        <is>
+          <t>{"appearance":["medium ruby"],"nose":["medium to pronounced intensity","red cherry","red plum","strawberry","blackberry"],"palate":["dry","high acidity","medium body","medium alcohol","soft to medium tannin","delicate red fruit","high acidity","soft tannin"],"quality":["good to very good"],"ageing":["short to medium ageing"],"diagnostic_features":["dao_red_core","lighter and softer than Douro","higher acidity and delicate red fruit"]}</t>
+        </is>
+      </c>
+      <c r="AR71" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Dão delicacy","Portuguese mountain reds","soft tannin high acidity"],"learning_objectives":["identify Dão red","separate Dão from Douro","connect diurnal range to acidity"],"typical_misconceptions":["Portuguese reds are all full-bodied Douro","soft tannin means low quality","Dão is only white Encruzado"],"mentor_focus":["ask if high acidity and soft tannin suggest Dão"],"exam_traps":["calling Dão Douro","overstating body and tannin"],"memory_hooks":["Dão is Portugal's fresher mountain red counterpoint to Douro"],"comparison_styles":["Douro Red","Rioja Reserva"]}</t>
+        </is>
+      </c>
+      <c r="AS71" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_069"],"frequently_confused_with":["SAT_WINE_069","SAT_WINE_066"],"distinguishing_features":["lighter and softer than Douro","higher acidity and delicate red fruit","mountainous Dão source"]}</t>
+        </is>
+      </c>
+      <c r="AT71" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Dão lies at 200 to 400 metres","Dão reds show delicate red fruit, soft tannin and high acidity","Touriga Nacional, Tinta Roriz, Jaen and Alfrocheiro are planted"],"mentor_hints":["Ask if tannin is actually ripe-high or soft-medium.","Use Dão as the Portuguese elegance contrast."],"student_traps":["confusing Dão with Douro","ignoring high acidity"],"revision_priority":"medium"}</t>
+        </is>
+      </c>
+      <c r="AU71" t="inlineStr">
+        <is>
+          <t>["dao_red_core"]</t>
+        </is>
+      </c>
+      <c r="AV71" t="inlineStr">
+        <is>
+          <t>{"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"knowledge_summary":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"canonical_id":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wine_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"wine_style":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_name":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"display_label":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"PUBLIC"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"climate":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"DERIVED_FROM_STYLE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"body":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"sat_constraints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"PUBLIC"},"reusable_knowledge_refs":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"TRAINING"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"expected_sat_observations":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"INFERRED_HIGH_CONFIDENCE","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"SERVER_ONLY"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW71" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","line_references":["13555-13572"],"line_reference":["13555-13572"],"evidence":["Dão vineyards are in a mountainous area at 200 to 400 metres with significant day-night temperature variation.","Dão reds often display delicate red fruit aromas, soft tannins and high acidity, with varieties including Touriga Nacional, Tinta Roriz, Jaen and Alfrocheiro."]}</t>
+        </is>
+      </c>
+      <c r="AX71" t="inlineStr">
+        <is>
+          <t>{"title":"WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","batch":"CWP-12-BATCH-009","schema_version":"CWP-02"}</t>
+        </is>
+      </c>
+      <c r="AY71" t="inlineStr">
+        <is>
+          <t>31 Portugal</t>
+        </is>
+      </c>
+      <c r="AZ71" t="inlineStr">
+        <is>
+          <t>Dão</t>
+        </is>
+      </c>
+      <c r="BA71" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="BB71" t="inlineStr">
+        <is>
+          <t>["13555-13572"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add WSET official sparkling wines batch 011
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -25578,6 +25578,1910 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>SAT_WINE_094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>WSET Official Sparkling Wines</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Champagne Non-Vintage</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Traditional-method non-vintage Champagne</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Champagne Non-Vintage</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>ESPUMOSO</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Champagne</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Champagne</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Champagne AC</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>["Chardonnay","Pinot Noir","Meunier"]</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>cool continental Champagne climate with high acid base wines and vintage variability</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>slope exposure and village classification are more diagnostic than a single altitude value</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>chalk-dominant soils with water retention and drainage benefits</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>["cool-climate disease and frost pressure","high-acid grapes suitable for sparkling base wine"]</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>["traditional method","second fermentation in bottle","blend across varieties, villages and reserve wines","lees ageing before disgorgement","dosage after disgorgement"]</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>usually limited; some base wines or reserve components may see old oak depending on producer</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>brut to extra brut commonly, with dosage balancing high acidity</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>["green apple","lemon","brioche","toast","yeast"]</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>["citrus","apple","biscuit","bread dough","toast"]</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB95" t="inlineStr">
+        <is>
+          <t>drink now; better examples can develop autolytic and tertiary complexity</t>
+        </is>
+      </c>
+      <c r="AC95" t="inlineStr">
+        <is>
+          <t>["pale lemon","persistent mousse","high acidity","dry to off-dry balance","citrus and apple fruit","brioche or toast autolysis"]</t>
+        </is>
+      </c>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>["Champagne non-vintage is an essential WSET tasting recommendation","non-vintage style is built through blending and reserve wines","traditional method and lees ageing create autolytic notes"]</t>
+        </is>
+      </c>
+      <c r="AE95" t="inlineStr">
+        <is>
+          <t>["assuming all Champagne is vintage","missing dosage when judging dryness","calling every autolytic sparkling wine Champagne"]</t>
+        </is>
+      </c>
+      <c r="AF95" t="inlineStr">
+        <is>
+          <t>["Separate method character from origin: mousse and autolysis are not enough without Champagne-level acidity and profile."]</t>
+        </is>
+      </c>
+      <c r="AG95" t="inlineStr">
+        <is>
+          <t>["pale lemon","persistent bubbles","high acidity","brut","green apple","lemon","brioche","toast","bread dough","yeast"]</t>
+        </is>
+      </c>
+      <c r="AH95" t="inlineStr">
+        <is>
+          <t>["Do not reveal Champagne, France, grape varieties, vintage status or appellation in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI95" t="inlineStr">
+        <is>
+          <t>Chosen because WSET specifies Champagne non-vintage as an imprescindible sparkling tasting style.</t>
+        </is>
+      </c>
+      <c r="AJ95" t="inlineStr">
+        <is>
+          <t>Practica WSET 094 - Vino espumoso</t>
+        </is>
+      </c>
+      <c r="AK95" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL95" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM95" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN95" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO95" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP95" t="inlineStr">
+        <is>
+          <t>Cool-climate traditional-method sparkling wine with high acidity, fine mousse, citrus/apple fruit and autolytic bread or toast notes.</t>
+        </is>
+      </c>
+      <c r="AQ95" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon","persistent fine bubbles"],"nose":["green apple","lemon","brioche","toast"],"palate":["dry to off-dry","high acidity","light to medium body","persistent mousse"],"quality":["good to outstanding","autolytic complexity"],"ageing":["reserve wine and lees ageing add complexity"],"diagnostic_features":["traditional method","high acidity","autolysis","non-vintage blend"]}</t>
+        </is>
+      </c>
+      <c r="AR95" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["traditional method","non-vintage blending","lees autolysis","dosage balance"],"learning_objectives":["identify Champagne NV as a benchmark sparkling style","connect reserve wines to consistency","explain high acid base wine logic"],"typical_misconceptions":["assuming all Champagne is vintage","missing dosage when judging dryness","calling every autolytic sparkling wine Champagne"],"mentor_focus":["Separate method character from origin: mousse and autolysis are not enough without Champagne-level acidity and profile."],"exam_traps":["confusing Cava or Cremant with Champagne solely from autolysis"],"memory_hooks":["NV equals house style plus reserve wine consistency"],"comparison_styles":["Cava","Cremant","traditional method New World sparkling"]}</t>
+        </is>
+      </c>
+      <c r="AS95" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_095","SAT_WINE_096","SAT_WINE_097","SAT_WINE_100"],"frequently_confused_with":["Cava","Cremant","premium New World traditional method sparkling"],"distinguishing_features":["higher acidity and chalky cool-climate tension","reserve wine complexity","fine persistent mousse"]}</t>
+        </is>
+      </c>
+      <c r="AT95" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Champagne non-vintage is an essential WSET tasting recommendation","non-vintage style is built through blending and reserve wines","traditional method and lees ageing create autolytic notes"],"mentor_hints":["Separate method character from origin: mousse and autolysis are not enough without Champagne-level acidity and profile."],"student_traps":["assuming all Champagne is vintage","missing dosage when judging dryness","calling every autolytic sparkling wine Champagne"],"revision_priority":"High: official WSET essential sparkling tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU95" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","cool_climate_high_acid_white","premium_chardonnay_winemaking"]</t>
+        </is>
+      </c>
+      <c r="AV95" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW95" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 42 / Champagne","line_references":["17214-17398"],"evidence":"Specification recommends Champagne non-vintage; book explains Champagne AC, traditional method, blending, quality levels and sweetness."}</t>
+        </is>
+      </c>
+      <c r="AX95" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY95" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Sparkling wines</t>
+        </is>
+      </c>
+      <c r="AZ95" t="inlineStr">
+        <is>
+          <t>Champagne / Champagne AC</t>
+        </is>
+      </c>
+      <c r="BA95" t="inlineStr">
+        <is>
+          <t>WSET specification line 1909; WSET3 rebuilt lines 17214-17398</t>
+        </is>
+      </c>
+      <c r="BB95" t="inlineStr">
+        <is>
+          <t>["1909-1909"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>SAT_WINE_095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>WSET Official Sparkling Wines</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Champagne Vintage / Prestige Cuvee</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Premium vintage or prestige cuvee Champagne</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Champagne Vintage / Prestige Cuvee</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>ESPUMOSO</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Champagne</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Champagne</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Champagne AC</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>["Chardonnay","Pinot Noir","Meunier"]</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>cool continental Champagne climate with vintage variation important for declared vintage wines</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>best village and cru sites are more diagnostic than a single altitude value</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>chalk and limestone-influenced Champagne soils</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>["fruit selection from high-quality sites","vintage declaration only in suitable years for vintage styles"]</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>["traditional method","longer lees ageing than many non-vintage wines","vintage or prestige cuvee selection","possible oak or reserve component depending on house style","dosage after disgorgement"]</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>usually subtle if used; prestige cuvees may include barrel-fermented base wine components</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>brut commonly</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>pale lemon to medium gold</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>["lemon","apple","brioche","toast","almond","honey"]</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>["citrus","ripe apple","pastry","toast","nut","cream"]</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>very good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB96" t="inlineStr">
+        <is>
+          <t>capable of bottle ageing with toast, nut and honey development</t>
+        </is>
+      </c>
+      <c r="AC96" t="inlineStr">
+        <is>
+          <t>["persistent mousse","high acidity","dry balance","ripe citrus and apple","pronounced autolysis","long finish"]</t>
+        </is>
+      </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>["WSET lists Champagne vintage or prestige cuvee as an optional tasting recommendation","vintage and prestige styles show greater concentration and ageing potential","quality level and lees influence should be explicit in SAT reasoning"]</t>
+        </is>
+      </c>
+      <c r="AE96" t="inlineStr">
+        <is>
+          <t>["treating prestige cuvee as simply older NV","forgetting that vintage Champagne depends on declared year conditions","overcalling sweetness because of richness"]</t>
+        </is>
+      </c>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>["Look for the same Champagne skeleton as NV, then ask whether concentration, autolysis and finish are elevated."]</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>["persistent bubbles","high acidity","brut","lemon","apple","brioche","toast","almond","honey","long finish"]</t>
+        </is>
+      </c>
+      <c r="AH96" t="inlineStr">
+        <is>
+          <t>["Do not reveal Champagne, France, vintage, prestige cuvee, grape varieties or appellation in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI96" t="inlineStr">
+        <is>
+          <t>Included because it is an official optional WSET sparkling tasting recommendation and fits cleanly within the sparkling batch.</t>
+        </is>
+      </c>
+      <c r="AJ96" t="inlineStr">
+        <is>
+          <t>Practica WSET 095 - Vino espumoso</t>
+        </is>
+      </c>
+      <c r="AK96" t="inlineStr">
+        <is>
+          <t>P1_WSET_RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="AL96" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM96" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AN96" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AO96" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP96" t="inlineStr">
+        <is>
+          <t>Premium traditional-method Champagne with high acidity, fine mousse, deeper autolysis, longer finish and stronger ageing potential.</t>
+        </is>
+      </c>
+      <c r="AQ96" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon to medium gold","fine persistent bubbles"],"nose":["citrus","ripe apple","brioche","toast","nut"],"palate":["dry","high acidity","medium body","creamy mousse","long finish"],"quality":["very good to outstanding","greater autolytic and bottle-age complexity"],"ageing":["can develop nutty, honeyed, toasty complexity"],"diagnostic_features":["traditional method","vintage or prestige selection","long lees ageing","premium Champagne concentration"]}</t>
+        </is>
+      </c>
+      <c r="AR96" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["vintage declaration","prestige cuvee selection","extended lees ageing","premium quality assessment"],"learning_objectives":["distinguish NV from vintage/prestige Champagne","explain concentration and ageing cues","connect finish length to quality"],"typical_misconceptions":["treating prestige cuvee as simply older NV","forgetting that vintage Champagne depends on declared year conditions","overcalling sweetness because of richness"],"mentor_focus":["Look for the same Champagne skeleton as NV, then ask whether concentration, autolysis and finish are elevated."],"exam_traps":["assuming all Champagne vintage is sweeter","confusing autolytic richness with low acidity"],"memory_hooks":["prestige/vintage equals Champagne skeleton plus more selection and time"],"comparison_styles":["Champagne Non-Vintage","Cremant","Cava"]}</t>
+        </is>
+      </c>
+      <c r="AS96" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_094","SAT_WINE_096","SAT_WINE_097"],"frequently_confused_with":["non-vintage Champagne","premium Cava","premium Cremant"],"distinguishing_features":["greater concentration","longer finish","more pronounced lees and bottle-age complexity"]}</t>
+        </is>
+      </c>
+      <c r="AT96" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["WSET lists Champagne vintage or prestige cuvee as an optional tasting recommendation","vintage and prestige styles show greater concentration and ageing potential","quality level and lees influence should be explicit in SAT reasoning"],"mentor_hints":["Look for the same Champagne skeleton as NV, then ask whether concentration, autolysis and finish are elevated."],"student_traps":["treating prestige cuvee as simply older NV","forgetting that vintage Champagne depends on declared year conditions","overcalling sweetness because of richness"],"revision_priority":"Medium-high: official WSET optional sparkling tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU96" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","cool_climate_high_acid_white","premium_chardonnay_winemaking"]</t>
+        </is>
+      </c>
+      <c r="AV96" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW96" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 42 / Champagne quality levels","line_references":["17158-17164","17355-17372"],"evidence":"Specification recommends vintage or prestige cuvee Champagne optionally; book explains vintage and prestige cuvee Champagne."}</t>
+        </is>
+      </c>
+      <c r="AX96" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY96" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Sparkling wines</t>
+        </is>
+      </c>
+      <c r="AZ96" t="inlineStr">
+        <is>
+          <t>Champagne / Champagne AC</t>
+        </is>
+      </c>
+      <c r="BA96" t="inlineStr">
+        <is>
+          <t>WSET specification line 1911; WSET3 rebuilt lines 17158-17164 and 17355-17372</t>
+        </is>
+      </c>
+      <c r="BB96" t="inlineStr">
+        <is>
+          <t>["1911-1911"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SAT_WINE_096</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>WSET Official Sparkling Wines</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Cremant</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Traditional-method French Cremant</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Cremant</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>ESPUMOSO</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Alsace / Burgundy / Loire</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>regional Cremant appellations</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Cremant d'Alsace / Cremant de Bourgogne / Cremant de Loire</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>["Chardonnay","Pinot Blanc","Chenin Blanc","Pinot Noir"]</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>varies by French region, generally producing fresh high-acid sparkling base wines</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>regional and producer dependent</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>varied limestone, clay and regional soils depending on Cremant appellation</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>["grape selection for sparkling base wine freshness","regional permitted varieties shape style"]</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>["traditional method","second fermentation in bottle","lees ageing","dosage after disgorgement"]</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>typically none or minimal</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>dry to off-dry depending on dosage</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>["apple","lemon","pear","bread dough","biscuit"]</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>["citrus","orchard fruit","biscuit","cream"]</t>
+        </is>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB97" t="inlineStr">
+        <is>
+          <t>generally for early drinking; best examples can gain some autolytic complexity</t>
+        </is>
+      </c>
+      <c r="AC97" t="inlineStr">
+        <is>
+          <t>["pale lemon","mousse","medium to high acidity","citrus or orchard fruit","subtle autolysis"]</t>
+        </is>
+      </c>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>["WSET lists Cremant as an optional sparkling tasting recommendation","Cremant uses traditional method but is not Champagne","regional grape choices can alter fruit profile"]</t>
+        </is>
+      </c>
+      <c r="AE97" t="inlineStr">
+        <is>
+          <t>["calling Cremant Champagne","expecting the same intensity or price tier as Champagne","ignoring regional grape signatures"]</t>
+        </is>
+      </c>
+      <c r="AF97" t="inlineStr">
+        <is>
+          <t>["Use method markers first, then keep the origin label generic until debrief."]</t>
+        </is>
+      </c>
+      <c r="AG97" t="inlineStr">
+        <is>
+          <t>["pale lemon","bubbles","medium acidity","high acidity","apple","pear","lemon","biscuit","bread dough","cream"]</t>
+        </is>
+      </c>
+      <c r="AH97" t="inlineStr">
+        <is>
+          <t>["Do not reveal Cremant, France, region, grape varieties or appellation in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI97" t="inlineStr">
+        <is>
+          <t>Included because Crémant is an official optional WSET sparkling recommendation and does not require a separate non-sparkling batch.</t>
+        </is>
+      </c>
+      <c r="AJ97" t="inlineStr">
+        <is>
+          <t>Practica WSET 096 - Vino espumoso</t>
+        </is>
+      </c>
+      <c r="AK97" t="inlineStr">
+        <is>
+          <t>P1_WSET_RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="AL97" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM97" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AN97" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO97" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP97" t="inlineStr">
+        <is>
+          <t>French traditional-method sparkling wine outside Champagne, typically fresh, dry, citrus or orchard-fruited with subtle autolysis.</t>
+        </is>
+      </c>
+      <c r="AQ97" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon","persistent bubbles"],"nose":["apple","pear","lemon","biscuit"],"palate":["dry to off-dry","medium to high acidity","light to medium body","mousse"],"quality":["good to very good","moderate autolytic complexity"],"ageing":["usually early drinking"],"diagnostic_features":["traditional method","French Cremant appellation","fresh fruit","subtle autolysis"]}</t>
+        </is>
+      </c>
+      <c r="AR97" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["traditional method outside Champagne","regional permitted varieties","lees-derived notes"],"learning_objectives":["differentiate Cremant from Champagne","recognize autolysis at lower intensity","explain regional variety variation"],"typical_misconceptions":["calling Cremant Champagne","expecting the same intensity or price tier as Champagne","ignoring regional grape signatures"],"mentor_focus":["Use method markers first, then keep the origin label generic until debrief."],"exam_traps":["over-identifying all autolytic sparkling as Champagne"],"memory_hooks":["Cremant equals traditional method France, outside Champagne"],"comparison_styles":["Champagne Non-Vintage","Cava","traditional method New World sparkling"]}</t>
+        </is>
+      </c>
+      <c r="AS97" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_094","SAT_WINE_097","SAT_WINE_100"],"frequently_confused_with":["Champagne","Cava","New World traditional method sparkling"],"distinguishing_features":["usually less intense than Champagne","regional grape variation","fresh fruit with moderate autolysis"]}</t>
+        </is>
+      </c>
+      <c r="AT97" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["WSET lists Cremant as an optional sparkling tasting recommendation","Cremant uses traditional method but is not Champagne","regional grape choices can alter fruit profile"],"mentor_hints":["Use method markers first, then keep the origin label generic until debrief."],"student_traps":["calling Cremant Champagne","expecting the same intensity or price tier as Champagne","ignoring regional grape signatures"],"revision_priority":"Medium-high: official WSET optional sparkling tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU97" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV97" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW97" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 42 / Sparkling wines from France","line_references":["17407-17422"],"evidence":"Specification recommends Cremant optionally; book identifies Cremant dAlsace, Cremant de Bourgogne and Cremant de Loire."}</t>
+        </is>
+      </c>
+      <c r="AX97" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY97" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Sparkling wines</t>
+        </is>
+      </c>
+      <c r="AZ97" t="inlineStr">
+        <is>
+          <t>Alsace / Burgundy / Loire / Cremant d'Alsace / Cremant de Bourgogne / Cremant de Loire</t>
+        </is>
+      </c>
+      <c r="BA97" t="inlineStr">
+        <is>
+          <t>WSET specification line 1913; WSET3 rebuilt lines 17407-17422</t>
+        </is>
+      </c>
+      <c r="BB97" t="inlineStr">
+        <is>
+          <t>["1913-1913"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>SAT_WINE_097</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>WSET Official Sparkling Wines</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Cava</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Traditional-method Cava</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Cava</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>ESPUMOSO</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Catalonia / Spain</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Penedes / permitted Cava zones</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Cava DO</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>["Macabeo","Xarel-lo","Parellada"]</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>warm Mediterranean-influenced regions with altitude and site selection preserving acidity</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>varies; higher sites help retain acidity</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>varied Cava DO soils, often limestone and clay depending on zone</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>["traditional local varieties suited to sparkling wine","site selection for acidity and freshness"]</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>["traditional method","second fermentation in bottle","lees ageing","usually non-vintage and dry"]</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>dry to off-dry depending on dosage</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>["lemon","green apple","pear","bread dough","almond"]</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>["citrus","apple","pear","biscuit","almond"]</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB98" t="inlineStr">
+        <is>
+          <t>mostly early drinking; premium examples with longer lees ageing can develop more complexity</t>
+        </is>
+      </c>
+      <c r="AC98" t="inlineStr">
+        <is>
+          <t>["pale lemon","mousse","medium to high acidity","dry profile","citrus and apple fruit","subtle bread or almond notes"]</t>
+        </is>
+      </c>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>["Cava is an essential WSET sparkling tasting style","Cava is traditional method but generally less bready/toasty than Champagne","Macabeo, Xarel-lo and Parellada are key traditional grapes"]</t>
+        </is>
+      </c>
+      <c r="AE98" t="inlineStr">
+        <is>
+          <t>["assuming tank method because it is often inexpensive","overcalling Champagne from bottle-fermentation notes","forgetting local Spanish grape varieties"]</t>
+        </is>
+      </c>
+      <c r="AF98" t="inlineStr">
+        <is>
+          <t>["Traditional method plus Mediterranean fruit and moderate autolysis points toward Cava rather than Champagne."]</t>
+        </is>
+      </c>
+      <c r="AG98" t="inlineStr">
+        <is>
+          <t>["pale lemon","bubbles","medium acidity","high acidity","dry","lemon","apple","pear","biscuit","almond"]</t>
+        </is>
+      </c>
+      <c r="AH98" t="inlineStr">
+        <is>
+          <t>["Do not reveal Cava, Spain, region, grape varieties or DO in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI98" t="inlineStr">
+        <is>
+          <t>Chosen because WSET specifies Cava as an imprescindible sparkling tasting recommendation.</t>
+        </is>
+      </c>
+      <c r="AJ98" t="inlineStr">
+        <is>
+          <t>Practica WSET 097 - Vino espumoso</t>
+        </is>
+      </c>
+      <c r="AK98" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL98" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM98" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN98" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO98" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP98" t="inlineStr">
+        <is>
+          <t>Spanish traditional-method sparkling wine, commonly dry, fresh and citrus/orchard-fruited with moderate autolytic notes.</t>
+        </is>
+      </c>
+      <c r="AQ98" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon","persistent bubbles"],"nose":["lemon","apple","pear","biscuit","almond"],"palate":["dry","medium to high acidity","light to medium body","mousse"],"quality":["good to very good","traditional-method complexity"],"ageing":["usually ready to drink; premium longer-aged styles can develop"],"diagnostic_features":["traditional method","Cava DO","Macabeo Xarel-lo Parellada","moderate autolysis"]}</t>
+        </is>
+      </c>
+      <c r="AR98" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["traditional method","Spanish local grapes","non-vintage dry sparkling","lees ageing"],"learning_objectives":["identify Cava as a required WSET sparkling style","distinguish Cava from Champagne and Prosecco","connect method to autolysis"],"typical_misconceptions":["assuming tank method because it is often inexpensive","overcalling Champagne from bottle-fermentation notes","forgetting local Spanish grape varieties"],"mentor_focus":["Traditional method plus Mediterranean fruit and moderate autolysis points toward Cava rather than Champagne."],"exam_traps":["confusing all traditional method sparkling with Champagne"],"memory_hooks":["Cava equals Spanish traditional method with local grapes"],"comparison_styles":["Champagne Non-Vintage","Cremant","Prosecco"]}</t>
+        </is>
+      </c>
+      <c r="AS98" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_094","SAT_WINE_096","SAT_WINE_100"],"frequently_confused_with":["Champagne","Cremant","traditional method New World sparkling"],"distinguishing_features":["Spanish local grapes","often less intense autolysis than Champagne","Mediterranean fruit profile"]}</t>
+        </is>
+      </c>
+      <c r="AT98" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Cava is an essential WSET sparkling tasting style","Cava is traditional method but generally less bready/toasty than Champagne","Macabeo, Xarel-lo and Parellada are key traditional grapes"],"mentor_hints":["Traditional method plus Mediterranean fruit and moderate autolysis points toward Cava rather than Champagne."],"student_traps":["assuming tank method because it is often inexpensive","overcalling Champagne from bottle-fermentation notes","forgetting local Spanish grape varieties"],"revision_priority":"High: official WSET essential sparkling tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU98" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","cool_climate_high_acid_white"]</t>
+        </is>
+      </c>
+      <c r="AV98" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW98" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 42 / Cava","line_references":["17441-17474"],"evidence":"Specification recommends Cava; book explains Cava DO, traditional grapes, method and common style."}</t>
+        </is>
+      </c>
+      <c r="AX98" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY98" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Sparkling wines</t>
+        </is>
+      </c>
+      <c r="AZ98" t="inlineStr">
+        <is>
+          <t>Catalonia / Spain / Cava DO</t>
+        </is>
+      </c>
+      <c r="BA98" t="inlineStr">
+        <is>
+          <t>WSET specification line 1917; WSET3 rebuilt lines 17441-17474</t>
+        </is>
+      </c>
+      <c r="BB98" t="inlineStr">
+        <is>
+          <t>["1917-1917"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>SAT_WINE_098</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>WSET Official Sparkling Wines</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Asti</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Sweet sparkling Asti</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Asti</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>ESPUMOSO</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Piemonte</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Asti</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Asti DOCG</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>["Muscat Blanc a Petits Grains"]</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>moderate continental Piemonte climate with aromatic Muscat grown around Asti</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>hills around Asti and Alba; exact altitude varies by vineyard</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>varied calcareous marls and regional hillside soils</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>["aromatic Muscat fruit harvested to preserve perfume","healthy grapes for fresh sweet sparkling production"]</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>["Asti method","single fermentation stopped to retain sweetness and dissolved carbon dioxide","made to preserve primary grape aroma"]</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>["grape","orange blossom","peach","pear","floral"]</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>["grapey fruit","peach","pear","orange blossom","sweet citrus"]</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB99" t="inlineStr">
+        <is>
+          <t>drink young to preserve primary fruit and floral aromas</t>
+        </is>
+      </c>
+      <c r="AC99" t="inlineStr">
+        <is>
+          <t>["pale lemon","frothy bubbles","sweet","low alcohol","medium acidity","grapey Muscat aroma","floral notes"]</t>
+        </is>
+      </c>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>["Asti is an essential WSET sparkling tasting style","Asti is sweet, low alcohol and Muscat based","Asti method preserves primary grapey aromas"]</t>
+        </is>
+      </c>
+      <c r="AE99" t="inlineStr">
+        <is>
+          <t>["calling Asti dry","confusing Asti with Prosecco because both are Italian sparkling wines","missing low alcohol as a key clue"]</t>
+        </is>
+      </c>
+      <c r="AF99" t="inlineStr">
+        <is>
+          <t>["Low alcohol plus sweet grapey floral aroma is the fast diagnostic route."]</t>
+        </is>
+      </c>
+      <c r="AG99" t="inlineStr">
+        <is>
+          <t>["pale lemon","bubbles","sweet","low alcohol","medium acidity","grape","orange blossom","peach","pear","floral"]</t>
+        </is>
+      </c>
+      <c r="AH99" t="inlineStr">
+        <is>
+          <t>["Do not reveal Asti, Italy, Piemonte, Muscat or DOCG in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI99" t="inlineStr">
+        <is>
+          <t>Chosen because WSET specifies Asti as an imprescindible sparkling tasting recommendation.</t>
+        </is>
+      </c>
+      <c r="AJ99" t="inlineStr">
+        <is>
+          <t>Practica WSET 098 - Vino espumoso</t>
+        </is>
+      </c>
+      <c r="AK99" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL99" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN99" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO99" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP99" t="inlineStr">
+        <is>
+          <t>Sweet low-alcohol aromatic sparkling wine from Piemonte, with grapey Muscat fruit and floral perfume.</t>
+        </is>
+      </c>
+      <c r="AQ99" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon","bubbles"],"nose":["grape","orange blossom","peach","floral"],"palate":["sweet","low alcohol","medium acidity","light body","frothy mousse"],"quality":["good to very good","primary aromatic intensity"],"ageing":["best consumed young"],"diagnostic_features":["Asti method","Muscat aroma","sweetness","low alcohol"]}</t>
+        </is>
+      </c>
+      <c r="AR99" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["Asti method","Muscat aromatics","fermentation stopped for sweetness","low alcohol"],"learning_objectives":["identify sweet low-alcohol sparkling structure","separate Asti from Prosecco","connect production method to primary fruit"],"typical_misconceptions":["calling Asti dry","confusing Asti with Prosecco because both are Italian sparkling wines","missing low alcohol as a key clue"],"mentor_focus":["Low alcohol plus sweet grapey floral aroma is the fast diagnostic route."],"exam_traps":["assuming all sparkling wine is dry","using country alone to confuse Asti and Prosecco"],"memory_hooks":["Asti equals sweet, low alcohol, grapey Muscat"],"comparison_styles":["Prosecco","Moscato-style aromatic whites","German sweet Riesling for sweetness-acid balance"]}</t>
+        </is>
+      </c>
+      <c r="AS99" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_099","SAT_WINE_017","SAT_WINE_006"],"frequently_confused_with":["Prosecco","off-dry aromatic white wine","sweet Riesling"],"distinguishing_features":["low alcohol","sweet sparkling profile","grapey Muscat and floral aromas"]}</t>
+        </is>
+      </c>
+      <c r="AT99" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Asti is an essential WSET sparkling tasting style","Asti is sweet, low alcohol and Muscat based","Asti method preserves primary grapey aromas"],"mentor_hints":["Low alcohol plus sweet grapey floral aroma is the fast diagnostic route."],"student_traps":["calling Asti dry","confusing Asti with Prosecco because both are Italian sparkling wines","missing low alcohol as a key clue"],"revision_priority":"High: official WSET essential sparkling tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU99" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","aromatic_alsace_white"]</t>
+        </is>
+      </c>
+      <c r="AV99" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW99" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 42 / Asti","line_references":["17478-17486"],"evidence":"Specification recommends Asti; book explains Asti DOCG, Asti method, sweet low-alcohol Muscat style."}</t>
+        </is>
+      </c>
+      <c r="AX99" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY99" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Sparkling wines</t>
+        </is>
+      </c>
+      <c r="AZ99" t="inlineStr">
+        <is>
+          <t>Piemonte / Asti DOCG</t>
+        </is>
+      </c>
+      <c r="BA99" t="inlineStr">
+        <is>
+          <t>WSET specification line 1915; WSET3 rebuilt lines 17478-17486</t>
+        </is>
+      </c>
+      <c r="BB99" t="inlineStr">
+        <is>
+          <t>["1915-1915"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>SAT_WINE_099</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>WSET Official Sparkling Wines</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Prosecco</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Tank-method Prosecco</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Prosecco</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>ESPUMOSO</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Veneto / Friuli</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Prosecco DOC / Conegliano-Valdobbiadene</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Prosecco DOC / Conegliano-Valdobbiadene DOCG</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>["Glera"]</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>moderate north-east Italian climate, with hillside DOCG sites giving fresher premium fruit</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>hillside sites in Conegliano-Valdobbiadene can improve freshness and concentration</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>varied hillside and plain soils across DOC and DOCG zones</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>["Glera grown for fresh aromatic fruit","higher-quality hillside fruit in premium zones"]</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>["tank method","secondary fermentation in pressurised tank","short lees contact to preserve primary fruit","bottled under pressure"]</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>brut to extra dry; residual sugar may be perceptible</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>["pear","apple","white peach","lemon","floral"]</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>["pear","apple","peach","citrus","blossom"]</t>
+        </is>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>short to medium</t>
+        </is>
+      </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB100" t="inlineStr">
+        <is>
+          <t>drink young for freshness and primary fruit</t>
+        </is>
+      </c>
+      <c r="AC100" t="inlineStr">
+        <is>
+          <t>["pale lemon","bubbles","medium to high acidity","fresh pear and apple fruit","little or no autolysis","possible extra dry sweetness"]</t>
+        </is>
+      </c>
+      <c r="AD100" t="inlineStr">
+        <is>
+          <t>["Prosecco is an essential WSET sparkling tasting style","tank method preserves fresh primary fruit","Glera and north-east Italy are the core identity points for debrief"]</t>
+        </is>
+      </c>
+      <c r="AE100" t="inlineStr">
+        <is>
+          <t>["expecting autolytic brioche notes","confusing extra dry with fully dry","calling Prosecco traditional method"]</t>
+        </is>
+      </c>
+      <c r="AF100" t="inlineStr">
+        <is>
+          <t>["If the bubbles are fruit-led rather than bread-led, think tank method before traditional method."]</t>
+        </is>
+      </c>
+      <c r="AG100" t="inlineStr">
+        <is>
+          <t>["pale lemon","bubbles","pear","apple","peach","lemon","floral","medium acidity","high acidity","extra dry"]</t>
+        </is>
+      </c>
+      <c r="AH100" t="inlineStr">
+        <is>
+          <t>["Do not reveal Prosecco, Italy, Veneto/Friuli, Glera or appellation in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI100" t="inlineStr">
+        <is>
+          <t>Chosen because WSET specifies Prosecco as an imprescindible sparkling tasting recommendation.</t>
+        </is>
+      </c>
+      <c r="AJ100" t="inlineStr">
+        <is>
+          <t>Practica WSET 099 - Vino espumoso</t>
+        </is>
+      </c>
+      <c r="AK100" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL100" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM100" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN100" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AO100" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP100" t="inlineStr">
+        <is>
+          <t>Fresh fruit-led tank-method sparkling wine from north-east Italy, typically pear/apple/floral with little autolysis.</t>
+        </is>
+      </c>
+      <c r="AQ100" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon","bubbles"],"nose":["pear","apple","white peach","floral"],"palate":["brut to extra dry","medium to high acidity","light to medium body","fresh fruit"],"quality":["good to very good","primary fruit expression"],"ageing":["best consumed young"],"diagnostic_features":["tank method","Glera","pear and apple fruit","minimal autolysis"]}</t>
+        </is>
+      </c>
+      <c r="AR100" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["tank method","primary fruit preservation","Glera","DOC versus DOCG hierarchy"],"learning_objectives":["identify fruit-led sparkling wine","differentiate Prosecco from Cava and Champagne","explain tank method impact"],"typical_misconceptions":["expecting autolytic brioche notes","confusing extra dry with fully dry","calling Prosecco traditional method"],"mentor_focus":["If the bubbles are fruit-led rather than bread-led, think tank method before traditional method."],"exam_traps":["looking for bread notes where tank method should preserve fruit"],"memory_hooks":["Prosecco equals pear, peach, bubbles and tank method freshness"],"comparison_styles":["Asti","Cava","Champagne Non-Vintage"]}</t>
+        </is>
+      </c>
+      <c r="AS100" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_098","SAT_WINE_097","SAT_WINE_094"],"frequently_confused_with":["Asti","Cava","simple sparkling wine from other countries"],"distinguishing_features":["tank method fruit profile","Glera pear character","minimal autolysis compared with traditional method wines"]}</t>
+        </is>
+      </c>
+      <c r="AT100" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Prosecco is an essential WSET sparkling tasting style","tank method preserves fresh primary fruit","Glera and north-east Italy are the core identity points for debrief"],"mentor_hints":["If the bubbles are fruit-led rather than bread-led, think tank method before traditional method."],"student_traps":["expecting autolytic brioche notes","confusing extra dry with fully dry","calling Prosecco traditional method"],"revision_priority":"High: official WSET essential sparkling tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU100" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","italian_pinot_grigio_core"]</t>
+        </is>
+      </c>
+      <c r="AV100" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW100" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 42 / Prosecco","line_references":["17490-17507"],"evidence":"Specification recommends Prosecco; book explains Prosecco DOC/DOCG, Glera, tank method and fruit-led style."}</t>
+        </is>
+      </c>
+      <c r="AX100" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY100" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Sparkling wines</t>
+        </is>
+      </c>
+      <c r="AZ100" t="inlineStr">
+        <is>
+          <t>Veneto / Friuli / Prosecco DOC / Conegliano-Valdobbiadene DOCG</t>
+        </is>
+      </c>
+      <c r="BA100" t="inlineStr">
+        <is>
+          <t>WSET specification line 1915; WSET3 rebuilt lines 17490-17507</t>
+        </is>
+      </c>
+      <c r="BB100" t="inlineStr">
+        <is>
+          <t>["1915-1915"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>SAT_WINE_100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>WSET Official Sparkling Wines</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>New World Traditional Method Sparkling</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Traditional-method sparkling wine from Australia, New Zealand, South Africa or USA</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>New World Traditional Method Sparkling</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>ESPUMOSO</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Tasmania</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Tasmania</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Tasmania GI</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>["Chardonnay","Pinot Noir"]</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>cool maritime Tasmanian climate suited to high-acid traditional-method base wines</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>varies by Tasmanian site; cool latitude and maritime influence are key</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>varied Tasmanian vineyard soils depending on site</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>["cool-climate Chardonnay and Pinot Noir for sparkling base wine","harvest for acidity and moderate potential alcohol"]</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>["traditional method","second fermentation in bottle","lees ageing","blend of Chardonnay and Pinot Noir","dosage after disgorgement"]</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>usually none to subtle depending on producer and base wine handling</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>brut commonly</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>light to medium</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>pale lemon</t>
+        </is>
+      </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>["lemon","green apple","white peach","biscuit","toast"]</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>["citrus","apple","stone fruit","biscuit","cream"]</t>
+        </is>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB101" t="inlineStr">
+        <is>
+          <t>drink now; premium examples can gain autolytic and nutty complexity</t>
+        </is>
+      </c>
+      <c r="AC101" t="inlineStr">
+        <is>
+          <t>["pale lemon","persistent mousse","high acidity","dry balance","citrus and apple fruit","biscuit or toast autolysis"]</t>
+        </is>
+      </c>
+      <c r="AD101" t="inlineStr">
+        <is>
+          <t>["WSET requires at least one traditional-method sparkling wine from Australia, New Zealand, South Africa or the USA","traditional method cues should be separated from Champagne identity","cool-climate sites such as Tasmania can make premium sparkling base wines"]</t>
+        </is>
+      </c>
+      <c r="AE101" t="inlineStr">
+        <is>
+          <t>["defaulting every traditional-method sparkling to Champagne","forgetting New World examples in WSET LO3","ignoring fruit ripeness differences versus Champagne"]</t>
+        </is>
+      </c>
+      <c r="AF101" t="inlineStr">
+        <is>
+          <t>["Use method first, then decide whether fruit ripeness and origin clues move it away from Champagne."]</t>
+        </is>
+      </c>
+      <c r="AG101" t="inlineStr">
+        <is>
+          <t>["pale lemon","persistent bubbles","high acidity","dry","lemon","apple","white peach","biscuit","toast","cream"]</t>
+        </is>
+      </c>
+      <c r="AH101" t="inlineStr">
+        <is>
+          <t>["Do not reveal country, Tasmania, grape varieties, traditional method region or GI in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI101" t="inlineStr">
+        <is>
+          <t>Chosen to satisfy WSET imprescindible requirement for one traditional-method sparkling wine from Australia / New Zealand / South Africa / USA.</t>
+        </is>
+      </c>
+      <c r="AJ101" t="inlineStr">
+        <is>
+          <t>Practica WSET 100 - Vino espumoso</t>
+        </is>
+      </c>
+      <c r="AK101" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL101" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM101" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN101" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO101" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP101" t="inlineStr">
+        <is>
+          <t>Premium New World traditional-method sparkling profile, represented by cool-climate Tasmania with high acidity, citrus fruit and autolytic biscuit notes.</t>
+        </is>
+      </c>
+      <c r="AQ101" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon","persistent bubbles"],"nose":["lemon","apple","white peach","biscuit","toast"],"palate":["dry","high acidity","light to medium body","persistent mousse"],"quality":["good to outstanding","traditional-method complexity"],"ageing":["premium examples can develop more autolysis with bottle age"],"diagnostic_features":["traditional method","New World cool-climate fruit","Chardonnay Pinot Noir base","autolytic biscuit notes"]}</t>
+        </is>
+      </c>
+      <c r="AR101" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["traditional method beyond Champagne","cool-climate New World sparkling","Chardonnay Pinot Noir base","autolysis and dosage"],"learning_objectives":["cover WSET New World traditional-method sparkling requirement","distinguish method from origin","compare Tasmania with Champagne and Cava"],"typical_misconceptions":["defaulting every traditional-method sparkling to Champagne","forgetting New World examples in WSET LO3","ignoring fruit ripeness differences versus Champagne"],"mentor_focus":["Use method first, then decide whether fruit ripeness and origin clues move it away from Champagne."],"exam_traps":["using method as origin proof","forgetting New World sparkling in LO3"],"memory_hooks":["New World traditional method equals Champagne toolkit, different place signal"],"comparison_styles":["Champagne Non-Vintage","Cava","Cremant"]}</t>
+        </is>
+      </c>
+      <c r="AS101" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_094","SAT_WINE_096","SAT_WINE_097"],"frequently_confused_with":["Champagne","Cava","Cremant"],"distinguishing_features":["New World fruit ripeness","Tasmanian cool-climate profile","less Champagne-specific reserve wine identity"]}</t>
+        </is>
+      </c>
+      <c r="AT101" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["WSET requires at least one traditional-method sparkling wine from Australia, New Zealand, South Africa or the USA","traditional method cues should be separated from Champagne identity","cool-climate sites such as Tasmania can make premium sparkling base wines"],"mentor_hints":["Use method first, then decide whether fruit ripeness and origin clues move it away from Champagne."],"student_traps":["defaulting every traditional-method sparkling to Champagne","forgetting New World examples in WSET LO3","ignoring fruit ripeness differences versus Champagne"],"revision_priority":"High: official WSET essential sparkling tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU101" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","cool_climate_high_acid_white","premium_chardonnay_winemaking"]</t>
+        </is>
+      </c>
+      <c r="AV101" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW101" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 42 / Sparkling wines of the New World","line_references":["17575-17575"],"evidence":"Specification recommends traditional-method sparkling from Australia, New Zealand, South Africa or USA; book discusses classic Champagne varieties in New World sparkling contexts."}</t>
+        </is>
+      </c>
+      <c r="AX101" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY101" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Sparkling wines</t>
+        </is>
+      </c>
+      <c r="AZ101" t="inlineStr">
+        <is>
+          <t>Tasmania / Tasmania GI</t>
+        </is>
+      </c>
+      <c r="BA101" t="inlineStr">
+        <is>
+          <t>WSET specification lines 1922-1923; WSET3 rebuilt line 17575</t>
+        </is>
+      </c>
+      <c r="BB101" t="inlineStr">
+        <is>
+          <t>["1922-1923"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(cwp): add WSET official fortified wines batch 012
</commit_message>
<xml_diff>
--- a/canonical-wine-catalog/exports/canonical_wines.xlsx
+++ b/canonical-wine-catalog/exports/canonical_wines.xlsx
@@ -27482,6 +27482,1910 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>SAT_WINE_101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>WSET Official Fortified Wines</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Fino / Manzanilla</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Biologically aged dry Sherry</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Fino / Manzanilla</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>FORTIFICADO</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Jerez</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Jerez / Sanlucar de Barrameda</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Jerez-Xeres-Sherry / Manzanilla-Sanlucar</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>["Palomino"]</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>warm Mediterranean climate around Jerez, with coastal humidity important for Manzanilla flor in Sanlucar</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>low-lying coastal and inland vineyard zones; exact altitude is less diagnostic than flor ageing environment</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>albariza chalky soils are central to high-quality Palomino vineyards</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>["Palomino grown for neutral base wine and freshness","site and climate support flor-ageing style after fortification"]</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>["base white wine fermented dry","fortified to a level that permits flor growth","biological ageing under flor in a solera system","bottled pale and dry"]</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>old neutral American oak butts used for maturation, not new-oak flavour</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>pale lemon to pale gold</t>
+        </is>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>["almond","green apple","lemon","yeast","saline"]</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>["almond","apple","lemon","bread dough","salty"]</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB102" t="inlineStr">
+        <is>
+          <t>best consumed fresh after bottling; biological freshness fades once opened</t>
+        </is>
+      </c>
+      <c r="AC102" t="inlineStr">
+        <is>
+          <t>["pale lemon","dry","medium acidity","medium to high alcohol","light body","flor-derived almond and yeast notes","saline finish"]</t>
+        </is>
+      </c>
+      <c r="AD102" t="inlineStr">
+        <is>
+          <t>["Fino or Manzanilla is an essential WSET fortified tasting style","biological ageing under flor is the diagnostic production feature","Manzanilla is closely linked to Sanlucar de Barrameda"]</t>
+        </is>
+      </c>
+      <c r="AE102" t="inlineStr">
+        <is>
+          <t>["calling dry Sherry sweet","missing flor character","confusing Manzanilla with a separate grape variety"]</t>
+        </is>
+      </c>
+      <c r="AF102" t="inlineStr">
+        <is>
+          <t>["Dryness plus flor almond and saline notes is the core diagnostic route."]</t>
+        </is>
+      </c>
+      <c r="AG102" t="inlineStr">
+        <is>
+          <t>["pale lemon","dry","medium acidity","medium alcohol","almond","yeast","green apple","lemon","saline","bread dough"]</t>
+        </is>
+      </c>
+      <c r="AH102" t="inlineStr">
+        <is>
+          <t>["Do not reveal Sherry, Jerez, Manzanilla, Spain, Palomino or appellation in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI102" t="inlineStr">
+        <is>
+          <t>Chosen because WSET specifies Fino or Manzanilla as an imprescindible fortified tasting style.</t>
+        </is>
+      </c>
+      <c r="AJ102" t="inlineStr">
+        <is>
+          <t>Practica WSET 101 - Vino fortificado</t>
+        </is>
+      </c>
+      <c r="AK102" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL102" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM102" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN102" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO102" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP102" t="inlineStr">
+        <is>
+          <t>Pale dry biologically aged Sherry with flor-derived almond, yeast, apple and saline notes.</t>
+        </is>
+      </c>
+      <c r="AQ102" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon to pale gold"],"nose":["almond","yeast","green apple","saline"],"palate":["dry","medium acidity","medium to high alcohol","light body","salty finish"],"quality":["good to very good","clear flor character"],"ageing":["fresh bottled style with biological ageing already complete"],"diagnostic_features":["fortified dry wine","flor ageing","Palomino","solera system"]}</t>
+        </is>
+      </c>
+      <c r="AR102" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["biological ageing","flor","fortification level","solera"],"learning_objectives":["identify dry biologically aged Sherry","separate Fino/Manzanilla from oxidative Sherry","connect flor to aroma profile"],"typical_misconceptions":["calling dry Sherry sweet","missing flor character","confusing Manzanilla with a separate grape variety"],"mentor_focus":["Dryness plus flor almond and saline notes is the core diagnostic route."],"exam_traps":["assuming fortified means sweet"],"memory_hooks":["Fino equals pale, dry, flor and almond"],"comparison_styles":["Amontillado / Oloroso","Medium / Cream Sherry","Asti for sweetness contrast"]}</t>
+        </is>
+      </c>
+      <c r="AS102" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_102","SAT_WINE_105"],"frequently_confused_with":["dry white wine with oxidative notes","Amontillado","Manzanilla style wine"],"distinguishing_features":["pale colour","dry palate","flor almond and saline profile","lighter body than oxidative Sherry"]}</t>
+        </is>
+      </c>
+      <c r="AT102" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Fino or Manzanilla is an essential WSET fortified tasting style","biological ageing under flor is the diagnostic production feature","Manzanilla is closely linked to Sanlucar de Barrameda"],"mentor_hints":["Dryness plus flor almond and saline notes is the core diagnostic route."],"student_traps":["calling dry Sherry sweet","missing flor character","confusing Manzanilla with a separate grape variety"],"revision_priority":"High: official WSET essential fortified tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU102" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV102" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW102" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 43 / Sherry styles","line_references":["18078-18095"],"evidence":"Specification recommends Fino or Manzanilla; book describes biological ageing and Manzanilla from Sanlucar."}</t>
+        </is>
+      </c>
+      <c r="AX102" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY102" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Fortified wines</t>
+        </is>
+      </c>
+      <c r="AZ102" t="inlineStr">
+        <is>
+          <t>Jerez / Jerez-Xeres-Sherry / Manzanilla-Sanlucar</t>
+        </is>
+      </c>
+      <c r="BA102" t="inlineStr">
+        <is>
+          <t>WSET specification line 1939; WSET3 rebuilt lines 18078-18095</t>
+        </is>
+      </c>
+      <c r="BB102" t="inlineStr">
+        <is>
+          <t>["1939-1939"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>SAT_WINE_102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>WSET Official Fortified Wines</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Dry Amontillado / Oloroso</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Oxidatively aged dry Sherry</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Dry Amontillado / Oloroso</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>FORTIFICADO</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Jerez</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Jerez</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Jerez-Xeres-Sherry</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>["Palomino"]</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>warm Mediterranean climate around Jerez, producing neutral Palomino base wines for ageing</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>vineyard zone and albariza exposure matter more than a single altitude value</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>albariza chalk-rich soils associated with quality Palomino production</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>["Palomino grown for dry base wine","healthy grapes suitable for fortification and long maturation"]</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>["base wine fermented dry","fortification and solera ageing","Amontillado begins with biological ageing then ages oxidatively","Oloroso ages oxidatively without flor"]</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>old neutral American oak butts with oxidative maturation</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>dry</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>amber to brown</t>
+        </is>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>["walnut","hazelnut","dried fruit","caramel","orange peel"]</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>["nut","toffee","dried fig","caramel","savory"]</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB103" t="inlineStr">
+        <is>
+          <t>long oxidative maturation before release; stable after opening compared with Fino</t>
+        </is>
+      </c>
+      <c r="AC103" t="inlineStr">
+        <is>
+          <t>["amber or brown colour","dry","high alcohol","medium acidity","nutty oxidative aromas","long finish"]</t>
+        </is>
+      </c>
+      <c r="AD103" t="inlineStr">
+        <is>
+          <t>["Amontillado seco or Oloroso seco is an essential WSET fortified tasting style","Amontillado combines biological then oxidative ageing; Oloroso is oxidative","dryness must be stated even with nutty caramel aromas"]</t>
+        </is>
+      </c>
+      <c r="AE103" t="inlineStr">
+        <is>
+          <t>["assuming brown Sherry is sweet","forgetting Amontillado and Oloroso are dry unless sweetened","missing oxidative ageing as the main driver"]</t>
+        </is>
+      </c>
+      <c r="AF103" t="inlineStr">
+        <is>
+          <t>["Colour and nutty oxidative notes separate this from Fino; dryness separates it from Cream."]</t>
+        </is>
+      </c>
+      <c r="AG103" t="inlineStr">
+        <is>
+          <t>["amber","brown","dry","high alcohol","medium acidity","walnut","hazelnut","dried fruit","caramel","orange peel","long finish"]</t>
+        </is>
+      </c>
+      <c r="AH103" t="inlineStr">
+        <is>
+          <t>["Do not reveal Sherry, Jerez, Spain, Palomino, Amontillado, Oloroso or appellation in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI103" t="inlineStr">
+        <is>
+          <t>Chosen because WSET specifies dry Amontillado or dry Oloroso as an imprescindible fortified tasting style.</t>
+        </is>
+      </c>
+      <c r="AJ103" t="inlineStr">
+        <is>
+          <t>Practica WSET 102 - Vino fortificado</t>
+        </is>
+      </c>
+      <c r="AK103" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL103" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM103" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN103" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AO103" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP103" t="inlineStr">
+        <is>
+          <t>Dry oxidative Sherry family with amber/brown colour, high alcohol, nutty aromas and long savoury finish.</t>
+        </is>
+      </c>
+      <c r="AQ103" t="inlineStr">
+        <is>
+          <t>{"appearance":["amber to brown"],"nose":["walnut","hazelnut","dried fruit","caramel"],"palate":["dry","high alcohol","medium acidity","medium to full body"],"quality":["good to outstanding","long oxidative complexity"],"ageing":["oxidative solera maturation before release"],"diagnostic_features":["fortified dry wine","oxidative ageing","nutty profile","solera system"]}</t>
+        </is>
+      </c>
+      <c r="AR103" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["oxidative ageing","solera","Amontillado versus Oloroso pathway","dry fortified style"],"learning_objectives":["identify oxidative dry Sherry","distinguish from Fino and Cream","explain why brown colour does not equal sweetness"],"typical_misconceptions":["assuming brown Sherry is sweet","forgetting Amontillado and Oloroso are dry unless sweetened","missing oxidative ageing as the main driver"],"mentor_focus":["Colour and nutty oxidative notes separate this from Fino; dryness separates it from Cream."],"exam_traps":["equating caramel aroma with sweetness"],"memory_hooks":["Oloroso/Amontillado equals brown, dry, nutty and high alcohol"],"comparison_styles":["Fino / Manzanilla","Medium / Cream Sherry","Tawny Port"]}</t>
+        </is>
+      </c>
+      <c r="AS103" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_101","SAT_WINE_105","SAT_WINE_104"],"frequently_confused_with":["Medium or Cream Sherry","Tawny Port","old dry white wine"],"distinguishing_features":["dry palate","Palomino savoury nut profile","no red-fruit Port structure"]}</t>
+        </is>
+      </c>
+      <c r="AT103" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Amontillado seco or Oloroso seco is an essential WSET fortified tasting style","Amontillado combines biological then oxidative ageing; Oloroso is oxidative","dryness must be stated even with nutty caramel aromas"],"mentor_hints":["Colour and nutty oxidative notes separate this from Fino; dryness separates it from Cream."],"student_traps":["assuming brown Sherry is sweet","forgetting Amontillado and Oloroso are dry unless sweetened","missing oxidative ageing as the main driver"],"revision_priority":"High: official WSET essential fortified tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU103" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV103" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW103" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 43 / Sherry styles","line_references":["18103-18134"],"evidence":"Specification recommends dry Amontillado or dry Oloroso; book explains oxidative ageing and style differences."}</t>
+        </is>
+      </c>
+      <c r="AX103" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY103" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Fortified wines</t>
+        </is>
+      </c>
+      <c r="AZ103" t="inlineStr">
+        <is>
+          <t>Jerez / Jerez-Xeres-Sherry</t>
+        </is>
+      </c>
+      <c r="BA103" t="inlineStr">
+        <is>
+          <t>WSET specification line 1940; WSET3 rebuilt lines 18103-18134</t>
+        </is>
+      </c>
+      <c r="BB103" t="inlineStr">
+        <is>
+          <t>["1940-1940"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>SAT_WINE_103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>WSET Official Fortified Wines</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>LBV / Vintage Port</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Bottle-aged or late-bottled ruby Port</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LBV / Vintage Port</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>FORTIFICADO</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Douro</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Douro Valley</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Port</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>["Touriga Franca","Tinta Roriz","Touriga Nacional"]</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>warm to hot continental Douro climate with steep vineyard sites and low rainfall pressure inland</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>steep Douro vineyards vary widely in altitude and aspect</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>schistous soils associated with Douro Port vineyards</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>["black grapes grown in steep Douro vineyards","ripe fruit harvested for concentration and colour"]</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>["fermentation stopped by grape spirit fortification","short extraction-focused fermentation","aged as LBV or Vintage Port depending on style","Vintage Port bottled with capacity for long bottle ageing"]</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>large old vessels or short ageing depending on LBV/Vintage pathway; no new-oak flavour focus</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>deep ruby to purple</t>
+        </is>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>["blackberry","black plum","black cherry","violet","chocolate"]</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>["black fruit","spice","chocolate","liquorice","grape spirit warmth"]</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>very good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB104" t="inlineStr">
+        <is>
+          <t>LBV may be ready to drink; Vintage Port can age for decades in bottle</t>
+        </is>
+      </c>
+      <c r="AC104" t="inlineStr">
+        <is>
+          <t>["deep ruby","sweet","high alcohol","full body","medium to high tannin","black fruit concentration","long finish"]</t>
+        </is>
+      </c>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t>["LBV or Vintage Port is an essential WSET fortified tasting style","fermentation is stopped by fortification to retain sweetness","unfiltered LBV and Vintage Port can throw sediment"]</t>
+        </is>
+      </c>
+      <c r="AE104" t="inlineStr">
+        <is>
+          <t>["calling Port dry because tannin is high","missing grape-spirit fortification as production logic","confusing Tawny oxidative notes with ruby Port fruit"]</t>
+        </is>
+      </c>
+      <c r="AF104" t="inlineStr">
+        <is>
+          <t>["Sweetness plus high alcohol plus black-fruit tannic structure points to ruby-family Port."]</t>
+        </is>
+      </c>
+      <c r="AG104" t="inlineStr">
+        <is>
+          <t>["deep ruby","sweet","high alcohol","full body","medium tannin","high tannin","blackberry","black plum","chocolate","spice","long finish"]</t>
+        </is>
+      </c>
+      <c r="AH104" t="inlineStr">
+        <is>
+          <t>["Do not reveal Port, Portugal, Douro, LBV, Vintage or grape varieties in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI104" t="inlineStr">
+        <is>
+          <t>Chosen because WSET specifies LBV or Vintage Port as an imprescindible fortified tasting style.</t>
+        </is>
+      </c>
+      <c r="AJ104" t="inlineStr">
+        <is>
+          <t>Practica WSET 103 - Vino fortificado</t>
+        </is>
+      </c>
+      <c r="AK104" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL104" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM104" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN104" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO104" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP104" t="inlineStr">
+        <is>
+          <t>Sweet full-bodied ruby-family Port with deep colour, high alcohol, black fruit, tannin and long finish.</t>
+        </is>
+      </c>
+      <c r="AQ104" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep ruby to purple"],"nose":["blackberry","black plum","violet","chocolate"],"palate":["sweet","high alcohol","full body","medium to high tannin","long finish"],"quality":["very good to outstanding","high concentration"],"ageing":["LBV often drinkable; Vintage Port has long bottle-age potential"],"diagnostic_features":["fortification stops fermentation","Douro black grapes","ruby Port fruit concentration","sweet high-alcohol structure"]}</t>
+        </is>
+      </c>
+      <c r="AR104" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["fortification during fermentation","ruby Port family","LBV versus Vintage ageing","sweet fortified red structure"],"learning_objectives":["identify LBV/Vintage Port as required WSET style","separate ruby Port from Tawny Port","connect extraction and fortification to SAT structure"],"typical_misconceptions":["calling Port dry because tannin is high","missing grape-spirit fortification as production logic","confusing Tawny oxidative notes with ruby Port fruit"],"mentor_focus":["Sweetness plus high alcohol plus black-fruit tannic structure points to ruby-family Port."],"exam_traps":["confusing tannin with dryness"],"memory_hooks":["Ruby Port equals sweet, black, strong and structured"],"comparison_styles":["Tawny Port","Douro Red","Rutherglen Muscat"]}</t>
+        </is>
+      </c>
+      <c r="AS104" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_104","SAT_WINE_069"],"frequently_confused_with":["Douro red table wine","Tawny Port","sweet red wine"],"distinguishing_features":["sweetness with high alcohol","black fruit and tannin","fortified warmth"]}</t>
+        </is>
+      </c>
+      <c r="AT104" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["LBV or Vintage Port is an essential WSET fortified tasting style","fermentation is stopped by fortification to retain sweetness","unfiltered LBV and Vintage Port can throw sediment"],"mentor_hints":["Sweetness plus high alcohol plus black-fruit tannic structure points to ruby-family Port."],"student_traps":["calling Port dry because tannin is high","missing grape-spirit fortification as production logic","confusing Tawny oxidative notes with ruby Port fruit"],"revision_priority":"High: official WSET essential fortified tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU104" t="inlineStr">
+        <is>
+          <t>["douro_red_core","dao_red_core"]</t>
+        </is>
+      </c>
+      <c r="AV104" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW104" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 44 / Port styles","line_references":["18461-18469","18524-18536"],"evidence":"Specification recommends LBV or Vintage Port; book describes LBV and Vintage Port ageing and filtration differences."}</t>
+        </is>
+      </c>
+      <c r="AX104" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY104" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Fortified wines</t>
+        </is>
+      </c>
+      <c r="AZ104" t="inlineStr">
+        <is>
+          <t>Douro / Port</t>
+        </is>
+      </c>
+      <c r="BA104" t="inlineStr">
+        <is>
+          <t>WSET specification line 1944; WSET3 rebuilt lines 18461-18469 and 18524-18536</t>
+        </is>
+      </c>
+      <c r="BB104" t="inlineStr">
+        <is>
+          <t>["1944-1944"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>SAT_WINE_104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>WSET Official Fortified Wines</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Aged Tawny Port</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Tawny Port with indication of age</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Aged Tawny Port</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>FORTIFICADO</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Douro</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Douro Valley</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Port</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>["Touriga Franca","Tinta Roriz","Touriga Nacional"]</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>warm to hot continental Douro climate producing ripe grapes for fortified wines</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>Douro vineyards range across steep slopes with varied altitude and aspect</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>schistous Douro soils</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>["ripe black grapes grown for concentration","vineyard blending is common in traditional Port production"]</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>["fermentation stopped by grape spirit fortification","long oxidative ageing in wood","blending to age-indicated Tawny style","bottled ready to drink"]</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>long maturation in old wooden vessels gives oxidative character rather than new-oak flavour</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>low to medium</t>
+        </is>
+      </c>
+      <c r="W105" t="inlineStr">
+        <is>
+          <t>tawny to brown</t>
+        </is>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>["caramel","walnut","toffee","dried fig","orange peel"]</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>["dried fruit","nut","caramel","coffee","spice"]</t>
+        </is>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>very good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB105" t="inlineStr">
+        <is>
+          <t>aged oxidatively before release; bottled ready to drink</t>
+        </is>
+      </c>
+      <c r="AC105" t="inlineStr">
+        <is>
+          <t>["tawny or brown colour","sweet","high alcohol","medium acidity","nutty oxidative aromas","dried fruit and caramel","long finish"]</t>
+        </is>
+      </c>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t>["Tawny Port with indication of age is an essential WSET fortified tasting style","long oxidative wood ageing differentiates Tawny from LBV/Vintage Port","age indication reflects a blended style rather than a single exact age"]</t>
+        </is>
+      </c>
+      <c r="AE105" t="inlineStr">
+        <is>
+          <t>["confusing Tawny Port with Oloroso because both are nutty","expecting high tannin like Vintage Port","assuming age indication means bottle ageing"]</t>
+        </is>
+      </c>
+      <c r="AF105" t="inlineStr">
+        <is>
+          <t>["Sweetness and Port warmth separate it from dry oxidative Sherry; colour and nuts separate it from ruby Port."]</t>
+        </is>
+      </c>
+      <c r="AG105" t="inlineStr">
+        <is>
+          <t>["tawny","brown","sweet","high alcohol","caramel","walnut","toffee","dried fig","orange peel","long finish"]</t>
+        </is>
+      </c>
+      <c r="AH105" t="inlineStr">
+        <is>
+          <t>["Do not reveal Port, Portugal, Douro, Tawny, age indication or grape varieties in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI105" t="inlineStr">
+        <is>
+          <t>Chosen because WSET specifies Porto Tawny with indication of age as an imprescindible fortified tasting style.</t>
+        </is>
+      </c>
+      <c r="AJ105" t="inlineStr">
+        <is>
+          <t>Practica WSET 104 - Vino fortificado</t>
+        </is>
+      </c>
+      <c r="AK105" t="inlineStr">
+        <is>
+          <t>P0_WSET_ESSENTIAL</t>
+        </is>
+      </c>
+      <c r="AL105" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="AM105" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN105" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO105" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP105" t="inlineStr">
+        <is>
+          <t>Sweet oxidative Port with tawny/brown colour, high alcohol, dried fruit, nuts, caramel and long finish.</t>
+        </is>
+      </c>
+      <c r="AQ105" t="inlineStr">
+        <is>
+          <t>{"appearance":["tawny to brown"],"nose":["caramel","walnut","toffee","dried fig"],"palate":["sweet","high alcohol","medium acidity","medium to full body","long finish"],"quality":["very good to outstanding","complex oxidative wood-aged profile"],"ageing":["long wood ageing before bottling; ready to drink"],"diagnostic_features":["age-indicated Tawny Port","oxidative wood ageing","sweet fortified structure","nut and dried-fruit complexity"]}</t>
+        </is>
+      </c>
+      <c r="AR105" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["oxidative ageing in wood","age-indicated blending","Port fortification","ruby versus tawny contrast"],"learning_objectives":["identify aged Tawny Port as required WSET style","distinguish from LBV/Vintage Port","distinguish from dry oxidative Sherry"],"typical_misconceptions":["confusing Tawny Port with Oloroso because both are nutty","expecting high tannin like Vintage Port","assuming age indication means bottle ageing"],"mentor_focus":["Sweetness and Port warmth separate it from dry oxidative Sherry; colour and nuts separate it from ruby Port."],"exam_traps":["forgetting Tawny remains sweet"],"memory_hooks":["Tawny Port equals sweet, brown, nutty and wood-aged"],"comparison_styles":["LBV / Vintage Port","Dry Amontillado / Oloroso","Rutherglen Muscat"]}</t>
+        </is>
+      </c>
+      <c r="AS105" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_103","SAT_WINE_102","SAT_WINE_107"],"frequently_confused_with":["Oloroso Sherry","Rutherglen Muscat","old red wine"],"distinguishing_features":["sweet Port structure","Douro spirit warmth","less flor/savoury than Sherry"]}</t>
+        </is>
+      </c>
+      <c r="AT105" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Tawny Port with indication of age is an essential WSET fortified tasting style","long oxidative wood ageing differentiates Tawny from LBV/Vintage Port","age indication reflects a blended style rather than a single exact age"],"mentor_hints":["Sweetness and Port warmth separate it from dry oxidative Sherry; colour and nuts separate it from ruby Port."],"student_traps":["confusing Tawny Port with Oloroso because both are nutty","expecting high tannin like Vintage Port","assuming age indication means bottle ageing"],"revision_priority":"High: official WSET essential fortified tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU105" t="inlineStr">
+        <is>
+          <t>["douro_red_core"]</t>
+        </is>
+      </c>
+      <c r="AV105" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW105" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 44 / Tawny Port","line_references":["18479-18479","18539-18567"],"evidence":"Specification recommends Tawny Port with indication of age; book explains long oxidative wood ageing and age indication."}</t>
+        </is>
+      </c>
+      <c r="AX105" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY105" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Fortified wines</t>
+        </is>
+      </c>
+      <c r="AZ105" t="inlineStr">
+        <is>
+          <t>Douro / Port</t>
+        </is>
+      </c>
+      <c r="BA105" t="inlineStr">
+        <is>
+          <t>WSET specification line 1945; WSET3 rebuilt lines 18479 and 18539-18567</t>
+        </is>
+      </c>
+      <c r="BB105" t="inlineStr">
+        <is>
+          <t>["1945-1945"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>SAT_WINE_105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>WSET Official Fortified Wines</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Medium / Cream Sherry</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Sweetened blended Sherry</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Medium / Cream Sherry</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>FORTIFICADO</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Jerez</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Jerez</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Jerez-Xeres-Sherry</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>["Palomino","Pedro Ximenez","Muscat"]</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>warm Mediterranean Jerez climate with Palomino base wines and sweetening components from PX or Muscat</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>regional vineyard zones; exact altitude is less diagnostic than blending and ageing choices</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>albariza for Palomino plus sites suited to sweetening varieties</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>["Palomino for dry base wine","Pedro Ximenez or Muscat for sweetening components"]</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>["dry Sherry base aged biologically and/or oxidatively","sweetened with sweet wine or sweetening component","blended to Medium or Cream style","solera maturation may contribute complexity"]</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>old neutral American oak butts used in maturation</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>medium-sweet to sweet</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>medium to full</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>amber to brown</t>
+        </is>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>["raisin","caramel","walnut","fig","toffee"]</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>["dried fruit","caramel","nut","molasses","sweet spice"]</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA106" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB106" t="inlineStr">
+        <is>
+          <t>stable style; generally bottled ready to drink</t>
+        </is>
+      </c>
+      <c r="AC106" t="inlineStr">
+        <is>
+          <t>["amber or brown colour","medium-sweet to sweet","high alcohol","nutty oxidative notes","dried fruit sweetness"]</t>
+        </is>
+      </c>
+      <c r="AD106" t="inlineStr">
+        <is>
+          <t>["Medium or Cream Sherry is an official optional WSET fortified tasting recommendation","sweetening distinguishes it from dry Amontillado/Oloroso","base wine may show biological and/or oxidative ageing"]</t>
+        </is>
+      </c>
+      <c r="AE106" t="inlineStr">
+        <is>
+          <t>["calling all brown Sherry dry","missing added sweetness as the key contrast with Oloroso","assuming Cream means dairy flavour"]</t>
+        </is>
+      </c>
+      <c r="AF106" t="inlineStr">
+        <is>
+          <t>["Use sweetness as the first branch: dry oxidative Sherry versus sweetened Medium/Cream."]</t>
+        </is>
+      </c>
+      <c r="AG106" t="inlineStr">
+        <is>
+          <t>["amber","brown","medium sweet","sweet","high alcohol","raisin","caramel","walnut","fig","toffee"]</t>
+        </is>
+      </c>
+      <c r="AH106" t="inlineStr">
+        <is>
+          <t>["Do not reveal Sherry, Jerez, Spain, Cream, Medium or grape varieties in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI106" t="inlineStr">
+        <is>
+          <t>Included because Medium or Cream Sherry is an official optional WSET fortified tasting recommendation and fits the generosos batch.</t>
+        </is>
+      </c>
+      <c r="AJ106" t="inlineStr">
+        <is>
+          <t>Practica WSET 105 - Vino fortificado</t>
+        </is>
+      </c>
+      <c r="AK106" t="inlineStr">
+        <is>
+          <t>P1_WSET_RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="AL106" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM106" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AN106" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO106" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP106" t="inlineStr">
+        <is>
+          <t>Sweetened Sherry style with amber/brown colour, high alcohol, dried fruit, caramel and nutty oxidative notes.</t>
+        </is>
+      </c>
+      <c r="AQ106" t="inlineStr">
+        <is>
+          <t>{"appearance":["amber to brown"],"nose":["raisin","caramel","walnut","fig"],"palate":["medium-sweet to sweet","high alcohol","medium acidity","medium to full body"],"quality":["good to very good","sweet oxidative complexity"],"ageing":["bottled ready to drink after blending and maturation"],"diagnostic_features":["sweetened Sherry","Palomino base plus sweet component","oxidative and dried-fruit notes","high alcohol"]}</t>
+        </is>
+      </c>
+      <c r="AR106" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["sweetened Sherry category","Medium versus Cream","blending dry and sweet components","solera context"],"learning_objectives":["differentiate Medium/Cream from dry Sherry","identify sweetness in fortified tasting","explain PX or Muscat sweetening role"],"typical_misconceptions":["calling all brown Sherry dry","missing added sweetness as the key contrast with Oloroso","assuming Cream means dairy flavour"],"mentor_focus":["Use sweetness as the first branch: dry oxidative Sherry versus sweetened Medium/Cream."],"exam_traps":["treating colour as a sweetness proxy"],"memory_hooks":["Cream Sherry equals Sherry framework plus sweetness"],"comparison_styles":["Dry Amontillado / Oloroso","Fino / Manzanilla","Tawny Port"]}</t>
+        </is>
+      </c>
+      <c r="AS106" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_102","SAT_WINE_101","SAT_WINE_104"],"frequently_confused_with":["Oloroso Sherry","Tawny Port","PX-like sweet wine"],"distinguishing_features":["sweetened Sherry character","Jerez nutty profile","no Port red-fruit structure"]}</t>
+        </is>
+      </c>
+      <c r="AT106" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Medium or Cream Sherry is an official optional WSET fortified tasting recommendation","sweetening distinguishes it from dry Amontillado/Oloroso","base wine may show biological and/or oxidative ageing"],"mentor_hints":["Use sweetness as the first branch: dry oxidative Sherry versus sweetened Medium/Cream."],"student_traps":["calling all brown Sherry dry","missing added sweetness as the key contrast with Oloroso","assuming Cream means dairy flavour"],"revision_priority":"Medium-high: official WSET optional fortified tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU106" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core"]</t>
+        </is>
+      </c>
+      <c r="AV106" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW106" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 43 / Sweetened Sherry styles","line_references":["18153-18170"],"evidence":"Specification recommends Medium or Cream Sherry optionally; book explains Pale Cream, Medium and Cream as sweetened/blended styles."}</t>
+        </is>
+      </c>
+      <c r="AX106" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY106" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Fortified wines</t>
+        </is>
+      </c>
+      <c r="AZ106" t="inlineStr">
+        <is>
+          <t>Jerez / Jerez-Xeres-Sherry</t>
+        </is>
+      </c>
+      <c r="BA106" t="inlineStr">
+        <is>
+          <t>WSET specification line 1942; WSET3 rebuilt lines 18153-18170</t>
+        </is>
+      </c>
+      <c r="BB106" t="inlineStr">
+        <is>
+          <t>["1942-1942"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>SAT_WINE_106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>WSET Official Fortified Wines</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Muscat de Beaumes-de-Venise</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Youthful fortified Muscat</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Muscat de Beaumes-de-Venise</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>FORTIFICADO</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Southern Rhone</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Beaumes-de-Venise</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Muscat de Beaumes-de-Venise</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>["Muscat Blanc a Petits Grains"]</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>warm Mediterranean Southern Rhone climate supporting ripe aromatic Muscat grapes</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>hillside vineyards around Beaumes-de-Venise; exact altitude varies by site</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>varied Southern Rhone limestone, clay and stony soils depending on site</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>["aromatic Muscat harvested ripe","fruit handled to preserve primary floral and grapey character"]</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>["fermentation stopped by fortification to retain sweetness","youthful unaged style","protective handling to preserve primary Muscat aromas"]</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>sweet</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>low to medium</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>medium to high</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>pale lemon to gold</t>
+        </is>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>["grape","orange blossom","rose","peach","apricot"]</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>["grapey fruit","orange blossom","stone fruit","honey","sweet citrus"]</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>medium to long</t>
+        </is>
+      </c>
+      <c r="AA107" t="inlineStr">
+        <is>
+          <t>good to very good</t>
+        </is>
+      </c>
+      <c r="AB107" t="inlineStr">
+        <is>
+          <t>best young for primary Muscat perfume, though some examples can hold briefly</t>
+        </is>
+      </c>
+      <c r="AC107" t="inlineStr">
+        <is>
+          <t>["pale lemon to gold","sweet","medium to high alcohol","grapey Muscat aroma","floral and stone-fruit notes"]</t>
+        </is>
+      </c>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t>["Muscat de Beaumes-de-Venise is an official optional WSET fortified tasting recommendation","it represents youthful unaged fortified Muscat","fortification preserves sweetness and primary aroma"]</t>
+        </is>
+      </c>
+      <c r="AE107" t="inlineStr">
+        <is>
+          <t>["confusing fortified Muscat with Asti because both are grapey","forgetting this is still fortified not sparkling","overlooking low to medium acidity"]</t>
+        </is>
+      </c>
+      <c r="AF107" t="inlineStr">
+        <is>
+          <t>["Grapey floral sweetness without bubbles points away from Asti and toward fortified Muscat."]</t>
+        </is>
+      </c>
+      <c r="AG107" t="inlineStr">
+        <is>
+          <t>["pale lemon","gold","sweet","grape","orange blossom","rose","peach","apricot","honey","medium alcohol"]</t>
+        </is>
+      </c>
+      <c r="AH107" t="inlineStr">
+        <is>
+          <t>["Do not reveal Muscat de Beaumes-de-Venise, France, Southern Rhone, Muscat or appellation in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI107" t="inlineStr">
+        <is>
+          <t>Included because Muscat de Beaumes-de-Venise is an official optional WSET fortified tasting recommendation and fits the generosos batch.</t>
+        </is>
+      </c>
+      <c r="AJ107" t="inlineStr">
+        <is>
+          <t>Practica WSET 106 - Vino fortificado</t>
+        </is>
+      </c>
+      <c r="AK107" t="inlineStr">
+        <is>
+          <t>P1_WSET_RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="AL107" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM107" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AN107" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO107" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP107" t="inlineStr">
+        <is>
+          <t>Sweet youthful fortified Muscat from the Southern Rhone with grapey, floral and stone-fruit aromatics.</t>
+        </is>
+      </c>
+      <c r="AQ107" t="inlineStr">
+        <is>
+          <t>{"appearance":["pale lemon to gold"],"nose":["grape","orange blossom","rose","peach"],"palate":["sweet","medium to high alcohol","low to medium acidity","medium body"],"quality":["good to very good","primary aromatic intensity"],"ageing":["best young for perfume"],"diagnostic_features":["fortified Muscat","youthful unaged style","grapey floral aroma","sweetness retained by fortification"]}</t>
+        </is>
+      </c>
+      <c r="AR107" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["fortified Muscat","youthful unaged style","aromatic grape variety","fortification retaining sweetness"],"learning_objectives":["identify youthful fortified Muscat","separate still fortified Muscat from Asti","contrast with aged Rutherglen Muscat"],"typical_misconceptions":["confusing fortified Muscat with Asti because both are grapey","forgetting this is still fortified not sparkling","overlooking low to medium acidity"],"mentor_focus":["Grapey floral sweetness without bubbles points away from Asti and toward fortified Muscat."],"exam_traps":["assuming all Muscat styles sparkle"],"memory_hooks":["Beaumes-de-Venise equals still sweet grapey fortified Muscat"],"comparison_styles":["Rutherglen Muscat","Asti","Alsace Gewurztraminer"]}</t>
+        </is>
+      </c>
+      <c r="AS107" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_107","SAT_WINE_098","SAT_WINE_006"],"frequently_confused_with":["Asti","late-harvest aromatic white","Rutherglen Muscat"],"distinguishing_features":["still fortified structure","youthful primary grape and floral notes","less oxidative than Rutherglen"]}</t>
+        </is>
+      </c>
+      <c r="AT107" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Muscat de Beaumes-de-Venise is an official optional WSET fortified tasting recommendation","it represents youthful unaged fortified Muscat","fortification preserves sweetness and primary aroma"],"mentor_hints":["Grapey floral sweetness without bubbles points away from Asti and toward fortified Muscat."],"student_traps":["confusing fortified Muscat with Asti because both are grapey","forgetting this is still fortified not sparkling","overlooking low to medium acidity"],"revision_priority":"Medium-high: official WSET optional fortified tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU107" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","aromatic_alsace_white"]</t>
+        </is>
+      </c>
+      <c r="AV107" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW107" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 45 / Fortified Muscats","line_references":["18636-18643"],"evidence":"Specification recommends Muscat de Beaumes-de-Venise optionally; book presents it as a youthful unaged fortified Muscat example."}</t>
+        </is>
+      </c>
+      <c r="AX107" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY107" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Fortified wines</t>
+        </is>
+      </c>
+      <c r="AZ107" t="inlineStr">
+        <is>
+          <t>Southern Rhone / Muscat de Beaumes-de-Venise</t>
+        </is>
+      </c>
+      <c r="BA107" t="inlineStr">
+        <is>
+          <t>WSET specification line 1950; WSET3 rebuilt lines 18636-18643</t>
+        </is>
+      </c>
+      <c r="BB107" t="inlineStr">
+        <is>
+          <t>["1950-1950"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>SAT_WINE_107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>WSET Official Fortified Wines</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Rutherglen Muscat</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Aged fortified Muscat</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Rutherglen Muscat</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>FORTIFICADO</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Rutherglen</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Rutherglen</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Rutherglen</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>["Muscat"]</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>warm inland Australian climate around Rutherglen, supporting very ripe Muscat grapes</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>regional vineyard altitude varies; warm inland ripeness is more diagnostic</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>varied Rutherglen soils depending on vineyard</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>["Muscat grapes harvested very ripe","fruit concentration supports luscious fortified style"]</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>["fermentation stopped by fortification","long oxidative ageing in old wood","fractional blending systems may build complexity","bottled with developed character"]</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>long ageing in old wooden vessels gives oxidative concentration, not new-oak flavour</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>lusciously sweet</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>deep amber to brown</t>
+        </is>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>["raisin","fig","toffee","coffee","orange peel"]</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>["molasses","caramel","dried fruit","coffee","sweet spice"]</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="AA108" t="inlineStr">
+        <is>
+          <t>very good to outstanding</t>
+        </is>
+      </c>
+      <c r="AB108" t="inlineStr">
+        <is>
+          <t>aged oxidatively before bottling; very stable and complex on release</t>
+        </is>
+      </c>
+      <c r="AC108" t="inlineStr">
+        <is>
+          <t>["deep amber or brown","lusciously sweet","high alcohol","full body","dried fruit and toffee","long oxidative finish"]</t>
+        </is>
+      </c>
+      <c r="AD108" t="inlineStr">
+        <is>
+          <t>["Rutherglen Muscat is an official optional WSET fortified tasting recommendation","it represents fully developed aged fortified Muscat","oxidative ageing and concentration distinguish it from youthful Muscat"]</t>
+        </is>
+      </c>
+      <c r="AE108" t="inlineStr">
+        <is>
+          <t>["confusing it with Tawny Port solely because both are brown and sweet","missing Muscat grapey/orange-peel lift beneath oxidative notes","underestimating sweetness and body"]</t>
+        </is>
+      </c>
+      <c r="AF108" t="inlineStr">
+        <is>
+          <t>["When the wine is brown, sweet and intense, check whether Muscat perfume remains under the oxidative layer."]</t>
+        </is>
+      </c>
+      <c r="AG108" t="inlineStr">
+        <is>
+          <t>["deep amber","brown","lusciously sweet","high alcohol","full body","raisin","fig","toffee","coffee","orange peel","long finish"]</t>
+        </is>
+      </c>
+      <c r="AH108" t="inlineStr">
+        <is>
+          <t>["Do not reveal Rutherglen, Australia, Muscat or region in blind labels."]</t>
+        </is>
+      </c>
+      <c r="AI108" t="inlineStr">
+        <is>
+          <t>Included because Rutherglen Muscat is an official optional WSET fortified tasting recommendation and fits the generosos batch.</t>
+        </is>
+      </c>
+      <c r="AJ108" t="inlineStr">
+        <is>
+          <t>Practica WSET 107 - Vino fortificado</t>
+        </is>
+      </c>
+      <c r="AK108" t="inlineStr">
+        <is>
+          <t>P1_WSET_RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="AL108" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="AM108" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AN108" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AO108" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="AP108" t="inlineStr">
+        <is>
+          <t>Lusciously sweet aged fortified Muscat with deep amber colour, dried fruit, toffee, coffee and long oxidative complexity.</t>
+        </is>
+      </c>
+      <c r="AQ108" t="inlineStr">
+        <is>
+          <t>{"appearance":["deep amber to brown"],"nose":["raisin","fig","toffee","coffee","orange peel"],"palate":["lusciously sweet","high alcohol","full body","medium acidity","long finish"],"quality":["very good to outstanding","high concentration and oxidative complexity"],"ageing":["long oxidative ageing before release"],"diagnostic_features":["aged fortified Muscat","Rutherglen style","luscious sweetness","oxidative dried-fruit and toffee profile"]}</t>
+        </is>
+      </c>
+      <c r="AR108" t="inlineStr">
+        <is>
+          <t>{"core_concepts":["aged fortified Muscat","oxidative ageing","luscious sweetness","Australian Rutherglen benchmark"],"learning_objectives":["identify aged fortified Muscat","distinguish from Tawny Port","contrast with youthful Muscat de Beaumes-de-Venise"],"typical_misconceptions":["confusing it with Tawny Port solely because both are brown and sweet","missing Muscat grapey/orange-peel lift beneath oxidative notes","underestimating sweetness and body"],"mentor_focus":["When the wine is brown, sweet and intense, check whether Muscat perfume remains under the oxidative layer."],"exam_traps":["calling every sweet brown fortified wine Tawny Port"],"memory_hooks":["Rutherglen Muscat equals brown, sweet, raisin, toffee and Muscat lift"],"comparison_styles":["Aged Tawny Port","Muscat de Beaumes-de-Venise","Medium / Cream Sherry"]}</t>
+        </is>
+      </c>
+      <c r="AS108" t="inlineStr">
+        <is>
+          <t>{"similar_profiles":["SAT_WINE_104","SAT_WINE_106","SAT_WINE_105"],"frequently_confused_with":["Tawny Port","Cream Sherry","old sweet wine"],"distinguishing_features":["Muscat aromatic lift","luscious texture","Australian aged fortified Muscat identity"]}</t>
+        </is>
+      </c>
+      <c r="AT108" t="inlineStr">
+        <is>
+          <t>{"common_exam_points":["Rutherglen Muscat is an official optional WSET fortified tasting recommendation","it represents fully developed aged fortified Muscat","oxidative ageing and concentration distinguish it from youthful Muscat"],"mentor_hints":["When the wine is brown, sweet and intense, check whether Muscat perfume remains under the oxidative layer."],"student_traps":["confusing it with Tawny Port solely because both are brown and sweet","missing Muscat grapey/orange-peel lift beneath oxidative notes","underestimating sweetness and body"],"revision_priority":"Medium-high: official WSET optional fortified tasting style."}</t>
+        </is>
+      </c>
+      <c r="AU108" t="inlineStr">
+        <is>
+          <t>["white_wine_sat_core","aromatic_alsace_white"]</t>
+        </is>
+      </c>
+      <c r="AV108" t="inlineStr">
+        <is>
+          <t>{"canonical_id":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"wine_family":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_style":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"display_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"wine_name":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wine_type":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"country":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"region":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"subregion":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"appellation":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"grape_varieties":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"TRAINING"},"climate":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"altitude":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"soil":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"viticulture":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"winemaking":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"oak":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sweetness":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"body":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"acidity":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"alcohol":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"tannin":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"color":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"aroma_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"flavour_profile":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"finish":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"quality_level":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"ageing_potential":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"expected_sat_observations":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_exam_points":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"common_student_errors":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"mentor_hints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"descriptor_whitelist":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"sat_constraints":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"reasoning_notes":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"display_label":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"wset_importance":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"practice_priority":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"difficulty_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"confidence_score":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"knowledge_summary":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"sat_fingerprint":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"pedagogical_dna":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"comparison_engine":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"teaching_notes":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"reusable_knowledge_refs":{"knowledge_origin":"STANDARD_WINE_KNOWLEDGE","visibility_level":"TRAINING"},"source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"canonical_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"chapter":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"section":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"page_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"line_reference":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"},"style_category":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"PUBLIC"},"specification_source":{"knowledge_origin":"WSET_PRIMARY","visibility_level":"SERVER_ONLY"}}</t>
+        </is>
+      </c>
+      <c r="AW108" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","section":"Chapter 45 / Fortified Muscats","line_references":["18666-18698"],"evidence":"Specification recommends Rutherglen Muscat optionally; book presents Rutherglen as the classic aged Muscat example."}</t>
+        </is>
+      </c>
+      <c r="AX108" t="inlineStr">
+        <is>
+          <t>{"file":"D:\\Descargas\\Phone Link\\WSET3_rebuilt.md","sha256":"91B5D64859140AF5C98EDE988D2F55D52579B3C8DCD5004EE225A9B62569CC25","source_type":"rebuilt_markdown_from_official_wset_book"}</t>
+        </is>
+      </c>
+      <c r="AY108" t="inlineStr">
+        <is>
+          <t>WSET specification tasting recommendations / Fortified wines</t>
+        </is>
+      </c>
+      <c r="AZ108" t="inlineStr">
+        <is>
+          <t>Rutherglen / Rutherglen</t>
+        </is>
+      </c>
+      <c r="BA108" t="inlineStr">
+        <is>
+          <t>WSET specification line 1951; WSET3 rebuilt lines 18666-18698</t>
+        </is>
+      </c>
+      <c r="BB108" t="inlineStr">
+        <is>
+          <t>["1951-1951"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>